<commit_message>
Unité Humide workbook: panel / false-ceiling height 6.00 m
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011Ghrdsx3moo1sM21DD7JVm
</commit_message>
<xml_diff>
--- a/DWG_Plan_Modificatif/DWG Plan Modificatif/Unite Humide - dimensions panneaux froid.xlsx
+++ b/DWG_Plan_Modificatif/DWG Plan Modificatif/Unite Humide - dimensions panneaux froid.xlsx
@@ -279,7 +279,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">HSP 8 m sur le plan. Réduire si faux-plafond isotherme plus bas.</t>
+          <t xml:space="preserve">Hauteur des panneaux / faux-plafond isotherme : 6,00 m (demande client). HSP bâtiment sur le plan : 8 m.</t>
         </r>
       </text>
     </comment>
@@ -291,7 +291,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">HSP 8 m sur le plan. Réduire si faux-plafond isotherme plus bas.</t>
+          <t xml:space="preserve">Hauteur des panneaux / faux-plafond isotherme : 6,00 m (demande client). HSP bâtiment sur le plan : 8 m.</t>
         </r>
       </text>
     </comment>
@@ -303,7 +303,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">HSP 8 m sur le plan. Réduire si faux-plafond isotherme plus bas.</t>
+          <t xml:space="preserve">Hauteur des panneaux / faux-plafond isotherme : 6,00 m (demande client). HSP bâtiment sur le plan : 8 m.</t>
         </r>
       </text>
     </comment>
@@ -315,7 +315,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">HSP 8 m sur le plan. Réduire si faux-plafond isotherme plus bas.</t>
+          <t xml:space="preserve">Hauteur des panneaux / faux-plafond isotherme : 6,00 m (demande client). HSP bâtiment sur le plan : 8 m.</t>
         </r>
       </text>
     </comment>
@@ -327,7 +327,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">HSP 8 m sur le plan. Réduire si faux-plafond isotherme plus bas.</t>
+          <t xml:space="preserve">Hauteur des panneaux / faux-plafond isotherme : 6,00 m (demande client). HSP bâtiment sur le plan : 8 m.</t>
         </r>
       </text>
     </comment>
@@ -339,7 +339,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">HSP 8 m sur le plan. Réduire si faux-plafond isotherme plus bas.</t>
+          <t xml:space="preserve">Hauteur des panneaux / faux-plafond isotherme : 6,00 m (demande client). HSP bâtiment sur le plan : 8 m.</t>
         </r>
       </text>
     </comment>
@@ -351,7 +351,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">HSP 8 m sur le plan. Réduire si faux-plafond isotherme plus bas.</t>
+          <t xml:space="preserve">Hauteur des panneaux / faux-plafond isotherme : 6,00 m (demande client). HSP bâtiment sur le plan : 8 m.</t>
         </r>
       </text>
     </comment>
@@ -363,7 +363,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">HSP 8 m sur le plan. Réduire si faux-plafond isotherme plus bas.</t>
+          <t xml:space="preserve">Hauteur des panneaux / faux-plafond isotherme : 6,00 m (demande client). HSP bâtiment sur le plan : 8 m.</t>
         </r>
       </text>
     </comment>
@@ -375,7 +375,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">HSP 8 m sur le plan. Réduire si faux-plafond isotherme plus bas.</t>
+          <t xml:space="preserve">Hauteur des panneaux / faux-plafond isotherme : 6,00 m (demande client). HSP bâtiment sur le plan : 8 m.</t>
         </r>
       </text>
     </comment>
@@ -387,7 +387,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">HSP 8 m sur le plan. Réduire si faux-plafond isotherme plus bas.</t>
+          <t xml:space="preserve">Hauteur des panneaux / faux-plafond isotherme : 6,00 m (demande client). HSP bâtiment sur le plan : 8 m.</t>
         </r>
       </text>
     </comment>
@@ -1651,7 +1651,7 @@
     <t xml:space="preserve">Points d'attention</t>
   </si>
   <si>
-    <t xml:space="preserve">• Dimensions mesurées entre nus intérieurs des murs sur P1 RDC v2.dwg ; hauteur par défaut = HSP 8 m du plan (à réduire si les chambres ont un faux-plafond isotherme plus bas : le volume et les apports baissent d'autant).</t>
+    <t xml:space="preserve">• Dimensions mesurées entre nus intérieurs des murs sur P1 RDC v2.dwg ; hauteur des panneaux et du faux-plafond isotherme = 6,00 m pour toutes les zones (HSP bâtiment 8 m) – modifiable zone par zone (colonne G de Zones).</t>
   </si>
   <si>
     <t xml:space="preserve">• Par défaut, seules la salle de préparation viande (+10 °C), la chambre positive (+2 °C) et la chambre négative (−20 °C) sont réfrigérées ; passer une zone à « Oui » dans Zones pour l'inclure.</t>
@@ -1828,7 +1828,7 @@
     <t xml:space="preserve">Dimensions des zones – Unité Humide (RDC Modifié)</t>
   </si>
   <si>
-    <t xml:space="preserve">Mesuré sur P1 RDC v2.dwg (RDC Modifié), entre nus intérieurs des murs. Hauteur = hauteur des panneaux/plafond (HSP bâtiment 8 m par défaut).</t>
+    <t xml:space="preserve">Mesuré sur P1 RDC v2.dwg (RDC Modifié), entre nus intérieurs des murs. Hauteur = hauteur des panneaux / faux-plafond isotherme : 6,00 m (HSP bâtiment 8 m).</t>
   </si>
   <si>
     <t xml:space="preserve">Zone</t>
@@ -3864,11 +3864,11 @@
         <v>72.54</v>
       </c>
       <c r="G5" s="15" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H5" s="24" t="n">
         <f aca="false">E5*G5</f>
-        <v>2313.0016</v>
+        <v>1734.7512</v>
       </c>
       <c r="I5" s="25" t="s">
         <v>86</v>
@@ -3885,7 +3885,7 @@
       </c>
       <c r="M5" s="22" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A5,Parois!$J$5:$J$41)+SUMIF(Parois!$C$5:$C$41,A5,Parois!$J$5:$J$41)-SUMIFS(Parois!$J$5:$J$41,Parois!$B$5:$B$41,A5,Parois!$C$5:$C$41,A5)</f>
-        <v>573.43</v>
+        <v>428.55</v>
       </c>
       <c r="N5" s="22" t="n">
         <f aca="false">IF(I5="Oui",E5,0)</f>
@@ -3915,11 +3915,11 @@
         <v>56.16</v>
       </c>
       <c r="G6" s="15" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H6" s="24" t="n">
         <f aca="false">E6*G6</f>
-        <v>1503.04</v>
+        <v>1127.28</v>
       </c>
       <c r="I6" s="25" t="s">
         <v>86</v>
@@ -3936,7 +3936,7 @@
       </c>
       <c r="M6" s="22" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A6,Parois!$J$5:$J$41)+SUMIF(Parois!$C$5:$C$41,A6,Parois!$J$5:$J$41)-SUMIFS(Parois!$J$5:$J$41,Parois!$B$5:$B$41,A6,Parois!$C$5:$C$41,A6)</f>
-        <v>443.4</v>
+        <v>331.08</v>
       </c>
       <c r="N6" s="22" t="n">
         <f aca="false">IF(I6="Oui",E6,0)</f>
@@ -3966,11 +3966,11 @@
         <v>54.16</v>
       </c>
       <c r="G7" s="15" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H7" s="24" t="n">
         <f aca="false">E7*G7</f>
-        <v>1366.4</v>
+        <v>1024.8</v>
       </c>
       <c r="I7" s="25" t="s">
         <v>86</v>
@@ -3987,7 +3987,7 @@
       </c>
       <c r="M7" s="22" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A7,Parois!$J$5:$J$41)+SUMIF(Parois!$C$5:$C$41,A7,Parois!$J$5:$J$41)-SUMIFS(Parois!$J$5:$J$41,Parois!$B$5:$B$41,A7,Parois!$C$5:$C$41,A7)</f>
-        <v>373.58</v>
+        <v>279.45</v>
       </c>
       <c r="N7" s="22" t="n">
         <f aca="false">IF(I7="Oui",E7,0)</f>
@@ -4019,11 +4019,11 @@
         <v>54.39</v>
       </c>
       <c r="G8" s="15" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H8" s="24" t="n">
         <f aca="false">E8*G8</f>
-        <v>1130.392</v>
+        <v>847.794</v>
       </c>
       <c r="I8" s="25" t="s">
         <v>86</v>
@@ -4040,7 +4040,7 @@
       </c>
       <c r="M8" s="22" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A8,Parois!$J$5:$J$41)+SUMIF(Parois!$C$5:$C$41,A8,Parois!$J$5:$J$41)-SUMIFS(Parois!$J$5:$J$41,Parois!$B$5:$B$41,A8,Parois!$C$5:$C$41,A8)</f>
-        <v>373.28</v>
+        <v>278.49</v>
       </c>
       <c r="N8" s="22" t="n">
         <f aca="false">IF(I8="Oui",E8,0)</f>
@@ -4072,11 +4072,11 @@
         <v>60.37</v>
       </c>
       <c r="G9" s="15" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H9" s="24" t="n">
         <f aca="false">E9*G9</f>
-        <v>1613.576</v>
+        <v>1210.182</v>
       </c>
       <c r="I9" s="25" t="s">
         <v>86</v>
@@ -4093,7 +4093,7 @@
       </c>
       <c r="M9" s="22" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A9,Parois!$J$5:$J$41)+SUMIF(Parois!$C$5:$C$41,A9,Parois!$J$5:$J$41)-SUMIFS(Parois!$J$5:$J$41,Parois!$B$5:$B$41,A9,Parois!$C$5:$C$41,A9)</f>
-        <v>477.08</v>
+        <v>356.34</v>
       </c>
       <c r="N9" s="22" t="n">
         <f aca="false">IF(I9="Oui",E9,0)</f>
@@ -4123,11 +4123,11 @@
         <v>60.69</v>
       </c>
       <c r="G10" s="15" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H10" s="24" t="n">
         <f aca="false">E10*G10</f>
-        <v>1212.56</v>
+        <v>909.42</v>
       </c>
       <c r="I10" s="25" t="s">
         <v>86</v>
@@ -4144,7 +4144,7 @@
       </c>
       <c r="M10" s="22" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A10,Parois!$J$5:$J$41)+SUMIF(Parois!$C$5:$C$41,A10,Parois!$J$5:$J$41)-SUMIFS(Parois!$J$5:$J$41,Parois!$B$5:$B$41,A10,Parois!$C$5:$C$41,A10)</f>
-        <v>477.24</v>
+        <v>356.46</v>
       </c>
       <c r="N10" s="22" t="n">
         <f aca="false">IF(I10="Oui",E10,0)</f>
@@ -4176,11 +4176,11 @@
         <v>54.48</v>
       </c>
       <c r="G11" s="15" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H11" s="24" t="n">
         <f aca="false">E11*G11</f>
-        <v>547.456</v>
+        <v>410.592</v>
       </c>
       <c r="I11" s="25" t="s">
         <v>86</v>
@@ -4197,7 +4197,7 @@
       </c>
       <c r="M11" s="22" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A11,Parois!$J$5:$J$41)+SUMIF(Parois!$C$5:$C$41,A11,Parois!$J$5:$J$41)-SUMIFS(Parois!$J$5:$J$41,Parois!$B$5:$B$41,A11,Parois!$C$5:$C$41,A11)</f>
-        <v>441.98</v>
+        <v>327.81</v>
       </c>
       <c r="N11" s="22" t="n">
         <f aca="false">IF(I11="Oui",E11,0)</f>
@@ -4229,11 +4229,11 @@
         <v>68.7</v>
       </c>
       <c r="G12" s="15" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H12" s="24" t="n">
         <f aca="false">E12*G12</f>
-        <v>2322.3472</v>
+        <v>1741.7604</v>
       </c>
       <c r="I12" s="25" t="s">
         <v>86</v>
@@ -4250,7 +4250,7 @@
       </c>
       <c r="M12" s="22" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A12,Parois!$J$5:$J$41)+SUMIF(Parois!$C$5:$C$41,A12,Parois!$J$5:$J$41)-SUMIFS(Parois!$J$5:$J$41,Parois!$B$5:$B$41,A12,Parois!$C$5:$C$41,A12)</f>
-        <v>535.32</v>
+        <v>397.92</v>
       </c>
       <c r="N12" s="22" t="n">
         <f aca="false">IF(I12="Oui",E12,0)</f>
@@ -4282,11 +4282,11 @@
         <v>40.02</v>
       </c>
       <c r="G13" s="15" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H13" s="24" t="n">
         <f aca="false">E13*G13</f>
-        <v>600.4</v>
+        <v>450.3</v>
       </c>
       <c r="I13" s="25" t="s">
         <v>86</v>
@@ -4303,7 +4303,7 @@
       </c>
       <c r="M13" s="22" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A13,Parois!$J$5:$J$41)+SUMIF(Parois!$C$5:$C$41,A13,Parois!$J$5:$J$41)-SUMIFS(Parois!$J$5:$J$41,Parois!$B$5:$B$41,A13,Parois!$C$5:$C$41,A13)</f>
-        <v>317.22</v>
+        <v>237.18</v>
       </c>
       <c r="N13" s="22" t="n">
         <f aca="false">IF(I13="Oui",E13,0)</f>
@@ -4331,11 +4331,11 @@
         <v>130.38</v>
       </c>
       <c r="G14" s="15" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H14" s="24" t="n">
         <f aca="false">E14*G14</f>
-        <v>2532.64</v>
+        <v>1899.48</v>
       </c>
       <c r="I14" s="25" t="s">
         <v>63</v>
@@ -4352,7 +4352,7 @@
       </c>
       <c r="M14" s="22" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A14,Parois!$J$5:$J$41)+SUMIF(Parois!$C$5:$C$41,A14,Parois!$J$5:$J$41)-SUMIFS(Parois!$J$5:$J$41,Parois!$B$5:$B$41,A14,Parois!$C$5:$C$41,A14)</f>
-        <v>1147.58</v>
+        <v>857.01</v>
       </c>
       <c r="N14" s="22" t="n">
         <f aca="false">IF(I14="Oui",E14,0)</f>
@@ -4372,11 +4372,11 @@
       </c>
       <c r="H15" s="30" t="n">
         <f aca="false">SUM(H5:H14)</f>
-        <v>15141.8128</v>
+        <v>11356.3596</v>
       </c>
       <c r="M15" s="29" t="n">
         <f aca="false">SUM(M5:M14)</f>
-        <v>5160.11</v>
+        <v>3850.29</v>
       </c>
       <c r="N15" s="29" t="n">
         <f aca="false">SUM(N5:N14)</f>
@@ -5046,11 +5046,11 @@
       </c>
       <c r="F5" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B5,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C5,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G5" s="22" t="n">
         <f aca="false">E5*F5</f>
-        <v>195.52</v>
+        <v>146.64</v>
       </c>
       <c r="H5" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A5,Portes!$H$5:$H$20)</f>
@@ -5062,7 +5062,7 @@
       </c>
       <c r="J5" s="22" t="n">
         <f aca="false">MAX(0,G5-H5)</f>
-        <v>195.52</v>
+        <v>146.64</v>
       </c>
       <c r="K5" s="18" t="n">
         <f aca="false">IF(I5="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B5,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C5,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -5082,7 +5082,7 @@
       </c>
       <c r="O5" s="24" t="n">
         <f aca="false">L5*J5*MAX(0,N5-M5)</f>
-        <v>716.906666666667</v>
+        <v>537.68</v>
       </c>
       <c r="P5" s="24" t="n">
         <f aca="false">L5*J5*MAX(0,M5-N5)</f>
@@ -5107,11 +5107,11 @@
       </c>
       <c r="F6" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B6,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C6,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G6" s="22" t="n">
         <f aca="false">E6*F6</f>
-        <v>94.64</v>
+        <v>70.98</v>
       </c>
       <c r="H6" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A6,Portes!$H$5:$H$20)</f>
@@ -5123,7 +5123,7 @@
       </c>
       <c r="J6" s="22" t="n">
         <f aca="false">MAX(0,G6-H6)</f>
-        <v>91.49</v>
+        <v>67.83</v>
       </c>
       <c r="K6" s="18" t="n">
         <f aca="false">IF(I6="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B6,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C6,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -5168,11 +5168,11 @@
       </c>
       <c r="F7" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B7,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C7,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G7" s="22" t="n">
         <f aca="false">E7*F7</f>
-        <v>94.64</v>
+        <v>70.98</v>
       </c>
       <c r="H7" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A7,Portes!$H$5:$H$20)</f>
@@ -5184,7 +5184,7 @@
       </c>
       <c r="J7" s="22" t="n">
         <f aca="false">MAX(0,G7-H7)</f>
-        <v>94.64</v>
+        <v>70.98</v>
       </c>
       <c r="K7" s="18" t="n">
         <f aca="false">IF(I7="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B7,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C7,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -5204,7 +5204,7 @@
       </c>
       <c r="O7" s="24" t="n">
         <f aca="false">L7*J7*MAX(0,N7-M7)</f>
-        <v>347.013333333333</v>
+        <v>260.26</v>
       </c>
       <c r="P7" s="24" t="n">
         <f aca="false">L7*J7*MAX(0,M7-N7)</f>
@@ -5229,11 +5229,11 @@
       </c>
       <c r="F8" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B8,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C8,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G8" s="22" t="n">
         <f aca="false">E8*F8</f>
-        <v>58.08</v>
+        <v>43.56</v>
       </c>
       <c r="H8" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A8,Portes!$H$5:$H$20)</f>
@@ -5245,7 +5245,7 @@
       </c>
       <c r="J8" s="22" t="n">
         <f aca="false">MAX(0,G8-H8)</f>
-        <v>58.08</v>
+        <v>43.56</v>
       </c>
       <c r="K8" s="18" t="n">
         <f aca="false">IF(I8="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B8,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C8,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -5290,11 +5290,11 @@
       </c>
       <c r="F9" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B9,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C9,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G9" s="22" t="n">
         <f aca="false">E9*F9</f>
-        <v>136.64</v>
+        <v>102.48</v>
       </c>
       <c r="H9" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A9,Portes!$H$5:$H$20)</f>
@@ -5306,7 +5306,7 @@
       </c>
       <c r="J9" s="22" t="n">
         <f aca="false">MAX(0,G9-H9)</f>
-        <v>133.7</v>
+        <v>99.54</v>
       </c>
       <c r="K9" s="18" t="n">
         <f aca="false">IF(I9="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B9,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C9,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -5351,11 +5351,11 @@
       </c>
       <c r="F10" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B10,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C10,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G10" s="22" t="n">
         <f aca="false">E10*F10</f>
-        <v>88</v>
+        <v>66</v>
       </c>
       <c r="H10" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A10,Portes!$H$5:$H$20)</f>
@@ -5367,7 +5367,7 @@
       </c>
       <c r="J10" s="22" t="n">
         <f aca="false">MAX(0,G10-H10)</f>
-        <v>88</v>
+        <v>66</v>
       </c>
       <c r="K10" s="18" t="n">
         <f aca="false">IF(I10="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B10,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C10,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -5387,7 +5387,7 @@
       </c>
       <c r="O10" s="24" t="n">
         <f aca="false">L10*J10*MAX(0,N10-M10)</f>
-        <v>322.666666666667</v>
+        <v>242</v>
       </c>
       <c r="P10" s="24" t="n">
         <f aca="false">L10*J10*MAX(0,M10-N10)</f>
@@ -5412,11 +5412,11 @@
       </c>
       <c r="F11" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B11,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C11,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G11" s="22" t="n">
         <f aca="false">E11*F11</f>
-        <v>136.64</v>
+        <v>102.48</v>
       </c>
       <c r="H11" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A11,Portes!$H$5:$H$20)</f>
@@ -5428,7 +5428,7 @@
       </c>
       <c r="J11" s="22" t="n">
         <f aca="false">MAX(0,G11-H11)</f>
-        <v>133.7</v>
+        <v>99.54</v>
       </c>
       <c r="K11" s="18" t="n">
         <f aca="false">IF(I11="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B11,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C11,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="O11" s="24" t="n">
         <f aca="false">L11*J11*MAX(0,N11-M11)</f>
-        <v>245.116666666667</v>
+        <v>182.49</v>
       </c>
       <c r="P11" s="24" t="n">
         <f aca="false">L11*J11*MAX(0,M11-N11)</f>
@@ -5473,11 +5473,11 @@
       </c>
       <c r="F12" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B12,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C12,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G12" s="22" t="n">
         <f aca="false">E12*F12</f>
-        <v>88</v>
+        <v>66</v>
       </c>
       <c r="H12" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A12,Portes!$H$5:$H$20)</f>
@@ -5489,7 +5489,7 @@
       </c>
       <c r="J12" s="22" t="n">
         <f aca="false">MAX(0,G12-H12)</f>
-        <v>88</v>
+        <v>66</v>
       </c>
       <c r="K12" s="18" t="n">
         <f aca="false">IF(I12="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B12,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C12,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -5534,11 +5534,11 @@
       </c>
       <c r="F13" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B13,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C13,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G13" s="22" t="n">
         <f aca="false">E13*F13</f>
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="H13" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A13,Portes!$H$5:$H$20)</f>
@@ -5550,7 +5550,7 @@
       </c>
       <c r="J13" s="22" t="n">
         <f aca="false">MAX(0,G13-H13)</f>
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K13" s="18" t="n">
         <f aca="false">IF(I13="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B13,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C13,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -5570,7 +5570,7 @@
       </c>
       <c r="O13" s="24" t="n">
         <f aca="false">L13*J13*MAX(0,N13-M13)</f>
-        <v>146.666666666667</v>
+        <v>110</v>
       </c>
       <c r="P13" s="24" t="n">
         <f aca="false">L13*J13*MAX(0,M13-N13)</f>
@@ -5595,11 +5595,11 @@
       </c>
       <c r="F14" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B14,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C14,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G14" s="22" t="n">
         <f aca="false">E14*F14</f>
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="H14" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A14,Portes!$H$5:$H$20)</f>
@@ -5611,7 +5611,7 @@
       </c>
       <c r="J14" s="22" t="n">
         <f aca="false">MAX(0,G14-H14)</f>
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="K14" s="18" t="n">
         <f aca="false">IF(I14="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B14,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C14,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -5635,7 +5635,7 @@
       </c>
       <c r="P14" s="24" t="n">
         <f aca="false">L14*J14*MAX(0,M14-N14)</f>
-        <v>146.666666666667</v>
+        <v>110</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5656,11 +5656,11 @@
       </c>
       <c r="F15" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B15,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C15,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G15" s="22" t="n">
         <f aca="false">E15*F15</f>
-        <v>79.88</v>
+        <v>59.91</v>
       </c>
       <c r="H15" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A15,Portes!$H$5:$H$20)</f>
@@ -5672,7 +5672,7 @@
       </c>
       <c r="J15" s="22" t="n">
         <f aca="false">MAX(0,G15-H15)</f>
-        <v>79.88</v>
+        <v>59.91</v>
       </c>
       <c r="K15" s="18" t="n">
         <f aca="false">IF(I15="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B15,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C15,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -5717,11 +5717,11 @@
       </c>
       <c r="F16" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B16,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C16,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G16" s="22" t="n">
         <f aca="false">E16*F16</f>
-        <v>161.6</v>
+        <v>121.2</v>
       </c>
       <c r="H16" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A16,Portes!$H$5:$H$20)</f>
@@ -5733,7 +5733,7 @@
       </c>
       <c r="J16" s="22" t="n">
         <f aca="false">MAX(0,G16-H16)</f>
-        <v>158.66</v>
+        <v>118.26</v>
       </c>
       <c r="K16" s="18" t="n">
         <f aca="false">IF(I16="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B16,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C16,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -5778,11 +5778,11 @@
       </c>
       <c r="F17" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B17,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C17,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G17" s="22" t="n">
         <f aca="false">E17*F17</f>
-        <v>161.6</v>
+        <v>121.2</v>
       </c>
       <c r="H17" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A17,Portes!$H$5:$H$20)</f>
@@ -5794,7 +5794,7 @@
       </c>
       <c r="J17" s="22" t="n">
         <f aca="false">MAX(0,G17-H17)</f>
-        <v>158.66</v>
+        <v>118.26</v>
       </c>
       <c r="K17" s="18" t="n">
         <f aca="false">IF(I17="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B17,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C17,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -5814,7 +5814,7 @@
       </c>
       <c r="O17" s="24" t="n">
         <f aca="false">L17*J17*MAX(0,N17-M17)</f>
-        <v>290.876666666667</v>
+        <v>216.81</v>
       </c>
       <c r="P17" s="24" t="n">
         <f aca="false">L17*J17*MAX(0,M17-N17)</f>
@@ -5839,11 +5839,11 @@
       </c>
       <c r="F18" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B18,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C18,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G18" s="22" t="n">
         <f aca="false">E18*F18</f>
-        <v>161.6</v>
+        <v>121.2</v>
       </c>
       <c r="H18" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A18,Portes!$H$5:$H$20)</f>
@@ -5855,7 +5855,7 @@
       </c>
       <c r="J18" s="22" t="n">
         <f aca="false">MAX(0,G18-H18)</f>
-        <v>161.6</v>
+        <v>121.2</v>
       </c>
       <c r="K18" s="18" t="n">
         <f aca="false">IF(I18="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B18,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C18,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -5875,7 +5875,7 @@
       </c>
       <c r="O18" s="24" t="n">
         <f aca="false">L18*J18*MAX(0,N18-M18)</f>
-        <v>296.266666666667</v>
+        <v>222.2</v>
       </c>
       <c r="P18" s="24" t="n">
         <f aca="false">L18*J18*MAX(0,M18-N18)</f>
@@ -5900,11 +5900,11 @@
       </c>
       <c r="F19" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B19,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C19,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G19" s="22" t="n">
         <f aca="false">E19*F19</f>
-        <v>55.96</v>
+        <v>41.97</v>
       </c>
       <c r="H19" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A19,Portes!$H$5:$H$20)</f>
@@ -5916,7 +5916,7 @@
       </c>
       <c r="J19" s="22" t="n">
         <f aca="false">MAX(0,G19-H19)</f>
-        <v>55.96</v>
+        <v>41.97</v>
       </c>
       <c r="K19" s="18" t="n">
         <f aca="false">IF(I19="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B19,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C19,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -5940,7 +5940,7 @@
       </c>
       <c r="P19" s="24" t="n">
         <f aca="false">L19*J19*MAX(0,M19-N19)</f>
-        <v>307.78</v>
+        <v>230.835</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5961,11 +5961,11 @@
       </c>
       <c r="F20" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B20,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C20,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G20" s="22" t="n">
         <f aca="false">E20*F20</f>
-        <v>41.32</v>
+        <v>30.99</v>
       </c>
       <c r="H20" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A20,Portes!$H$5:$H$20)</f>
@@ -5977,7 +5977,7 @@
       </c>
       <c r="J20" s="22" t="n">
         <f aca="false">MAX(0,G20-H20)</f>
-        <v>41.32</v>
+        <v>30.99</v>
       </c>
       <c r="K20" s="18" t="n">
         <f aca="false">IF(I20="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B20,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C20,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -6001,7 +6001,7 @@
       </c>
       <c r="P20" s="24" t="n">
         <f aca="false">L20*J20*MAX(0,M20-N20)</f>
-        <v>227.26</v>
+        <v>170.445</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6022,11 +6022,11 @@
       </c>
       <c r="F21" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B21,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C21,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G21" s="22" t="n">
         <f aca="false">E21*F21</f>
-        <v>79.88</v>
+        <v>59.91</v>
       </c>
       <c r="H21" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A21,Portes!$H$5:$H$20)</f>
@@ -6038,7 +6038,7 @@
       </c>
       <c r="J21" s="22" t="n">
         <f aca="false">MAX(0,G21-H21)</f>
-        <v>76.94</v>
+        <v>56.97</v>
       </c>
       <c r="K21" s="18" t="n">
         <f aca="false">IF(I21="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B21,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C21,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -6062,7 +6062,7 @@
       </c>
       <c r="P21" s="24" t="n">
         <f aca="false">L21*J21*MAX(0,M21-N21)</f>
-        <v>528.9625</v>
+        <v>391.66875</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6083,11 +6083,11 @@
       </c>
       <c r="F22" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B22,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C22,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G22" s="22" t="n">
         <f aca="false">E22*F22</f>
-        <v>46.4</v>
+        <v>34.8</v>
       </c>
       <c r="H22" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A22,Portes!$H$5:$H$20)</f>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="J22" s="22" t="n">
         <f aca="false">MAX(0,G22-H22)</f>
-        <v>46.4</v>
+        <v>34.8</v>
       </c>
       <c r="K22" s="18" t="n">
         <f aca="false">IF(I22="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B22,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C22,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -6123,7 +6123,7 @@
       </c>
       <c r="P22" s="24" t="n">
         <f aca="false">L22*J22*MAX(0,M22-N22)</f>
-        <v>255.2</v>
+        <v>191.4</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6144,11 +6144,11 @@
       </c>
       <c r="F23" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B23,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C23,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G23" s="22" t="n">
         <f aca="false">E23*F23</f>
-        <v>66.64</v>
+        <v>49.98</v>
       </c>
       <c r="H23" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A23,Portes!$H$5:$H$20)</f>
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J23" s="22" t="n">
         <f aca="false">MAX(0,G23-H23)</f>
-        <v>66.64</v>
+        <v>49.98</v>
       </c>
       <c r="K23" s="18" t="n">
         <f aca="false">IF(I23="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B23,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C23,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -6184,7 +6184,7 @@
       </c>
       <c r="P23" s="24" t="n">
         <f aca="false">L23*J23*MAX(0,M23-N23)</f>
-        <v>366.52</v>
+        <v>274.89</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6205,11 +6205,11 @@
       </c>
       <c r="F24" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B24,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C24,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G24" s="22" t="n">
         <f aca="false">E24*F24</f>
-        <v>31.44</v>
+        <v>23.58</v>
       </c>
       <c r="H24" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A24,Portes!$H$5:$H$20)</f>
@@ -6221,7 +6221,7 @@
       </c>
       <c r="J24" s="22" t="n">
         <f aca="false">MAX(0,G24-H24)</f>
-        <v>31.44</v>
+        <v>23.58</v>
       </c>
       <c r="K24" s="18" t="n">
         <f aca="false">IF(I24="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B24,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C24,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -6245,7 +6245,7 @@
       </c>
       <c r="P24" s="24" t="n">
         <f aca="false">L24*J24*MAX(0,M24-N24)</f>
-        <v>172.92</v>
+        <v>129.69</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6266,11 +6266,11 @@
       </c>
       <c r="F25" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B25,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C25,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G25" s="22" t="n">
         <f aca="false">E25*F25</f>
-        <v>17.6</v>
+        <v>13.2</v>
       </c>
       <c r="H25" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A25,Portes!$H$5:$H$20)</f>
@@ -6282,7 +6282,7 @@
       </c>
       <c r="J25" s="22" t="n">
         <f aca="false">MAX(0,G25-H25)</f>
-        <v>17.6</v>
+        <v>13.2</v>
       </c>
       <c r="K25" s="18" t="n">
         <f aca="false">IF(I25="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B25,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C25,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -6306,7 +6306,7 @@
       </c>
       <c r="P25" s="24" t="n">
         <f aca="false">L25*J25*MAX(0,M25-N25)</f>
-        <v>96.8</v>
+        <v>72.6</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6327,11 +6327,11 @@
       </c>
       <c r="F26" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B26,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C26,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G26" s="22" t="n">
         <f aca="false">E26*F26</f>
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="H26" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A26,Portes!$H$5:$H$20)</f>
@@ -6343,7 +6343,7 @@
       </c>
       <c r="J26" s="22" t="n">
         <f aca="false">MAX(0,G26-H26)</f>
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="K26" s="18" t="n">
         <f aca="false">IF(I26="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B26,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C26,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -6363,7 +6363,7 @@
       </c>
       <c r="O26" s="24" t="n">
         <f aca="false">L26*J26*MAX(0,N26-M26)</f>
-        <v>528</v>
+        <v>396</v>
       </c>
       <c r="P26" s="24" t="n">
         <f aca="false">L26*J26*MAX(0,M26-N26)</f>
@@ -6388,11 +6388,11 @@
       </c>
       <c r="F27" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B27,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C27,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G27" s="22" t="n">
         <f aca="false">E27*F27</f>
-        <v>79.88</v>
+        <v>59.91</v>
       </c>
       <c r="H27" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A27,Portes!$H$5:$H$20)</f>
@@ -6404,7 +6404,7 @@
       </c>
       <c r="J27" s="22" t="n">
         <f aca="false">MAX(0,G27-H27)</f>
-        <v>76.94</v>
+        <v>56.97</v>
       </c>
       <c r="K27" s="18" t="n">
         <f aca="false">IF(I27="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B27,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C27,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -6424,7 +6424,7 @@
       </c>
       <c r="O27" s="24" t="n">
         <f aca="false">L27*J27*MAX(0,N27-M27)</f>
-        <v>423.17</v>
+        <v>313.335</v>
       </c>
       <c r="P27" s="24" t="n">
         <f aca="false">L27*J27*MAX(0,M27-N27)</f>
@@ -6449,11 +6449,11 @@
       </c>
       <c r="F28" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B28,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C28,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G28" s="22" t="n">
         <f aca="false">E28*F28</f>
-        <v>83.44</v>
+        <v>62.58</v>
       </c>
       <c r="H28" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A28,Portes!$H$5:$H$20)</f>
@@ -6465,7 +6465,7 @@
       </c>
       <c r="J28" s="22" t="n">
         <f aca="false">MAX(0,G28-H28)</f>
-        <v>83.44</v>
+        <v>62.58</v>
       </c>
       <c r="K28" s="18" t="n">
         <f aca="false">IF(I28="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B28,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C28,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -6510,11 +6510,11 @@
       </c>
       <c r="F29" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B29,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C29,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G29" s="22" t="n">
         <f aca="false">E29*F29</f>
-        <v>31.44</v>
+        <v>23.58</v>
       </c>
       <c r="H29" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A29,Portes!$H$5:$H$20)</f>
@@ -6526,7 +6526,7 @@
       </c>
       <c r="J29" s="22" t="n">
         <f aca="false">MAX(0,G29-H29)</f>
-        <v>31.44</v>
+        <v>23.58</v>
       </c>
       <c r="K29" s="18" t="n">
         <f aca="false">IF(I29="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B29,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C29,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -6571,11 +6571,11 @@
       </c>
       <c r="F30" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B30,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C30,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G30" s="22" t="n">
         <f aca="false">E30*F30</f>
-        <v>22.4</v>
+        <v>16.8</v>
       </c>
       <c r="H30" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A30,Portes!$H$5:$H$20)</f>
@@ -6587,7 +6587,7 @@
       </c>
       <c r="J30" s="22" t="n">
         <f aca="false">MAX(0,G30-H30)</f>
-        <v>22.4</v>
+        <v>16.8</v>
       </c>
       <c r="K30" s="18" t="n">
         <f aca="false">IF(I30="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B30,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C30,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -6607,7 +6607,7 @@
       </c>
       <c r="O30" s="24" t="n">
         <f aca="false">L30*J30*MAX(0,N30-M30)</f>
-        <v>82.1333333333333</v>
+        <v>61.6</v>
       </c>
       <c r="P30" s="24" t="n">
         <f aca="false">L30*J30*MAX(0,M30-N30)</f>
@@ -6632,11 +6632,11 @@
       </c>
       <c r="F31" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B31,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C31,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G31" s="22" t="n">
         <f aca="false">E31*F31</f>
-        <v>22.4</v>
+        <v>16.8</v>
       </c>
       <c r="H31" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A31,Portes!$H$5:$H$20)</f>
@@ -6648,7 +6648,7 @@
       </c>
       <c r="J31" s="22" t="n">
         <f aca="false">MAX(0,G31-H31)</f>
-        <v>22.4</v>
+        <v>16.8</v>
       </c>
       <c r="K31" s="18" t="n">
         <f aca="false">IF(I31="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B31,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C31,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -6668,7 +6668,7 @@
       </c>
       <c r="O31" s="24" t="n">
         <f aca="false">L31*J31*MAX(0,N31-M31)</f>
-        <v>82.1333333333333</v>
+        <v>61.6</v>
       </c>
       <c r="P31" s="24" t="n">
         <f aca="false">L31*J31*MAX(0,M31-N31)</f>
@@ -6693,11 +6693,11 @@
       </c>
       <c r="F32" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B32,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C32,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G32" s="22" t="n">
         <f aca="false">E32*F32</f>
-        <v>22.4</v>
+        <v>16.8</v>
       </c>
       <c r="H32" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A32,Portes!$H$5:$H$20)</f>
@@ -6709,7 +6709,7 @@
       </c>
       <c r="J32" s="22" t="n">
         <f aca="false">MAX(0,G32-H32)</f>
-        <v>19.46</v>
+        <v>13.86</v>
       </c>
       <c r="K32" s="18" t="n">
         <f aca="false">IF(I32="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B32,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C32,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -6754,11 +6754,11 @@
       </c>
       <c r="F33" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B33,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C33,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G33" s="22" t="n">
         <f aca="false">E33*F33</f>
-        <v>154.72</v>
+        <v>116.04</v>
       </c>
       <c r="H33" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A33,Portes!$H$5:$H$20)</f>
@@ -6770,7 +6770,7 @@
       </c>
       <c r="J33" s="22" t="n">
         <f aca="false">MAX(0,G33-H33)</f>
-        <v>148.84</v>
+        <v>110.16</v>
       </c>
       <c r="K33" s="18" t="n">
         <f aca="false">IF(I33="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B33,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C33,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -6794,7 +6794,7 @@
       </c>
       <c r="P33" s="24" t="n">
         <f aca="false">L33*J33*MAX(0,M33-N33)</f>
-        <v>1091.49333333333</v>
+        <v>807.84</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6815,11 +6815,11 @@
       </c>
       <c r="F34" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B34,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C34,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G34" s="22" t="n">
         <f aca="false">E34*F34</f>
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="H34" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A34,Portes!$H$5:$H$20)</f>
@@ -6831,7 +6831,7 @@
       </c>
       <c r="J34" s="22" t="n">
         <f aca="false">MAX(0,G34-H34)</f>
-        <v>37.06</v>
+        <v>27.06</v>
       </c>
       <c r="K34" s="18" t="n">
         <f aca="false">IF(I34="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B34,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C34,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="P34" s="24" t="n">
         <f aca="false">L34*J34*MAX(0,M34-N34)</f>
-        <v>228.2896</v>
+        <v>166.6896</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6876,11 +6876,11 @@
       </c>
       <c r="F35" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B35,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C35,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G35" s="22" t="n">
         <f aca="false">E35*F35</f>
-        <v>120.08</v>
+        <v>90.06</v>
       </c>
       <c r="H35" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A35,Portes!$H$5:$H$20)</f>
@@ -6892,7 +6892,7 @@
       </c>
       <c r="J35" s="22" t="n">
         <f aca="false">MAX(0,G35-H35)</f>
-        <v>120.08</v>
+        <v>90.06</v>
       </c>
       <c r="K35" s="18" t="n">
         <f aca="false">IF(I35="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B35,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C35,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -6912,7 +6912,7 @@
       </c>
       <c r="O35" s="24" t="n">
         <f aca="false">L35*J35*MAX(0,N35-M35)</f>
-        <v>387.458133333333</v>
+        <v>290.5936</v>
       </c>
       <c r="P35" s="24" t="n">
         <f aca="false">L35*J35*MAX(0,M35-N35)</f>
@@ -6937,11 +6937,11 @@
       </c>
       <c r="F36" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B36,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C36,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G36" s="22" t="n">
         <f aca="false">E36*F36</f>
-        <v>120.08</v>
+        <v>90.06</v>
       </c>
       <c r="H36" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A36,Portes!$H$5:$H$20)</f>
@@ -6953,7 +6953,7 @@
       </c>
       <c r="J36" s="22" t="n">
         <f aca="false">MAX(0,G36-H36)</f>
-        <v>111.68</v>
+        <v>81.66</v>
       </c>
       <c r="K36" s="18" t="n">
         <f aca="false">IF(I36="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B36,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C36,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -6973,7 +6973,7 @@
       </c>
       <c r="O36" s="24" t="n">
         <f aca="false">L36*J36*MAX(0,N36-M36)</f>
-        <v>982.784</v>
+        <v>718.608</v>
       </c>
       <c r="P36" s="24" t="n">
         <f aca="false">L36*J36*MAX(0,M36-N36)</f>
@@ -6998,11 +6998,11 @@
       </c>
       <c r="F37" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B37,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C37,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G37" s="22" t="n">
         <f aca="false">E37*F37</f>
-        <v>154.72</v>
+        <v>116.04</v>
       </c>
       <c r="H37" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A37,Portes!$H$5:$H$20)</f>
@@ -7014,7 +7014,7 @@
       </c>
       <c r="J37" s="22" t="n">
         <f aca="false">MAX(0,G37-H37)</f>
-        <v>154.72</v>
+        <v>116.04</v>
       </c>
       <c r="K37" s="18" t="n">
         <f aca="false">IF(I37="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B37,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C37,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -7034,7 +7034,7 @@
       </c>
       <c r="O37" s="24" t="n">
         <f aca="false">L37*J37*MAX(0,N37-M37)</f>
-        <v>1021.152</v>
+        <v>765.864</v>
       </c>
       <c r="P37" s="24" t="n">
         <f aca="false">L37*J37*MAX(0,M37-N37)</f>
@@ -7059,11 +7059,11 @@
       </c>
       <c r="F38" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B38,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C38,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G38" s="22" t="n">
         <f aca="false">E38*F38</f>
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="H38" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A38,Portes!$H$5:$H$20)</f>
@@ -7075,7 +7075,7 @@
       </c>
       <c r="J38" s="22" t="n">
         <f aca="false">MAX(0,G38-H38)</f>
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K38" s="18" t="n">
         <f aca="false">IF(I38="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B38,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C38,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -7095,7 +7095,7 @@
       </c>
       <c r="O38" s="24" t="n">
         <f aca="false">L38*J38*MAX(0,N38-M38)</f>
-        <v>202.4</v>
+        <v>151.8</v>
       </c>
       <c r="P38" s="24" t="n">
         <f aca="false">L38*J38*MAX(0,M38-N38)</f>
@@ -7120,11 +7120,11 @@
       </c>
       <c r="F39" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B39,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C39,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G39" s="22" t="n">
         <f aca="false">E39*F39</f>
-        <v>120.08</v>
+        <v>90.06</v>
       </c>
       <c r="H39" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A39,Portes!$H$5:$H$20)</f>
@@ -7136,7 +7136,7 @@
       </c>
       <c r="J39" s="22" t="n">
         <f aca="false">MAX(0,G39-H39)</f>
-        <v>120.08</v>
+        <v>90.06</v>
       </c>
       <c r="K39" s="18" t="n">
         <f aca="false">IF(I39="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B39,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C39,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -7156,7 +7156,7 @@
       </c>
       <c r="O39" s="24" t="n">
         <f aca="false">L39*J39*MAX(0,N39-M39)</f>
-        <v>1003.8688</v>
+        <v>752.9016</v>
       </c>
       <c r="P39" s="24" t="n">
         <f aca="false">L39*J39*MAX(0,M39-N39)</f>
@@ -7181,11 +7181,11 @@
       </c>
       <c r="F40" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B40,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C40,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G40" s="22" t="n">
         <f aca="false">E40*F40</f>
-        <v>396</v>
+        <v>297</v>
       </c>
       <c r="H40" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A40,Portes!$H$5:$H$20)</f>
@@ -7197,7 +7197,7 @@
       </c>
       <c r="J40" s="22" t="n">
         <f aca="false">MAX(0,G40-H40)</f>
-        <v>390.12</v>
+        <v>291.12</v>
       </c>
       <c r="K40" s="18" t="n">
         <f aca="false">IF(I40="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B40,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C40,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -7242,11 +7242,11 @@
       </c>
       <c r="F41" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B41,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C41,Zones!$A$5:$A$14,0)),0))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G41" s="22" t="n">
         <f aca="false">E41*F41</f>
-        <v>140.8</v>
+        <v>105.6</v>
       </c>
       <c r="H41" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A41,Portes!$H$5:$H$20)</f>
@@ -7258,7 +7258,7 @@
       </c>
       <c r="J41" s="22" t="n">
         <f aca="false">MAX(0,G41-H41)</f>
-        <v>134.92</v>
+        <v>99.72</v>
       </c>
       <c r="K41" s="18" t="n">
         <f aca="false">IF(I41="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B41,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C41,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -7295,7 +7295,7 @@
       </c>
       <c r="G42" s="29" t="n">
         <f aca="false">SUM(G5:G41)</f>
-        <v>3568.52</v>
+        <v>2676.39</v>
       </c>
       <c r="H42" s="29" t="n">
         <f aca="false">SUM(H5:H41)</f>
@@ -7303,7 +7303,7 @@
       </c>
       <c r="J42" s="29" t="n">
         <f aca="false">SUM(J5:J41)</f>
-        <v>3515.81</v>
+        <v>2623.68</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7379,7 +7379,7 @@
       </c>
       <c r="B5" s="22" t="n">
         <f aca="false">SUMIFS(Parois!$J$5:$J$41,Parois!$K$5:$K$41,A5,Parois!$I$5:$I$41,"Oui")</f>
-        <v>535.32</v>
+        <v>397.92</v>
       </c>
       <c r="C5" s="22" t="n">
         <f aca="false">SUMIF(Zones!$L$5:$L$14,A5,Zones!$N$5:$N$14)</f>
@@ -7387,11 +7387,11 @@
       </c>
       <c r="D5" s="22" t="n">
         <f aca="false">B5+C5</f>
-        <v>825.6134</v>
+        <v>688.2134</v>
       </c>
       <c r="E5" s="22" t="n">
         <f aca="false">D5*(1+Hypothèses!$B$9)</f>
-        <v>866.89407</v>
+        <v>722.62407</v>
       </c>
       <c r="F5" s="34" t="n">
         <f aca="false">Hypothèses!C22</f>
@@ -7399,7 +7399,7 @@
       </c>
       <c r="G5" s="24" t="n">
         <f aca="false">E5*F5</f>
-        <v>364095.5094</v>
+        <v>303502.1094</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7409,7 +7409,7 @@
       </c>
       <c r="B6" s="22" t="n">
         <f aca="false">SUMIFS(Parois!$J$5:$J$41,Parois!$K$5:$K$41,A6,Parois!$I$5:$I$41,"Oui")</f>
-        <v>197.14</v>
+        <v>147.12</v>
       </c>
       <c r="C6" s="22" t="n">
         <f aca="false">SUMIF(Zones!$L$5:$L$14,A6,Zones!$N$5:$N$14)</f>
@@ -7417,11 +7417,11 @@
       </c>
       <c r="D6" s="22" t="n">
         <f aca="false">B6+C6</f>
-        <v>272.19</v>
+        <v>222.17</v>
       </c>
       <c r="E6" s="22" t="n">
         <f aca="false">D6*(1+Hypothèses!$B$9)</f>
-        <v>285.7995</v>
+        <v>233.2785</v>
       </c>
       <c r="F6" s="34" t="n">
         <f aca="false">Hypothèses!C23</f>
@@ -7429,7 +7429,7 @@
       </c>
       <c r="G6" s="24" t="n">
         <f aca="false">E6*F6</f>
-        <v>94313.835</v>
+        <v>76981.905</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7439,7 +7439,7 @@
       </c>
       <c r="B7" s="22" t="n">
         <f aca="false">SUMIFS(Parois!$J$5:$J$41,Parois!$K$5:$K$41,A7,Parois!$I$5:$I$41,"Oui")</f>
-        <v>477.24</v>
+        <v>356.46</v>
       </c>
       <c r="C7" s="22" t="n">
         <f aca="false">SUMIF(Zones!$L$5:$L$14,A7,Zones!$N$5:$N$14)</f>
@@ -7447,11 +7447,11 @@
       </c>
       <c r="D7" s="22" t="n">
         <f aca="false">B7+C7</f>
-        <v>628.81</v>
+        <v>508.03</v>
       </c>
       <c r="E7" s="22" t="n">
         <f aca="false">D7*(1+Hypothèses!$B$9)</f>
-        <v>660.2505</v>
+        <v>533.4315</v>
       </c>
       <c r="F7" s="34" t="n">
         <f aca="false">Hypothèses!C24</f>
@@ -7459,7 +7459,7 @@
       </c>
       <c r="G7" s="24" t="n">
         <f aca="false">E7*F7</f>
-        <v>191472.645</v>
+        <v>154695.135</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7469,7 +7469,7 @@
       </c>
       <c r="B8" s="22" t="n">
         <f aca="false">SUMIFS(Parois!$J$5:$J$41,Parois!$K$5:$K$41,A8,Parois!$I$5:$I$41,"Oui")</f>
-        <v>1781.07</v>
+        <v>1331.34</v>
       </c>
       <c r="C8" s="22" t="n">
         <f aca="false">SUMIF(Zones!$L$5:$L$14,A8,Zones!$N$5:$N$14)</f>
@@ -7477,11 +7477,11 @@
       </c>
       <c r="D8" s="22" t="n">
         <f aca="false">B8+C8</f>
-        <v>2840.3032</v>
+        <v>2390.5732</v>
       </c>
       <c r="E8" s="22" t="n">
         <f aca="false">D8*(1+Hypothèses!$B$9)</f>
-        <v>2982.31836</v>
+        <v>2510.10186</v>
       </c>
       <c r="F8" s="34" t="n">
         <f aca="false">Hypothèses!C25</f>
@@ -7489,7 +7489,7 @@
       </c>
       <c r="G8" s="24" t="n">
         <f aca="false">E8*F8</f>
-        <v>745579.59</v>
+        <v>627525.465</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7498,7 +7498,7 @@
       </c>
       <c r="B9" s="29" t="n">
         <f aca="false">SUM(B5:B8)</f>
-        <v>2990.77</v>
+        <v>2232.84</v>
       </c>
       <c r="C9" s="29" t="n">
         <f aca="false">SUM(C5:C8)</f>
@@ -7506,15 +7506,15 @@
       </c>
       <c r="D9" s="29" t="n">
         <f aca="false">SUM(D5:D8)</f>
-        <v>4566.9166</v>
+        <v>3808.9866</v>
       </c>
       <c r="E9" s="29" t="n">
         <f aca="false">SUM(E5:E8)</f>
-        <v>4795.26243</v>
+        <v>3999.43593</v>
       </c>
       <c r="G9" s="30" t="n">
         <f aca="false">SUM(G5:G8)</f>
-        <v>1395461.5794</v>
+        <v>1162704.6144</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7523,7 +7523,7 @@
       </c>
       <c r="G10" s="24" t="n">
         <f aca="false">G9*Hypothèses!$B$10</f>
-        <v>209319.23691</v>
+        <v>174405.69216</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7614,7 +7614,7 @@
       <c r="F18" s="28"/>
       <c r="G18" s="30" t="n">
         <f aca="false">G9+G10+D16</f>
-        <v>1910780.81631</v>
+        <v>1643110.30656</v>
       </c>
     </row>
   </sheetData>
@@ -7767,11 +7767,11 @@
       </c>
       <c r="F5" s="34" t="n">
         <f aca="false">Zones!H5</f>
-        <v>2313.0016</v>
+        <v>1734.7512</v>
       </c>
       <c r="G5" s="24" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A5,Parois!$O$5:$O$41)+SUMIF(Parois!$C$5:$C$41,A5,Parois!$P$5:$P$41)</f>
-        <v>1063.92</v>
+        <v>797.94</v>
       </c>
       <c r="H5" s="24" t="n">
         <f aca="false">IF(Zones!L5&gt;0,Hypothèses!$B$4/(Zones!L5/1000),0)*Zones!N5*MAX(0,Hypothèses!$B$14-D5)</f>
@@ -7838,7 +7838,7 @@
       </c>
       <c r="AA5" s="24" t="n">
         <f aca="false">G5+H5+I5+L5+P5+S5+T5+Z5</f>
-        <v>2124.04573333333</v>
+        <v>1858.06573333333</v>
       </c>
       <c r="AB5" s="10" t="n">
         <v>18</v>
@@ -7871,11 +7871,11 @@
       </c>
       <c r="F6" s="34" t="n">
         <f aca="false">Zones!H6</f>
-        <v>1503.04</v>
+        <v>1127.28</v>
       </c>
       <c r="G6" s="24" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A6,Parois!$O$5:$O$41)+SUMIF(Parois!$C$5:$C$41,A6,Parois!$P$5:$P$41)</f>
-        <v>567.783333333333</v>
+        <v>424.49</v>
       </c>
       <c r="H6" s="24" t="n">
         <f aca="false">IF(Zones!L6&gt;0,Hypothèses!$B$4/(Zones!L6/1000),0)*Zones!N6*MAX(0,Hypothèses!$B$14-D6)</f>
@@ -7942,7 +7942,7 @@
       </c>
       <c r="AA6" s="24" t="n">
         <f aca="false">G6+H6+I6+L6+P6+S6+T6+Z6</f>
-        <v>1256.67666666667</v>
+        <v>1113.38333333333</v>
       </c>
       <c r="AB6" s="10" t="n">
         <v>18</v>
@@ -7975,11 +7975,11 @@
       </c>
       <c r="F7" s="34" t="n">
         <f aca="false">Zones!H7</f>
-        <v>1366.4</v>
+        <v>1024.8</v>
       </c>
       <c r="G7" s="24" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A7,Parois!$O$5:$O$41)+SUMIF(Parois!$C$5:$C$41,A7,Parois!$P$5:$P$41)</f>
-        <v>146.666666666667</v>
+        <v>110</v>
       </c>
       <c r="H7" s="24" t="n">
         <f aca="false">IF(Zones!L7&gt;0,Hypothèses!$B$4/(Zones!L7/1000),0)*Zones!N7*MAX(0,Hypothèses!$B$14-D7)</f>
@@ -8046,7 +8046,7 @@
       </c>
       <c r="AA7" s="24" t="n">
         <f aca="false">G7+H7+I7+L7+P7+S7+T7+Z7</f>
-        <v>459.8</v>
+        <v>423.133333333333</v>
       </c>
       <c r="AB7" s="10" t="n">
         <v>18</v>
@@ -8079,11 +8079,11 @@
       </c>
       <c r="F8" s="34" t="n">
         <f aca="false">Zones!H8</f>
-        <v>1130.392</v>
+        <v>847.794</v>
       </c>
       <c r="G8" s="24" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A8,Parois!$O$5:$O$41)+SUMIF(Parois!$C$5:$C$41,A8,Parois!$P$5:$P$41)</f>
-        <v>290.876666666667</v>
+        <v>216.81</v>
       </c>
       <c r="H8" s="24" t="n">
         <f aca="false">IF(Zones!L8&gt;0,Hypothèses!$B$4/(Zones!L8/1000),0)*Zones!N8*MAX(0,Hypothèses!$B$14-D8)</f>
@@ -8150,7 +8150,7 @@
       </c>
       <c r="AA8" s="24" t="n">
         <f aca="false">G8+H8+I8+L8+P8+S8+T8+Z8</f>
-        <v>808.973</v>
+        <v>734.906333333333</v>
       </c>
       <c r="AB8" s="10" t="n">
         <v>18</v>
@@ -8183,11 +8183,11 @@
       </c>
       <c r="F9" s="34" t="n">
         <f aca="false">Zones!H9</f>
-        <v>1613.576</v>
+        <v>1210.182</v>
       </c>
       <c r="G9" s="24" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A9,Parois!$O$5:$O$41)+SUMIF(Parois!$C$5:$C$41,A9,Parois!$P$5:$P$41)</f>
-        <v>296.266666666667</v>
+        <v>222.2</v>
       </c>
       <c r="H9" s="24" t="n">
         <f aca="false">IF(Zones!L9&gt;0,Hypothèses!$B$4/(Zones!L9/1000),0)*Zones!N9*MAX(0,Hypothèses!$B$14-D9)</f>
@@ -8254,7 +8254,7 @@
       </c>
       <c r="AA9" s="24" t="n">
         <f aca="false">G9+H9+I9+L9+P9+S9+T9+Z9</f>
-        <v>666.0445</v>
+        <v>591.977833333333</v>
       </c>
       <c r="AB9" s="10" t="n">
         <v>18</v>
@@ -8287,11 +8287,11 @@
       </c>
       <c r="F10" s="34" t="n">
         <f aca="false">Zones!H10</f>
-        <v>1212.56</v>
+        <v>909.42</v>
       </c>
       <c r="G10" s="24" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A10,Parois!$O$5:$O$41)+SUMIF(Parois!$C$5:$C$41,A10,Parois!$P$5:$P$41)</f>
-        <v>2906.6125</v>
+        <v>2170.86375</v>
       </c>
       <c r="H10" s="24" t="n">
         <f aca="false">IF(Zones!L10&gt;0,Hypothèses!$B$4/(Zones!L10/1000),0)*Zones!N10*MAX(0,Hypothèses!$B$14-D10)</f>
@@ -8309,7 +8309,7 @@
       </c>
       <c r="L10" s="24" t="n">
         <f aca="false">J10*F10*Hypothèses!$B$5*K10*1000/86400</f>
-        <v>7578.5</v>
+        <v>5683.875</v>
       </c>
       <c r="M10" s="10" t="n">
         <v>6</v>
@@ -8358,14 +8358,14 @@
       </c>
       <c r="AA10" s="24" t="n">
         <f aca="false">G10+H10+I10+L10+P10+S10+T10+Z10</f>
-        <v>16495.4516666667</v>
+        <v>13865.0779166667</v>
       </c>
       <c r="AB10" s="10" t="n">
         <v>18</v>
       </c>
       <c r="AC10" s="37" t="n">
         <f aca="false">IF(C10="Oui",AA10*(1+Hypothèses!$B$8)*24/AB10/1000,0)</f>
-        <v>26.3927226666667</v>
+        <v>22.1841246666667</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8391,11 +8391,11 @@
       </c>
       <c r="F11" s="34" t="n">
         <f aca="false">Zones!H11</f>
-        <v>547.456</v>
+        <v>410.592</v>
       </c>
       <c r="G11" s="24" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A11,Parois!$O$5:$O$41)+SUMIF(Parois!$C$5:$C$41,A11,Parois!$P$5:$P$41)</f>
-        <v>164.266666666667</v>
+        <v>123.2</v>
       </c>
       <c r="H11" s="24" t="n">
         <f aca="false">IF(Zones!L11&gt;0,Hypothèses!$B$4/(Zones!L11/1000),0)*Zones!N11*MAX(0,Hypothèses!$B$14-D11)</f>
@@ -8462,7 +8462,7 @@
       </c>
       <c r="AA11" s="24" t="n">
         <f aca="false">G11+H11+I11+L11+P11+S11+T11+Z11</f>
-        <v>415.184</v>
+        <v>374.117333333333</v>
       </c>
       <c r="AB11" s="10" t="n">
         <v>18</v>
@@ -8495,11 +8495,11 @@
       </c>
       <c r="F12" s="34" t="n">
         <f aca="false">Zones!H12</f>
-        <v>2322.3472</v>
+        <v>1741.7604</v>
       </c>
       <c r="G12" s="24" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A12,Parois!$O$5:$O$41)+SUMIF(Parois!$C$5:$C$41,A12,Parois!$P$5:$P$41)</f>
-        <v>3482.88746666667</v>
+        <v>2582.9056</v>
       </c>
       <c r="H12" s="24" t="n">
         <f aca="false">IF(Zones!L12&gt;0,Hypothèses!$B$4/(Zones!L12/1000),0)*Zones!N12*MAX(0,Hypothèses!$B$14-D12)</f>
@@ -8517,7 +8517,7 @@
       </c>
       <c r="L12" s="24" t="n">
         <f aca="false">J12*F12*Hypothèses!$B$5*K12*1000/86400</f>
-        <v>8708.802</v>
+        <v>6531.6015</v>
       </c>
       <c r="M12" s="10" t="n">
         <v>2</v>
@@ -8566,14 +8566,14 @@
       </c>
       <c r="AA12" s="24" t="n">
         <f aca="false">G12+H12+I12+L12+P12+S12+T12+Z12</f>
-        <v>19481.8083940741</v>
+        <v>16404.6260274074</v>
       </c>
       <c r="AB12" s="10" t="n">
         <v>20</v>
       </c>
       <c r="AC12" s="37" t="n">
         <f aca="false">IF(C12="Oui",AA12*(1+Hypothèses!$B$8)*24/AB12/1000,0)</f>
-        <v>28.0538040874667</v>
+        <v>23.6226614794667</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8599,11 +8599,11 @@
       </c>
       <c r="F13" s="34" t="n">
         <f aca="false">Zones!H13</f>
-        <v>600.4</v>
+        <v>450.3</v>
       </c>
       <c r="G13" s="24" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A13,Parois!$O$5:$O$41)+SUMIF(Parois!$C$5:$C$41,A13,Parois!$P$5:$P$41)</f>
-        <v>1434.5584</v>
+        <v>1071.3912</v>
       </c>
       <c r="H13" s="24" t="n">
         <f aca="false">IF(Zones!L13&gt;0,Hypothèses!$B$4/(Zones!L13/1000),0)*Zones!N13*MAX(0,Hypothèses!$B$14-D13)</f>
@@ -8621,7 +8621,7 @@
       </c>
       <c r="L13" s="24" t="n">
         <f aca="false">J13*F13*Hypothèses!$B$5*K13*1000/86400</f>
-        <v>2001.33333333333</v>
+        <v>1501</v>
       </c>
       <c r="M13" s="10" t="n">
         <v>2</v>
@@ -8670,14 +8670,14 @@
       </c>
       <c r="AA13" s="24" t="n">
         <f aca="false">G13+H13+I13+L13+P13+S13+T13+Z13</f>
-        <v>5989.84232592593</v>
+        <v>5126.34179259259</v>
       </c>
       <c r="AB13" s="10" t="n">
         <v>18</v>
       </c>
       <c r="AC13" s="37" t="n">
         <f aca="false">IF(C13="Oui",AA13*(1+Hypothèses!$B$8)*24/AB13/1000,0)</f>
-        <v>9.58374772148148</v>
+        <v>8.20214686814815</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8703,11 +8703,11 @@
       </c>
       <c r="F14" s="34" t="n">
         <f aca="false">Zones!H14</f>
-        <v>2532.64</v>
+        <v>1899.48</v>
       </c>
       <c r="G14" s="24" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A14,Parois!$O$5:$O$41)+SUMIF(Parois!$C$5:$C$41,A14,Parois!$P$5:$P$41)</f>
-        <v>146.666666666667</v>
+        <v>110</v>
       </c>
       <c r="H14" s="24" t="n">
         <f aca="false">IF(Zones!L14&gt;0,Hypothèses!$B$4/(Zones!L14/1000),0)*Zones!N14*MAX(0,Hypothèses!$B$14-D14)</f>
@@ -8774,7 +8774,7 @@
       </c>
       <c r="AA14" s="24" t="n">
         <f aca="false">G14+H14+I14+L14+P14+S14+T14+Z14</f>
-        <v>146.666666666667</v>
+        <v>110</v>
       </c>
       <c r="AB14" s="10" t="n">
         <v>18</v>
@@ -8790,7 +8790,7 @@
       </c>
       <c r="AC15" s="38" t="n">
         <f aca="false">SUM(AC5:AC14)</f>
-        <v>64.0302744756148</v>
+        <v>54.0089330142815</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
P1 RDC v3: stérilisation 12.50 m with 6 Steriflow 1300 retorts
Wall between refroidissement (1) and stérilisation moved 2.5 m north
(8.50 / 12.50 m), its door moved to the east end next to a 1.87 m
passage. Six retorts drawn north-south (1.65 m wide, 0.95 m apart) with
0.58 m service strip and 4.50 m basket aisle, dimensioned. Area labels,
surface table, PDF and workbook updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011Ghrdsx3moo1sM21DD7JVm
</commit_message>
<xml_diff>
--- a/DWG_Plan_Modificatif/DWG Plan Modificatif/Unite Humide - dimensions panneaux froid.xlsx
+++ b/DWG_Plan_Modificatif/DWG Plan Modificatif/Unite Humide - dimensions panneaux froid.xlsx
@@ -1891,7 +1891,7 @@
     <t xml:space="preserve">Zone de stérilisation</t>
   </si>
   <si>
-    <t xml:space="preserve">Pas de mur entre stérilisation et sertissage sur le plan (espace ouvert sur 7,00 m).</t>
+    <t xml:space="preserve">6 autoclaves Steriflow 1300 (7 225 × ~1 650 mm, 10,4 t pleins d'eau chacun), allée paniers 4,50 m. Pas de mur entre stérilisation et sertissage sur le plan (espace ouvert sur 7,00 m).</t>
   </si>
   <si>
     <t xml:space="preserve">Z4</t>
@@ -3901,25 +3901,25 @@
         <v>88</v>
       </c>
       <c r="C6" s="21" t="n">
-        <v>11</v>
+        <v>8.5</v>
       </c>
       <c r="D6" s="21" t="n">
         <v>17.08</v>
       </c>
       <c r="E6" s="22" t="n">
         <f aca="false">C6*D6</f>
-        <v>187.88</v>
+        <v>145.18</v>
       </c>
       <c r="F6" s="23" t="n">
         <f aca="false">2*(C6+D6)</f>
-        <v>56.16</v>
+        <v>51.16</v>
       </c>
       <c r="G6" s="15" t="n">
         <v>6</v>
       </c>
       <c r="H6" s="24" t="n">
         <f aca="false">E6*G6</f>
-        <v>1127.28</v>
+        <v>871.08</v>
       </c>
       <c r="I6" s="25" t="s">
         <v>86</v>
@@ -3936,15 +3936,15 @@
       </c>
       <c r="M6" s="22" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A6,Parois!$J$5:$J$41)+SUMIF(Parois!$C$5:$C$41,A6,Parois!$J$5:$J$41)-SUMIFS(Parois!$J$5:$J$41,Parois!$B$5:$B$41,A6,Parois!$C$5:$C$41,A6)</f>
-        <v>331.08</v>
+        <v>301.08</v>
       </c>
       <c r="N6" s="22" t="n">
         <f aca="false">IF(I6="Oui",E6,0)</f>
-        <v>187.88</v>
+        <v>145.18</v>
       </c>
       <c r="O6" s="26"/>
     </row>
-    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
         <v>89</v>
       </c>
@@ -3952,25 +3952,25 @@
         <v>90</v>
       </c>
       <c r="C7" s="21" t="n">
-        <v>10</v>
+        <v>12.5</v>
       </c>
       <c r="D7" s="21" t="n">
         <v>17.08</v>
       </c>
       <c r="E7" s="22" t="n">
         <f aca="false">C7*D7</f>
-        <v>170.8</v>
+        <v>213.5</v>
       </c>
       <c r="F7" s="23" t="n">
         <f aca="false">2*(C7+D7)</f>
-        <v>54.16</v>
+        <v>59.16</v>
       </c>
       <c r="G7" s="15" t="n">
         <v>6</v>
       </c>
       <c r="H7" s="24" t="n">
         <f aca="false">E7*G7</f>
-        <v>1024.8</v>
+        <v>1281</v>
       </c>
       <c r="I7" s="25" t="s">
         <v>86</v>
@@ -3987,11 +3987,11 @@
       </c>
       <c r="M7" s="22" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A7,Parois!$J$5:$J$41)+SUMIF(Parois!$C$5:$C$41,A7,Parois!$J$5:$J$41)-SUMIFS(Parois!$J$5:$J$41,Parois!$B$5:$B$41,A7,Parois!$C$5:$C$41,A7)</f>
-        <v>279.45</v>
+        <v>309.45</v>
       </c>
       <c r="N7" s="22" t="n">
         <f aca="false">IF(I7="Oui",E7,0)</f>
-        <v>170.8</v>
+        <v>213.5</v>
       </c>
       <c r="O7" s="26" t="s">
         <v>91</v>
@@ -5347,7 +5347,7 @@
         <v>180</v>
       </c>
       <c r="E10" s="21" t="n">
-        <v>11</v>
+        <v>8.5</v>
       </c>
       <c r="F10" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B10,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C10,Zones!$A$5:$A$14,0)),0))</f>
@@ -5355,7 +5355,7 @@
       </c>
       <c r="G10" s="22" t="n">
         <f aca="false">E10*F10</f>
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="H10" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A10,Portes!$H$5:$H$20)</f>
@@ -5367,7 +5367,7 @@
       </c>
       <c r="J10" s="22" t="n">
         <f aca="false">MAX(0,G10-H10)</f>
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="K10" s="18" t="n">
         <f aca="false">IF(I10="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B10,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C10,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -5387,7 +5387,7 @@
       </c>
       <c r="O10" s="24" t="n">
         <f aca="false">L10*J10*MAX(0,N10-M10)</f>
-        <v>242</v>
+        <v>187</v>
       </c>
       <c r="P10" s="24" t="n">
         <f aca="false">L10*J10*MAX(0,M10-N10)</f>
@@ -5469,7 +5469,7 @@
         <v>183</v>
       </c>
       <c r="E12" s="21" t="n">
-        <v>11</v>
+        <v>8.5</v>
       </c>
       <c r="F12" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B12,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C12,Zones!$A$5:$A$14,0)),0))</f>
@@ -5477,7 +5477,7 @@
       </c>
       <c r="G12" s="22" t="n">
         <f aca="false">E12*F12</f>
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="H12" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A12,Portes!$H$5:$H$20)</f>
@@ -5489,7 +5489,7 @@
       </c>
       <c r="J12" s="22" t="n">
         <f aca="false">MAX(0,G12-H12)</f>
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="K12" s="18" t="n">
         <f aca="false">IF(I12="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B12,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C12,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -5530,7 +5530,7 @@
         <v>185</v>
       </c>
       <c r="E13" s="21" t="n">
-        <v>10</v>
+        <v>12.5</v>
       </c>
       <c r="F13" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B13,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C13,Zones!$A$5:$A$14,0)),0))</f>
@@ -5538,7 +5538,7 @@
       </c>
       <c r="G13" s="22" t="n">
         <f aca="false">E13*F13</f>
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="H13" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A13,Portes!$H$5:$H$20)</f>
@@ -5550,7 +5550,7 @@
       </c>
       <c r="J13" s="22" t="n">
         <f aca="false">MAX(0,G13-H13)</f>
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="K13" s="18" t="n">
         <f aca="false">IF(I13="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B13,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C13,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -5570,7 +5570,7 @@
       </c>
       <c r="O13" s="24" t="n">
         <f aca="false">L13*J13*MAX(0,N13-M13)</f>
-        <v>110</v>
+        <v>137.5</v>
       </c>
       <c r="P13" s="24" t="n">
         <f aca="false">L13*J13*MAX(0,M13-N13)</f>
@@ -5591,7 +5591,7 @@
         <v>187</v>
       </c>
       <c r="E14" s="21" t="n">
-        <v>10</v>
+        <v>12.5</v>
       </c>
       <c r="F14" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B14,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C14,Zones!$A$5:$A$14,0)),0))</f>
@@ -5599,7 +5599,7 @@
       </c>
       <c r="G14" s="22" t="n">
         <f aca="false">E14*F14</f>
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="H14" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$20,A14,Portes!$H$5:$H$20)</f>
@@ -5611,7 +5611,7 @@
       </c>
       <c r="J14" s="22" t="n">
         <f aca="false">MAX(0,G14-H14)</f>
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="K14" s="18" t="n">
         <f aca="false">IF(I14="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B14,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C14,Hypothèses!$A$37:$A$52,0))),0)</f>
@@ -5635,7 +5635,7 @@
       </c>
       <c r="P14" s="24" t="n">
         <f aca="false">L14*J14*MAX(0,M14-N14)</f>
-        <v>110</v>
+        <v>137.5</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7867,19 +7867,19 @@
       </c>
       <c r="E6" s="35" t="n">
         <f aca="false">Zones!E6</f>
-        <v>187.88</v>
+        <v>145.18</v>
       </c>
       <c r="F6" s="34" t="n">
         <f aca="false">Zones!H6</f>
-        <v>1127.28</v>
+        <v>871.08</v>
       </c>
       <c r="G6" s="24" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A6,Parois!$O$5:$O$41)+SUMIF(Parois!$C$5:$C$41,A6,Parois!$P$5:$P$41)</f>
-        <v>424.49</v>
+        <v>369.49</v>
       </c>
       <c r="H6" s="24" t="n">
         <f aca="false">IF(Zones!L6&gt;0,Hypothèses!$B$4/(Zones!L6/1000),0)*Zones!N6*MAX(0,Hypothèses!$B$14-D6)</f>
-        <v>688.893333333333</v>
+        <v>532.326666666667</v>
       </c>
       <c r="I6" s="24" t="n">
         <f aca="false">IF(D6&lt;0,Hypothèses!$B$6,Hypothèses!$B$7)*E6*MAX(0,Hypothèses!$B$15-D6)</f>
@@ -7942,7 +7942,7 @@
       </c>
       <c r="AA6" s="24" t="n">
         <f aca="false">G6+H6+I6+L6+P6+S6+T6+Z6</f>
-        <v>1113.38333333333</v>
+        <v>901.816666666667</v>
       </c>
       <c r="AB6" s="10" t="n">
         <v>18</v>
@@ -7971,19 +7971,19 @@
       </c>
       <c r="E7" s="35" t="n">
         <f aca="false">Zones!E7</f>
-        <v>170.8</v>
+        <v>213.5</v>
       </c>
       <c r="F7" s="34" t="n">
         <f aca="false">Zones!H7</f>
-        <v>1024.8</v>
+        <v>1281</v>
       </c>
       <c r="G7" s="24" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A7,Parois!$O$5:$O$41)+SUMIF(Parois!$C$5:$C$41,A7,Parois!$P$5:$P$41)</f>
-        <v>110</v>
+        <v>137.5</v>
       </c>
       <c r="H7" s="24" t="n">
         <f aca="false">IF(Zones!L7&gt;0,Hypothèses!$B$4/(Zones!L7/1000),0)*Zones!N7*MAX(0,Hypothèses!$B$14-D7)</f>
-        <v>313.133333333333</v>
+        <v>391.416666666667</v>
       </c>
       <c r="I7" s="24" t="n">
         <f aca="false">IF(D7&lt;0,Hypothèses!$B$6,Hypothèses!$B$7)*E7*MAX(0,Hypothèses!$B$15-D7)</f>
@@ -8046,7 +8046,7 @@
       </c>
       <c r="AA7" s="24" t="n">
         <f aca="false">G7+H7+I7+L7+P7+S7+T7+Z7</f>
-        <v>423.133333333333</v>
+        <v>528.916666666667</v>
       </c>
       <c r="AB7" s="10" t="n">
         <v>18</v>
@@ -8707,7 +8707,7 @@
       </c>
       <c r="G14" s="24" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A14,Parois!$O$5:$O$41)+SUMIF(Parois!$C$5:$C$41,A14,Parois!$P$5:$P$41)</f>
-        <v>110</v>
+        <v>137.5</v>
       </c>
       <c r="H14" s="24" t="n">
         <f aca="false">IF(Zones!L14&gt;0,Hypothèses!$B$4/(Zones!L14/1000),0)*Zones!N14*MAX(0,Hypothèses!$B$14-D14)</f>
@@ -8774,7 +8774,7 @@
       </c>
       <c r="AA14" s="24" t="n">
         <f aca="false">G14+H14+I14+L14+P14+S14+T14+Z14</f>
-        <v>110</v>
+        <v>137.5</v>
       </c>
       <c r="AB14" s="10" t="n">
         <v>18</v>

</xml_diff>

<commit_message>
P1 RDC v4: wet-process layout fitted to the equipment specs
Middle band of the Unité Humide redrawn around the vendor layouts:
- Préparation viande 22.35 x 6.20 m (+9.99 x 2.20 m): Karl Schnell
  mixer/emulsifier group, grinder with maintenance area, KS cabinet, and
  the JBT hopper / colour injection / extruder in line with the tunnel.
- Cuisson / extrusion 9.99 x 19.80 m: JBT 800x8000 steam tunnel through
  the prep wall, cooling conveyor, cutting unit, outfeed next to the
  door to sertissage; hood swing, MCC and exhausts shown.
- Sertissage 7.00 x 19.80 m: Waldner Dosomat 12.6 envelope.
New prep wall, doors (strip->prep, prep->sertissage, prep->cuisson) and
tunnel passage; dimensions, area labels, surface table, PDF and the
panel/refrigeration workbook updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011Ghrdsx3moo1sM21DD7JVm
</commit_message>
<xml_diff>
--- a/DWG_Plan_Modificatif/DWG Plan Modificatif/Unite Humide - dimensions panneaux froid.xlsx
+++ b/DWG_Plan_Modificatif/DWG Plan Modificatif/Unite Humide - dimensions panneaux froid.xlsx
@@ -713,6 +713,42 @@
         </r>
       </text>
     </comment>
+    <comment ref="F21" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Mesuré sur P1 RDC v2.dwg (RDC Modifié), entre nus intérieurs des murs</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F22" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Mesuré sur P1 RDC v2.dwg (RDC Modifié), entre nus intérieurs des murs</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F23" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Mesuré sur P1 RDC v2.dwg (RDC Modifié), entre nus intérieurs des murs</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -1616,7 +1652,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="280">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="287">
   <si>
     <t xml:space="preserve">Unité Humide – RDC Modifié (P1 RDC v2) : dimensions, panneaux sandwich et puissance frigorifique</t>
   </si>
@@ -1630,7 +1666,7 @@
     <t xml:space="preserve">• Parois : chaque mur une seule fois avec ses deux côtés → métré des panneaux sans double comptage, et flux thermiques.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Portes : 16 portes relevées sur le plan, surface déduite des murs.</t>
+    <t xml:space="preserve">• Portes : 18 portes + 1 passage de tunnel relevés sur le plan, surface déduite des murs.</t>
   </si>
   <si>
     <t xml:space="preserve">• Panneaux : quantités par épaisseur (murs + plafonds), chutes, prix, accessoires, portes → coût estimatif.</t>
@@ -1789,6 +1825,9 @@
     <t xml:space="preserve">Porte sectionnelle (quai)</t>
   </si>
   <si>
+    <t xml:space="preserve">Passage tunnel</t>
+  </si>
+  <si>
     <t xml:space="preserve">Hauteurs non cotées sur le plan : hypothèses. Prix = EXEMPLES, à remplacer.</t>
   </si>
   <si>
@@ -1900,16 +1939,16 @@
     <t xml:space="preserve">Zone de sertissage</t>
   </si>
   <si>
-    <t xml:space="preserve">Ouverte sur la stérilisation (voir Z3).</t>
+    <t xml:space="preserve">Waldner Dosomat 12.6 (2,88 × 5,35 m, ~20 kW). Ouverte sur l'allée des autoclaves.</t>
   </si>
   <si>
     <t xml:space="preserve">Z5</t>
   </si>
   <si>
-    <t xml:space="preserve">Zone de refroidissement (2) + cuisson</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Une seule pièce sur le plan (pas de cloison refroidissement / cuisson).</t>
+    <t xml:space="preserve">Zone de cuisson / extrusion (ligne JBT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tunnel vapeur JBT 800×8000 + convoyeur refroid. 800×4000 + découpe ; 2 extractions Ø356 à raccorder en toiture.</t>
   </si>
   <si>
     <t xml:space="preserve">Z6</t>
@@ -1921,7 +1960,7 @@
     <t xml:space="preserve">L</t>
   </si>
   <si>
-    <t xml:space="preserve">En L : 22,35 × 5,80 m + 9,99 × 2,20 m (surface et périmètre calculés sur la géométrie).</t>
+    <t xml:space="preserve">En L : 22,35 × 6,20 m + 9,99 × 2,20 m. Karl Schnell (mélangeur + émulsionneur, hachoir) + trémie / injection couleur / extrudeuse JBT.</t>
   </si>
   <si>
     <t xml:space="preserve">Z7</t>
@@ -2095,6 +2134,30 @@
     <t xml:space="preserve">Quai de déchargement : donne maintenant dans la chambre négative – à revoir.</t>
   </si>
   <si>
+    <t xml:space="preserve">D17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Circulation → préparation viande.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Préparation viande → sertissage.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Traversée du tunnel vapeur JBT (ouverture à habiller / calfeutrer).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Parois (chaque mur compté une seule fois) – longueurs mesurées sur le plan</t>
   </si>
   <si>
@@ -2185,22 +2248,19 @@
     <t xml:space="preserve">P12</t>
   </si>
   <si>
-    <t xml:space="preserve">Stérilisation / refroidissement (2) + cuisson</t>
+    <t xml:space="preserve">Stérilisation / cuisson</t>
   </si>
   <si>
     <t xml:space="preserve">Sertissage / circulation</t>
   </si>
   <si>
-    <t xml:space="preserve">Sertissage / refroidissement (2) + cuisson</t>
+    <t xml:space="preserve">Sertissage / cuisson</t>
   </si>
   <si>
     <t xml:space="preserve">P15</t>
   </si>
   <si>
-    <t xml:space="preserve">Refroidissement (2) + cuisson – façade est</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P16</t>
+    <t xml:space="preserve">Cuisson – façade est</t>
   </si>
   <si>
     <t xml:space="preserve">Sertissage / préparation viande</t>
@@ -2212,10 +2272,7 @@
     <t xml:space="preserve">Circulation / préparation viande (nord)</t>
   </si>
   <si>
-    <t xml:space="preserve">Refroidissement (2) + cuisson / préparation viande</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P19</t>
+    <t xml:space="preserve">Cuisson / préparation viande (passage tunnel JBT)</t>
   </si>
   <si>
     <t xml:space="preserve">Circulation / préparation viande (ouest)</t>
@@ -3183,7 +3240,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D52"/>
+  <dimension ref="A1:D53"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
@@ -3465,237 +3522,233 @@
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="13" t="s">
+      <c r="A33" s="14" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="5" t="s">
+      <c r="B33" s="15" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="C33" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="13" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="11" t="s">
+      <c r="A36" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="B36" s="11" t="s">
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="C36" s="11" t="s">
+      <c r="B37" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C37" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="D36" s="11" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="16" t="str">
+      <c r="D37" s="11" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="16" t="str">
         <f aca="false">Zones!A5</f>
         <v>Z1</v>
       </c>
-      <c r="B37" s="17" t="n">
+      <c r="B38" s="17" t="n">
         <f aca="false">Zones!K5</f>
         <v>30</v>
       </c>
-      <c r="C37" s="17" t="n">
+      <c r="C38" s="17" t="n">
         <f aca="false">Zones!L5</f>
         <v>60</v>
       </c>
-      <c r="D37" s="16" t="str">
+      <c r="D38" s="16" t="str">
         <f aca="false">Zones!I5</f>
         <v>Oui</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="16" t="str">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="16" t="str">
         <f aca="false">Zones!A6</f>
         <v>Z2</v>
       </c>
-      <c r="B38" s="17" t="n">
+      <c r="B39" s="17" t="n">
         <f aca="false">Zones!K6</f>
         <v>30</v>
       </c>
-      <c r="C38" s="17" t="n">
+      <c r="C39" s="17" t="n">
         <f aca="false">Zones!L6</f>
         <v>60</v>
       </c>
-      <c r="D38" s="16" t="str">
+      <c r="D39" s="16" t="str">
         <f aca="false">Zones!I6</f>
         <v>Oui</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="16" t="str">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="16" t="str">
         <f aca="false">Zones!A7</f>
         <v>Z3</v>
       </c>
-      <c r="B39" s="17" t="n">
+      <c r="B40" s="17" t="n">
         <f aca="false">Zones!K7</f>
         <v>35</v>
       </c>
-      <c r="C39" s="17" t="n">
+      <c r="C40" s="17" t="n">
         <f aca="false">Zones!L7</f>
         <v>60</v>
       </c>
-      <c r="D39" s="16" t="str">
+      <c r="D40" s="16" t="str">
         <f aca="false">Zones!I7</f>
         <v>Oui</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="16" t="str">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="16" t="str">
         <f aca="false">Zones!A8</f>
         <v>Z4</v>
       </c>
-      <c r="B40" s="17" t="n">
+      <c r="B41" s="17" t="n">
         <f aca="false">Zones!K8</f>
         <v>30</v>
       </c>
-      <c r="C40" s="17" t="n">
+      <c r="C41" s="17" t="n">
         <f aca="false">Zones!L8</f>
         <v>60</v>
       </c>
-      <c r="D40" s="16" t="str">
+      <c r="D41" s="16" t="str">
         <f aca="false">Zones!I8</f>
         <v>Oui</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="16" t="str">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="16" t="str">
         <f aca="false">Zones!A9</f>
         <v>Z5</v>
       </c>
-      <c r="B41" s="17" t="n">
+      <c r="B42" s="17" t="n">
         <f aca="false">Zones!K9</f>
         <v>35</v>
       </c>
-      <c r="C41" s="17" t="n">
+      <c r="C42" s="17" t="n">
         <f aca="false">Zones!L9</f>
         <v>60</v>
       </c>
-      <c r="D41" s="16" t="str">
+      <c r="D42" s="16" t="str">
         <f aca="false">Zones!I9</f>
         <v>Oui</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="16" t="str">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="16" t="str">
         <f aca="false">Zones!A10</f>
         <v>Z6</v>
       </c>
-      <c r="B42" s="17" t="n">
+      <c r="B43" s="17" t="n">
         <f aca="false">Zones!K10</f>
         <v>10</v>
       </c>
-      <c r="C42" s="17" t="n">
+      <c r="C43" s="17" t="n">
         <f aca="false">Zones!L10</f>
         <v>80</v>
       </c>
-      <c r="D42" s="16" t="str">
+      <c r="D43" s="16" t="str">
         <f aca="false">Zones!I10</f>
         <v>Oui</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="16" t="str">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="16" t="str">
         <f aca="false">Zones!A11</f>
         <v>Z7</v>
       </c>
-      <c r="B43" s="17" t="n">
+      <c r="B44" s="17" t="n">
         <f aca="false">Zones!K11</f>
         <v>30</v>
       </c>
-      <c r="C43" s="17" t="n">
+      <c r="C44" s="17" t="n">
         <f aca="false">Zones!L11</f>
         <v>60</v>
       </c>
-      <c r="D43" s="16" t="str">
+      <c r="D44" s="16" t="str">
         <f aca="false">Zones!I11</f>
         <v>Oui</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="16" t="str">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="16" t="str">
         <f aca="false">Zones!A12</f>
         <v>Z8</v>
       </c>
-      <c r="B44" s="17" t="n">
+      <c r="B45" s="17" t="n">
         <f aca="false">Zones!K12</f>
         <v>-20</v>
       </c>
-      <c r="C44" s="17" t="n">
+      <c r="C45" s="17" t="n">
         <f aca="false">Zones!L12</f>
         <v>150</v>
       </c>
-      <c r="D44" s="16" t="str">
+      <c r="D45" s="16" t="str">
         <f aca="false">Zones!I12</f>
         <v>Oui</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="16" t="str">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="16" t="str">
         <f aca="false">Zones!A13</f>
         <v>Z9</v>
       </c>
-      <c r="B45" s="17" t="n">
+      <c r="B46" s="17" t="n">
         <f aca="false">Zones!K13</f>
         <v>2</v>
       </c>
-      <c r="C45" s="17" t="n">
+      <c r="C46" s="17" t="n">
         <f aca="false">Zones!L13</f>
         <v>100</v>
       </c>
-      <c r="D45" s="16" t="str">
+      <c r="D46" s="16" t="str">
         <f aca="false">Zones!I13</f>
         <v>Oui</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="16" t="str">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="16" t="str">
         <f aca="false">Zones!A14</f>
         <v>Z10</v>
       </c>
-      <c r="B46" s="17" t="n">
+      <c r="B47" s="17" t="n">
         <f aca="false">Zones!K14</f>
         <v>30</v>
       </c>
-      <c r="C46" s="17" t="n">
+      <c r="C47" s="17" t="n">
         <f aca="false">Zones!L14</f>
         <v>0</v>
       </c>
-      <c r="D46" s="16" t="str">
+      <c r="D47" s="16" t="str">
         <f aca="false">Zones!I14</f>
         <v>Non</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="B47" s="18" t="n">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="B48" s="18" t="n">
         <f aca="false">Hypothèses!$B$13</f>
         <v>40</v>
       </c>
-      <c r="C47" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="D47" s="14" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="14" t="s">
+      <c r="C48" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" s="14" t="s">
         <v>64</v>
-      </c>
-      <c r="B48" s="18" t="n">
-        <f aca="false">Hypothèses!$B$14</f>
-        <v>40</v>
-      </c>
-      <c r="C48" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="D48" s="14" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3703,14 +3756,14 @@
         <v>65</v>
       </c>
       <c r="B49" s="18" t="n">
-        <f aca="false">Hypothèses!$B$15</f>
-        <v>20</v>
+        <f aca="false">Hypothèses!$B$14</f>
+        <v>40</v>
       </c>
       <c r="C49" s="18" t="n">
         <v>0</v>
       </c>
       <c r="D49" s="14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3718,14 +3771,14 @@
         <v>66</v>
       </c>
       <c r="B50" s="18" t="n">
-        <f aca="false">Hypothèses!$B$16</f>
-        <v>30</v>
+        <f aca="false">Hypothèses!$B$15</f>
+        <v>20</v>
       </c>
       <c r="C50" s="18" t="n">
         <v>0</v>
       </c>
       <c r="D50" s="14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3733,14 +3786,14 @@
         <v>67</v>
       </c>
       <c r="B51" s="18" t="n">
-        <f aca="false">Hypothèses!$B$17</f>
-        <v>25</v>
+        <f aca="false">Hypothèses!$B$16</f>
+        <v>30</v>
       </c>
       <c r="C51" s="18" t="n">
         <v>0</v>
       </c>
       <c r="D51" s="14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3748,14 +3801,29 @@
         <v>68</v>
       </c>
       <c r="B52" s="18" t="n">
+        <f aca="false">Hypothèses!$B$17</f>
+        <v>25</v>
+      </c>
+      <c r="C52" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D52" s="14" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="B53" s="18" t="n">
         <f aca="false">Hypothèses!$B$18</f>
         <v>30</v>
       </c>
-      <c r="C52" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="D52" s="14" t="s">
-        <v>63</v>
+      <c r="C53" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" s="14" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -3787,67 +3855,67 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I4" s="19" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J4" s="19" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="K4" s="19" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L4" s="19" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="M4" s="19" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N4" s="19" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="O4" s="19" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="20" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C5" s="21" t="n">
         <v>11.83</v>
@@ -3871,10 +3939,10 @@
         <v>1734.7512</v>
       </c>
       <c r="I5" s="25" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J5" s="25" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K5" s="10" t="n">
         <v>30</v>
@@ -3895,10 +3963,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C6" s="21" t="n">
         <v>8.5</v>
@@ -3922,10 +3990,10 @@
         <v>871.08</v>
       </c>
       <c r="I6" s="25" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J6" s="25" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K6" s="10" t="n">
         <v>30</v>
@@ -3946,10 +4014,10 @@
     </row>
     <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C7" s="21" t="n">
         <v>12.5</v>
@@ -3973,10 +4041,10 @@
         <v>1281</v>
       </c>
       <c r="I7" s="25" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J7" s="25" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K7" s="10" t="n">
         <v>35</v>
@@ -3994,42 +4062,42 @@
         <v>213.5</v>
       </c>
       <c r="O7" s="26" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C8" s="21" t="n">
-        <v>20.2</v>
+        <v>19.8</v>
       </c>
       <c r="D8" s="21" t="n">
         <v>6.995</v>
       </c>
       <c r="E8" s="22" t="n">
         <f aca="false">C8*D8</f>
-        <v>141.299</v>
+        <v>138.501</v>
       </c>
       <c r="F8" s="23" t="n">
         <f aca="false">2*(C8+D8)</f>
-        <v>54.39</v>
+        <v>53.59</v>
       </c>
       <c r="G8" s="15" t="n">
         <v>6</v>
       </c>
       <c r="H8" s="24" t="n">
         <f aca="false">E8*G8</f>
-        <v>847.794</v>
+        <v>831.006</v>
       </c>
       <c r="I8" s="25" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J8" s="25" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K8" s="10" t="n">
         <v>30</v>
@@ -4040,49 +4108,49 @@
       </c>
       <c r="M8" s="22" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A8,Parois!$J$5:$J$41)+SUMIF(Parois!$C$5:$C$41,A8,Parois!$J$5:$J$41)-SUMIFS(Parois!$J$5:$J$41,Parois!$B$5:$B$41,A8,Parois!$C$5:$C$41,A8)</f>
-        <v>278.49</v>
+        <v>270.75</v>
       </c>
       <c r="N8" s="22" t="n">
         <f aca="false">IF(I8="Oui",E8,0)</f>
-        <v>141.299</v>
+        <v>138.501</v>
       </c>
       <c r="O8" s="26" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C9" s="21" t="n">
-        <v>20.2</v>
+        <v>19.8</v>
       </c>
       <c r="D9" s="21" t="n">
         <v>9.985</v>
       </c>
       <c r="E9" s="22" t="n">
         <f aca="false">C9*D9</f>
-        <v>201.697</v>
+        <v>197.703</v>
       </c>
       <c r="F9" s="23" t="n">
         <f aca="false">2*(C9+D9)</f>
-        <v>60.37</v>
+        <v>59.57</v>
       </c>
       <c r="G9" s="15" t="n">
         <v>6</v>
       </c>
       <c r="H9" s="24" t="n">
         <f aca="false">E9*G9</f>
-        <v>1210.182</v>
+        <v>1186.218</v>
       </c>
       <c r="I9" s="25" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J9" s="25" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K9" s="10" t="n">
         <v>35</v>
@@ -4093,47 +4161,47 @@
       </c>
       <c r="M9" s="22" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A9,Parois!$J$5:$J$41)+SUMIF(Parois!$C$5:$C$41,A9,Parois!$J$5:$J$41)-SUMIFS(Parois!$J$5:$J$41,Parois!$B$5:$B$41,A9,Parois!$C$5:$C$41,A9)</f>
-        <v>356.34</v>
+        <v>345.94</v>
       </c>
       <c r="N9" s="22" t="n">
         <f aca="false">IF(I9="Oui",E9,0)</f>
-        <v>201.697</v>
+        <v>197.703</v>
       </c>
       <c r="O9" s="26" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E10" s="27" t="n">
-        <v>151.57</v>
+        <v>160.51</v>
       </c>
       <c r="F10" s="21" t="n">
-        <v>60.69</v>
+        <v>61.49</v>
       </c>
       <c r="G10" s="15" t="n">
         <v>6</v>
       </c>
       <c r="H10" s="24" t="n">
         <f aca="false">E10*G10</f>
-        <v>909.42</v>
+        <v>963.06</v>
       </c>
       <c r="I10" s="25" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J10" s="25" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K10" s="10" t="n">
         <v>10</v>
@@ -4144,22 +4212,22 @@
       </c>
       <c r="M10" s="22" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A10,Parois!$J$5:$J$41)+SUMIF(Parois!$C$5:$C$41,A10,Parois!$J$5:$J$41)-SUMIFS(Parois!$J$5:$J$41,Parois!$B$5:$B$41,A10,Parois!$C$5:$C$41,A10)</f>
-        <v>356.46</v>
+        <v>349.78</v>
       </c>
       <c r="N10" s="22" t="n">
         <f aca="false">IF(I10="Oui",E10,0)</f>
-        <v>151.57</v>
+        <v>160.51</v>
       </c>
       <c r="O10" s="26" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C11" s="21" t="n">
         <v>2.8</v>
@@ -4183,10 +4251,10 @@
         <v>410.592</v>
       </c>
       <c r="I11" s="25" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J11" s="25" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K11" s="10" t="n">
         <v>30</v>
@@ -4204,15 +4272,15 @@
         <v>68.432</v>
       </c>
       <c r="O11" s="26" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C12" s="21" t="n">
         <v>15.01</v>
@@ -4236,10 +4304,10 @@
         <v>1741.7604</v>
       </c>
       <c r="I12" s="25" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J12" s="25" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K12" s="10" t="n">
         <v>-20</v>
@@ -4257,15 +4325,15 @@
         <v>290.2934</v>
       </c>
       <c r="O12" s="26" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C13" s="21" t="n">
         <v>15.01</v>
@@ -4289,10 +4357,10 @@
         <v>450.3</v>
       </c>
       <c r="I13" s="25" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J13" s="25" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K13" s="10" t="n">
         <v>2</v>
@@ -4313,19 +4381,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E14" s="27" t="n">
-        <v>316.58</v>
+        <v>314.48</v>
       </c>
       <c r="F14" s="21" t="n">
         <v>130.38</v>
@@ -4335,13 +4403,13 @@
       </c>
       <c r="H14" s="24" t="n">
         <f aca="false">E14*G14</f>
-        <v>1899.48</v>
+        <v>1886.88</v>
       </c>
       <c r="I14" s="25" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J14" s="25" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K14" s="10" t="n">
         <v>30</v>
@@ -4352,35 +4420,35 @@
       </c>
       <c r="M14" s="22" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A14,Parois!$J$5:$J$41)+SUMIF(Parois!$C$5:$C$41,A14,Parois!$J$5:$J$41)-SUMIFS(Parois!$J$5:$J$41,Parois!$B$5:$B$41,A14,Parois!$C$5:$C$41,A14)</f>
-        <v>857.01</v>
+        <v>854.07</v>
       </c>
       <c r="N14" s="22" t="n">
         <f aca="false">IF(I14="Oui",E14,0)</f>
         <v>0</v>
       </c>
       <c r="O14" s="26" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="28" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E15" s="29" t="n">
         <f aca="false">SUM(E5:E14)</f>
-        <v>1892.7266</v>
+        <v>1892.7746</v>
       </c>
       <c r="H15" s="30" t="n">
         <f aca="false">SUM(H5:H14)</f>
-        <v>11356.3596</v>
+        <v>11356.6476</v>
       </c>
       <c r="M15" s="29" t="n">
         <f aca="false">SUM(M5:M14)</f>
-        <v>3850.29</v>
+        <v>3822.53</v>
       </c>
       <c r="N15" s="29" t="n">
         <f aca="false">SUM(N5:N14)</f>
-        <v>1576.1466</v>
+        <v>1578.2946</v>
       </c>
     </row>
   </sheetData>
@@ -4406,7 +4474,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -4418,55 +4486,55 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E4" s="19" t="s">
         <v>51</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G4" s="19" t="s">
         <v>52</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I4" s="19" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="20" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E5" s="14" t="s">
         <v>55</v>
@@ -4475,7 +4543,7 @@
         <v>1.5</v>
       </c>
       <c r="G5" s="31" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$30:$B$32,MATCH(E5,Hypothèses!$A$30:$A$32,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$30:$B$33,MATCH(E5,Hypothèses!$A$30:$A$33,0))</f>
         <v>2.1</v>
       </c>
       <c r="H5" s="22" t="n">
@@ -4483,21 +4551,21 @@
         <v>3.15</v>
       </c>
       <c r="I5" s="26" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E6" s="14" t="s">
         <v>54</v>
@@ -4506,7 +4574,7 @@
         <v>1.4</v>
       </c>
       <c r="G6" s="31" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$30:$B$32,MATCH(E6,Hypothèses!$A$30:$A$32,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$30:$B$33,MATCH(E6,Hypothèses!$A$30:$A$33,0))</f>
         <v>2.1</v>
       </c>
       <c r="H6" s="22" t="n">
@@ -4517,16 +4585,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E7" s="14" t="s">
         <v>54</v>
@@ -4535,7 +4603,7 @@
         <v>1.4</v>
       </c>
       <c r="G7" s="31" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$30:$B$32,MATCH(E7,Hypothèses!$A$30:$A$32,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$30:$B$33,MATCH(E7,Hypothèses!$A$30:$A$33,0))</f>
         <v>2.1</v>
       </c>
       <c r="H7" s="22" t="n">
@@ -4546,16 +4614,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E8" s="14" t="s">
         <v>54</v>
@@ -4564,7 +4632,7 @@
         <v>1.4</v>
       </c>
       <c r="G8" s="31" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$30:$B$32,MATCH(E8,Hypothèses!$A$30:$A$32,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$30:$B$33,MATCH(E8,Hypothèses!$A$30:$A$33,0))</f>
         <v>2.1</v>
       </c>
       <c r="H8" s="22" t="n">
@@ -4575,16 +4643,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E9" s="14" t="s">
         <v>54</v>
@@ -4593,7 +4661,7 @@
         <v>1.4</v>
       </c>
       <c r="G9" s="31" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$30:$B$32,MATCH(E9,Hypothèses!$A$30:$A$32,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$30:$B$33,MATCH(E9,Hypothèses!$A$30:$A$33,0))</f>
         <v>2.1</v>
       </c>
       <c r="H9" s="22" t="n">
@@ -4604,16 +4672,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E10" s="14" t="s">
         <v>54</v>
@@ -4622,7 +4690,7 @@
         <v>1.4</v>
       </c>
       <c r="G10" s="31" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$30:$B$32,MATCH(E10,Hypothèses!$A$30:$A$32,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$30:$B$33,MATCH(E10,Hypothèses!$A$30:$A$33,0))</f>
         <v>2.1</v>
       </c>
       <c r="H10" s="22" t="n">
@@ -4633,16 +4701,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E11" s="14" t="s">
         <v>54</v>
@@ -4651,7 +4719,7 @@
         <v>1.4</v>
       </c>
       <c r="G11" s="31" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$30:$B$32,MATCH(E11,Hypothèses!$A$30:$A$32,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$30:$B$33,MATCH(E11,Hypothèses!$A$30:$A$33,0))</f>
         <v>2.1</v>
       </c>
       <c r="H11" s="22" t="n">
@@ -4662,16 +4730,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E12" s="14" t="s">
         <v>54</v>
@@ -4680,7 +4748,7 @@
         <v>1.4</v>
       </c>
       <c r="G12" s="31" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$30:$B$32,MATCH(E12,Hypothèses!$A$30:$A$32,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$30:$B$33,MATCH(E12,Hypothèses!$A$30:$A$33,0))</f>
         <v>2.1</v>
       </c>
       <c r="H12" s="22" t="n">
@@ -4688,21 +4756,21 @@
         <v>2.94</v>
       </c>
       <c r="I12" s="26" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E13" s="14" t="s">
         <v>54</v>
@@ -4711,7 +4779,7 @@
         <v>1.4</v>
       </c>
       <c r="G13" s="31" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$30:$B$32,MATCH(E13,Hypothèses!$A$30:$A$32,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$30:$B$33,MATCH(E13,Hypothèses!$A$30:$A$33,0))</f>
         <v>2.1</v>
       </c>
       <c r="H13" s="22" t="n">
@@ -4719,21 +4787,21 @@
         <v>2.94</v>
       </c>
       <c r="I13" s="26" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E14" s="14" t="s">
         <v>54</v>
@@ -4742,7 +4810,7 @@
         <v>1.4</v>
       </c>
       <c r="G14" s="31" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$30:$B$32,MATCH(E14,Hypothèses!$A$30:$A$32,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$30:$B$33,MATCH(E14,Hypothèses!$A$30:$A$33,0))</f>
         <v>2.1</v>
       </c>
       <c r="H14" s="22" t="n">
@@ -4750,21 +4818,21 @@
         <v>2.94</v>
       </c>
       <c r="I14" s="26" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E15" s="14" t="s">
         <v>54</v>
@@ -4773,7 +4841,7 @@
         <v>1.4</v>
       </c>
       <c r="G15" s="31" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$30:$B$32,MATCH(E15,Hypothèses!$A$30:$A$32,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$30:$B$33,MATCH(E15,Hypothèses!$A$30:$A$33,0))</f>
         <v>2.1</v>
       </c>
       <c r="H15" s="22" t="n">
@@ -4784,16 +4852,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="20" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E16" s="14" t="s">
         <v>54</v>
@@ -4802,7 +4870,7 @@
         <v>1.4</v>
       </c>
       <c r="G16" s="31" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$30:$B$32,MATCH(E16,Hypothèses!$A$30:$A$32,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$30:$B$33,MATCH(E16,Hypothèses!$A$30:$A$33,0))</f>
         <v>2.1</v>
       </c>
       <c r="H16" s="22" t="n">
@@ -4810,21 +4878,21 @@
         <v>2.94</v>
       </c>
       <c r="I16" s="26" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E17" s="14" t="s">
         <v>54</v>
@@ -4833,7 +4901,7 @@
         <v>1.4</v>
       </c>
       <c r="G17" s="31" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$30:$B$32,MATCH(E17,Hypothèses!$A$30:$A$32,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$30:$B$33,MATCH(E17,Hypothèses!$A$30:$A$33,0))</f>
         <v>2.1</v>
       </c>
       <c r="H17" s="22" t="n">
@@ -4841,21 +4909,21 @@
         <v>2.94</v>
       </c>
       <c r="I17" s="26" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="20" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E18" s="14" t="s">
         <v>54</v>
@@ -4864,7 +4932,7 @@
         <v>1.4</v>
       </c>
       <c r="G18" s="31" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$30:$B$32,MATCH(E18,Hypothèses!$A$30:$A$32,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$30:$B$33,MATCH(E18,Hypothèses!$A$30:$A$33,0))</f>
         <v>2.1</v>
       </c>
       <c r="H18" s="22" t="n">
@@ -4872,21 +4940,21 @@
         <v>2.94</v>
       </c>
       <c r="I18" s="26" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="20" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E19" s="14" t="s">
         <v>54</v>
@@ -4895,7 +4963,7 @@
         <v>1.4</v>
       </c>
       <c r="G19" s="31" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$30:$B$32,MATCH(E19,Hypothèses!$A$30:$A$32,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$30:$B$33,MATCH(E19,Hypothèses!$A$30:$A$33,0))</f>
         <v>2.1</v>
       </c>
       <c r="H19" s="22" t="n">
@@ -4903,21 +4971,21 @@
         <v>2.94</v>
       </c>
       <c r="I19" s="26" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E20" s="14" t="s">
         <v>56</v>
@@ -4926,7 +4994,7 @@
         <v>2.8</v>
       </c>
       <c r="G20" s="31" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$30:$B$32,MATCH(E20,Hypothèses!$A$30:$A$32,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$30:$B$33,MATCH(E20,Hypothèses!$A$30:$A$33,0))</f>
         <v>3</v>
       </c>
       <c r="H20" s="22" t="n">
@@ -4934,7 +5002,100 @@
         <v>8.4</v>
       </c>
       <c r="I20" s="26" t="s">
-        <v>158</v>
+        <v>159</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="20" t="s">
+        <v>160</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="D21" s="14" t="s">
+        <v>161</v>
+      </c>
+      <c r="E21" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="F21" s="21" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G21" s="31" t="n">
+        <f aca="false">INDEX(Hypothèses!$B$30:$B$33,MATCH(E21,Hypothèses!$A$30:$A$33,0))</f>
+        <v>2.1</v>
+      </c>
+      <c r="H21" s="22" t="n">
+        <f aca="false">F21*G21</f>
+        <v>2.94</v>
+      </c>
+      <c r="I21" s="26" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="20" t="s">
+        <v>163</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="C22" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="D22" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="E22" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="F22" s="21" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G22" s="31" t="n">
+        <f aca="false">INDEX(Hypothèses!$B$30:$B$33,MATCH(E22,Hypothèses!$A$30:$A$33,0))</f>
+        <v>2.1</v>
+      </c>
+      <c r="H22" s="22" t="n">
+        <f aca="false">F22*G22</f>
+        <v>2.94</v>
+      </c>
+      <c r="I22" s="26" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="20" t="s">
+        <v>166</v>
+      </c>
+      <c r="B23" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="C23" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="D23" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="E23" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="F23" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="G23" s="31" t="n">
+        <f aca="false">INDEX(Hypothèses!$B$30:$B$33,MATCH(E23,Hypothèses!$A$30:$A$33,0))</f>
+        <v>2.8</v>
+      </c>
+      <c r="H23" s="22" t="n">
+        <f aca="false">F23*G23</f>
+        <v>5.6</v>
+      </c>
+      <c r="I23" s="26" t="s">
+        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -4970,76 +5131,76 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
+        <v>120</v>
+      </c>
+      <c r="B4" s="19" t="s">
+        <v>118</v>
+      </c>
+      <c r="C4" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="B4" s="19" t="s">
-        <v>117</v>
-      </c>
-      <c r="C4" s="19" t="s">
-        <v>118</v>
-      </c>
       <c r="D4" s="19" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>162</v>
+        <v>171</v>
       </c>
       <c r="F4" s="19" t="s">
         <v>52</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>163</v>
+        <v>172</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="I4" s="19" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="J4" s="19" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="K4" s="19" t="s">
         <v>47</v>
       </c>
       <c r="L4" s="19" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="M4" s="19" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="N4" s="19" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="O4" s="19" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="P4" s="19" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="20" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>172</v>
+        <v>181</v>
       </c>
       <c r="E5" s="21" t="n">
         <v>24.44</v>
@@ -5053,11 +5214,11 @@
         <v>146.64</v>
       </c>
       <c r="H5" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A5,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A5,Portes!$H$5:$H$23)</f>
         <v>0</v>
       </c>
       <c r="I5" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B5,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C5,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B5,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C5,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J5" s="22" t="n">
@@ -5065,7 +5226,7 @@
         <v>146.64</v>
       </c>
       <c r="K5" s="18" t="n">
-        <f aca="false">IF(I5="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B5,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C5,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I5="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B5,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C5,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>60</v>
       </c>
       <c r="L5" s="32" t="n">
@@ -5073,11 +5234,11 @@
         <v>0.366666666666667</v>
       </c>
       <c r="M5" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B5,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B5,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="N5" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C5,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C5,Hypothèses!$A$38:$A$53,0))</f>
         <v>40</v>
       </c>
       <c r="O5" s="24" t="n">
@@ -5091,16 +5252,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="E6" s="21" t="n">
         <v>11.83</v>
@@ -5114,11 +5275,11 @@
         <v>70.98</v>
       </c>
       <c r="H6" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A6,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A6,Portes!$H$5:$H$23)</f>
         <v>3.15</v>
       </c>
       <c r="I6" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B6,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C6,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B6,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C6,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J6" s="22" t="n">
@@ -5126,7 +5287,7 @@
         <v>67.83</v>
       </c>
       <c r="K6" s="18" t="n">
-        <f aca="false">IF(I6="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B6,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C6,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I6="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B6,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C6,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>60</v>
       </c>
       <c r="L6" s="32" t="n">
@@ -5134,11 +5295,11 @@
         <v>0.366666666666667</v>
       </c>
       <c r="M6" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B6,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B6,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="N6" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C6,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C6,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="O6" s="24" t="n">
@@ -5152,16 +5313,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
       <c r="E7" s="21" t="n">
         <v>11.83</v>
@@ -5175,11 +5336,11 @@
         <v>70.98</v>
       </c>
       <c r="H7" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A7,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A7,Portes!$H$5:$H$23)</f>
         <v>0</v>
       </c>
       <c r="I7" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B7,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C7,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B7,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C7,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J7" s="22" t="n">
@@ -5187,7 +5348,7 @@
         <v>70.98</v>
       </c>
       <c r="K7" s="18" t="n">
-        <f aca="false">IF(I7="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B7,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C7,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I7="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B7,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C7,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>60</v>
       </c>
       <c r="L7" s="32" t="n">
@@ -5195,11 +5356,11 @@
         <v>0.366666666666667</v>
       </c>
       <c r="M7" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B7,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B7,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="N7" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C7,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C7,Hypothèses!$A$38:$A$53,0))</f>
         <v>40</v>
       </c>
       <c r="O7" s="24" t="n">
@@ -5213,16 +5374,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="E8" s="21" t="n">
         <v>7.26</v>
@@ -5236,11 +5397,11 @@
         <v>43.56</v>
       </c>
       <c r="H8" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A8,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A8,Portes!$H$5:$H$23)</f>
         <v>0</v>
       </c>
       <c r="I8" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B8,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C8,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B8,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C8,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J8" s="22" t="n">
@@ -5248,7 +5409,7 @@
         <v>43.56</v>
       </c>
       <c r="K8" s="18" t="n">
-        <f aca="false">IF(I8="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B8,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C8,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I8="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B8,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C8,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>60</v>
       </c>
       <c r="L8" s="32" t="n">
@@ -5256,11 +5417,11 @@
         <v>0.366666666666667</v>
       </c>
       <c r="M8" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B8,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B8,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="N8" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C8,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C8,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="O8" s="24" t="n">
@@ -5274,16 +5435,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
       <c r="E9" s="21" t="n">
         <v>17.08</v>
@@ -5297,11 +5458,11 @@
         <v>102.48</v>
       </c>
       <c r="H9" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A9,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A9,Portes!$H$5:$H$23)</f>
         <v>2.94</v>
       </c>
       <c r="I9" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B9,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C9,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B9,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C9,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J9" s="22" t="n">
@@ -5309,7 +5470,7 @@
         <v>99.54</v>
       </c>
       <c r="K9" s="18" t="n">
-        <f aca="false">IF(I9="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B9,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C9,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I9="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B9,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C9,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>60</v>
       </c>
       <c r="L9" s="32" t="n">
@@ -5317,11 +5478,11 @@
         <v>0.366666666666667</v>
       </c>
       <c r="M9" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B9,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B9,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="N9" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C9,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C9,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="O9" s="24" t="n">
@@ -5335,16 +5496,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="E10" s="21" t="n">
         <v>8.5</v>
@@ -5358,11 +5519,11 @@
         <v>51</v>
       </c>
       <c r="H10" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A10,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A10,Portes!$H$5:$H$23)</f>
         <v>0</v>
       </c>
       <c r="I10" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B10,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C10,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B10,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C10,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J10" s="22" t="n">
@@ -5370,7 +5531,7 @@
         <v>51</v>
       </c>
       <c r="K10" s="18" t="n">
-        <f aca="false">IF(I10="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B10,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C10,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I10="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B10,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C10,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>60</v>
       </c>
       <c r="L10" s="32" t="n">
@@ -5378,11 +5539,11 @@
         <v>0.366666666666667</v>
       </c>
       <c r="M10" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B10,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B10,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="N10" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C10,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C10,Hypothèses!$A$38:$A$53,0))</f>
         <v>40</v>
       </c>
       <c r="O10" s="24" t="n">
@@ -5396,16 +5557,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="E11" s="21" t="n">
         <v>17.08</v>
@@ -5419,11 +5580,11 @@
         <v>102.48</v>
       </c>
       <c r="H11" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A11,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A11,Portes!$H$5:$H$23)</f>
         <v>2.94</v>
       </c>
       <c r="I11" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B11,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C11,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B11,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C11,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J11" s="22" t="n">
@@ -5431,7 +5592,7 @@
         <v>99.54</v>
       </c>
       <c r="K11" s="18" t="n">
-        <f aca="false">IF(I11="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B11,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C11,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I11="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B11,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C11,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>60</v>
       </c>
       <c r="L11" s="32" t="n">
@@ -5439,11 +5600,11 @@
         <v>0.366666666666667</v>
       </c>
       <c r="M11" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B11,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B11,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="N11" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C11,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C11,Hypothèses!$A$38:$A$53,0))</f>
         <v>35</v>
       </c>
       <c r="O11" s="24" t="n">
@@ -5457,16 +5618,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="E12" s="21" t="n">
         <v>8.5</v>
@@ -5480,11 +5641,11 @@
         <v>51</v>
       </c>
       <c r="H12" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A12,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A12,Portes!$H$5:$H$23)</f>
         <v>0</v>
       </c>
       <c r="I12" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B12,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C12,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B12,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C12,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J12" s="22" t="n">
@@ -5492,7 +5653,7 @@
         <v>51</v>
       </c>
       <c r="K12" s="18" t="n">
-        <f aca="false">IF(I12="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B12,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C12,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I12="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B12,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C12,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>60</v>
       </c>
       <c r="L12" s="32" t="n">
@@ -5500,11 +5661,11 @@
         <v>0.366666666666667</v>
       </c>
       <c r="M12" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B12,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B12,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="N12" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C12,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C12,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="O12" s="24" t="n">
@@ -5518,16 +5679,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>185</v>
+        <v>194</v>
       </c>
       <c r="E13" s="21" t="n">
         <v>12.5</v>
@@ -5541,11 +5702,11 @@
         <v>75</v>
       </c>
       <c r="H13" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A13,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A13,Portes!$H$5:$H$23)</f>
         <v>0</v>
       </c>
       <c r="I13" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B13,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C13,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B13,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C13,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J13" s="22" t="n">
@@ -5553,7 +5714,7 @@
         <v>75</v>
       </c>
       <c r="K13" s="18" t="n">
-        <f aca="false">IF(I13="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B13,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C13,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I13="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B13,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C13,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>60</v>
       </c>
       <c r="L13" s="32" t="n">
@@ -5561,11 +5722,11 @@
         <v>0.366666666666667</v>
       </c>
       <c r="M13" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B13,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B13,Hypothèses!$A$38:$A$53,0))</f>
         <v>35</v>
       </c>
       <c r="N13" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C13,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C13,Hypothèses!$A$38:$A$53,0))</f>
         <v>40</v>
       </c>
       <c r="O13" s="24" t="n">
@@ -5579,16 +5740,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="E14" s="21" t="n">
         <v>12.5</v>
@@ -5602,11 +5763,11 @@
         <v>75</v>
       </c>
       <c r="H14" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A14,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A14,Portes!$H$5:$H$23)</f>
         <v>0</v>
       </c>
       <c r="I14" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B14,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C14,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B14,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C14,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J14" s="22" t="n">
@@ -5614,7 +5775,7 @@
         <v>75</v>
       </c>
       <c r="K14" s="18" t="n">
-        <f aca="false">IF(I14="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B14,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C14,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I14="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B14,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C14,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>60</v>
       </c>
       <c r="L14" s="32" t="n">
@@ -5622,11 +5783,11 @@
         <v>0.366666666666667</v>
       </c>
       <c r="M14" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B14,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B14,Hypothèses!$A$38:$A$53,0))</f>
         <v>35</v>
       </c>
       <c r="N14" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C14,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C14,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="O14" s="24" t="n">
@@ -5640,16 +5801,16 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="s">
-        <v>188</v>
+        <v>197</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
       <c r="E15" s="21" t="n">
         <v>9.985</v>
@@ -5663,11 +5824,11 @@
         <v>59.91</v>
       </c>
       <c r="H15" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A15,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A15,Portes!$H$5:$H$23)</f>
         <v>0</v>
       </c>
       <c r="I15" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B15,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C15,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B15,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C15,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J15" s="22" t="n">
@@ -5675,7 +5836,7 @@
         <v>59.91</v>
       </c>
       <c r="K15" s="18" t="n">
-        <f aca="false">IF(I15="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B15,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C15,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I15="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B15,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C15,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>60</v>
       </c>
       <c r="L15" s="32" t="n">
@@ -5683,11 +5844,11 @@
         <v>0.366666666666667</v>
       </c>
       <c r="M15" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B15,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B15,Hypothèses!$A$38:$A$53,0))</f>
         <v>35</v>
       </c>
       <c r="N15" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C15,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C15,Hypothèses!$A$38:$A$53,0))</f>
         <v>35</v>
       </c>
       <c r="O15" s="24" t="n">
@@ -5701,19 +5862,19 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="20" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>190</v>
+        <v>199</v>
       </c>
       <c r="E16" s="21" t="n">
-        <v>20.2</v>
+        <v>19.8</v>
       </c>
       <c r="F16" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B16,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C16,Zones!$A$5:$A$14,0)),0))</f>
@@ -5721,22 +5882,22 @@
       </c>
       <c r="G16" s="22" t="n">
         <f aca="false">E16*F16</f>
-        <v>121.2</v>
+        <v>118.8</v>
       </c>
       <c r="H16" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A16,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A16,Portes!$H$5:$H$23)</f>
         <v>2.94</v>
       </c>
       <c r="I16" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B16,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C16,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B16,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C16,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J16" s="22" t="n">
         <f aca="false">MAX(0,G16-H16)</f>
-        <v>118.26</v>
+        <v>115.86</v>
       </c>
       <c r="K16" s="18" t="n">
-        <f aca="false">IF(I16="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B16,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C16,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I16="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B16,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C16,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>60</v>
       </c>
       <c r="L16" s="32" t="n">
@@ -5744,11 +5905,11 @@
         <v>0.366666666666667</v>
       </c>
       <c r="M16" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B16,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B16,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="N16" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C16,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C16,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="O16" s="24" t="n">
@@ -5762,19 +5923,19 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="E17" s="21" t="n">
-        <v>20.2</v>
+        <v>19.8</v>
       </c>
       <c r="F17" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B17,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C17,Zones!$A$5:$A$14,0)),0))</f>
@@ -5782,22 +5943,22 @@
       </c>
       <c r="G17" s="22" t="n">
         <f aca="false">E17*F17</f>
-        <v>121.2</v>
+        <v>118.8</v>
       </c>
       <c r="H17" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A17,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A17,Portes!$H$5:$H$23)</f>
         <v>2.94</v>
       </c>
       <c r="I17" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B17,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C17,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B17,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C17,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J17" s="22" t="n">
         <f aca="false">MAX(0,G17-H17)</f>
-        <v>118.26</v>
+        <v>115.86</v>
       </c>
       <c r="K17" s="18" t="n">
-        <f aca="false">IF(I17="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B17,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C17,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I17="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B17,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C17,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>60</v>
       </c>
       <c r="L17" s="32" t="n">
@@ -5805,16 +5966,16 @@
         <v>0.366666666666667</v>
       </c>
       <c r="M17" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B17,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B17,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="N17" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C17,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C17,Hypothèses!$A$38:$A$53,0))</f>
         <v>35</v>
       </c>
       <c r="O17" s="24" t="n">
         <f aca="false">L17*J17*MAX(0,N17-M17)</f>
-        <v>216.81</v>
+        <v>212.41</v>
       </c>
       <c r="P17" s="24" t="n">
         <f aca="false">L17*J17*MAX(0,M17-N17)</f>
@@ -5823,19 +5984,19 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="20" t="s">
-        <v>192</v>
+        <v>201</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="E18" s="21" t="n">
-        <v>20.2</v>
+        <v>19.8</v>
       </c>
       <c r="F18" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B18,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C18,Zones!$A$5:$A$14,0)),0))</f>
@@ -5843,22 +6004,22 @@
       </c>
       <c r="G18" s="22" t="n">
         <f aca="false">E18*F18</f>
-        <v>121.2</v>
+        <v>118.8</v>
       </c>
       <c r="H18" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A18,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A18,Portes!$H$5:$H$23)</f>
         <v>0</v>
       </c>
       <c r="I18" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B18,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C18,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B18,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C18,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J18" s="22" t="n">
         <f aca="false">MAX(0,G18-H18)</f>
-        <v>121.2</v>
+        <v>118.8</v>
       </c>
       <c r="K18" s="18" t="n">
-        <f aca="false">IF(I18="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B18,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C18,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I18="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B18,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C18,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>60</v>
       </c>
       <c r="L18" s="32" t="n">
@@ -5866,16 +6027,16 @@
         <v>0.366666666666667</v>
       </c>
       <c r="M18" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B18,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B18,Hypothèses!$A$38:$A$53,0))</f>
         <v>35</v>
       </c>
       <c r="N18" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C18,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C18,Hypothèses!$A$38:$A$53,0))</f>
         <v>40</v>
       </c>
       <c r="O18" s="24" t="n">
         <f aca="false">L18*J18*MAX(0,N18-M18)</f>
-        <v>222.2</v>
+        <v>217.8</v>
       </c>
       <c r="P18" s="24" t="n">
         <f aca="false">L18*J18*MAX(0,M18-N18)</f>
@@ -5884,16 +6045,16 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="20" t="s">
-        <v>194</v>
+        <v>164</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="E19" s="21" t="n">
         <v>6.995</v>
@@ -5907,19 +6068,19 @@
         <v>41.97</v>
       </c>
       <c r="H19" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A19,Portes!$H$5:$H$20)</f>
-        <v>0</v>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A19,Portes!$H$5:$H$23)</f>
+        <v>2.94</v>
       </c>
       <c r="I19" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B19,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C19,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B19,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C19,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J19" s="22" t="n">
         <f aca="false">MAX(0,G19-H19)</f>
-        <v>41.97</v>
+        <v>39.03</v>
       </c>
       <c r="K19" s="18" t="n">
-        <f aca="false">IF(I19="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B19,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C19,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I19="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B19,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C19,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>80</v>
       </c>
       <c r="L19" s="32" t="n">
@@ -5927,11 +6088,11 @@
         <v>0.275</v>
       </c>
       <c r="M19" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B19,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B19,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="N19" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C19,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C19,Hypothèses!$A$38:$A$53,0))</f>
         <v>10</v>
       </c>
       <c r="O19" s="24" t="n">
@@ -5940,21 +6101,21 @@
       </c>
       <c r="P19" s="24" t="n">
         <f aca="false">L19*J19*MAX(0,M19-N19)</f>
-        <v>230.835</v>
+        <v>214.665</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="E20" s="21" t="n">
         <v>5.165</v>
@@ -5968,11 +6129,11 @@
         <v>30.99</v>
       </c>
       <c r="H20" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A20,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A20,Portes!$H$5:$H$23)</f>
         <v>0</v>
       </c>
       <c r="I20" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B20,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C20,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B20,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C20,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J20" s="22" t="n">
@@ -5980,7 +6141,7 @@
         <v>30.99</v>
       </c>
       <c r="K20" s="18" t="n">
-        <f aca="false">IF(I20="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B20,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C20,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I20="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B20,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C20,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>80</v>
       </c>
       <c r="L20" s="32" t="n">
@@ -5988,11 +6149,11 @@
         <v>0.275</v>
       </c>
       <c r="M20" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B20,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B20,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="N20" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C20,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C20,Hypothèses!$A$38:$A$53,0))</f>
         <v>10</v>
       </c>
       <c r="O20" s="24" t="n">
@@ -6006,16 +6167,16 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="E21" s="21" t="n">
         <v>9.985</v>
@@ -6029,19 +6190,19 @@
         <v>59.91</v>
       </c>
       <c r="H21" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A21,Portes!$H$5:$H$20)</f>
-        <v>2.94</v>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A21,Portes!$H$5:$H$23)</f>
+        <v>8.54</v>
       </c>
       <c r="I21" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B21,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C21,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B21,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C21,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J21" s="22" t="n">
         <f aca="false">MAX(0,G21-H21)</f>
-        <v>56.97</v>
+        <v>51.37</v>
       </c>
       <c r="K21" s="18" t="n">
-        <f aca="false">IF(I21="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B21,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C21,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I21="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B21,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C21,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>80</v>
       </c>
       <c r="L21" s="32" t="n">
@@ -6049,11 +6210,11 @@
         <v>0.275</v>
       </c>
       <c r="M21" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B21,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B21,Hypothèses!$A$38:$A$53,0))</f>
         <v>35</v>
       </c>
       <c r="N21" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C21,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C21,Hypothèses!$A$38:$A$53,0))</f>
         <v>10</v>
       </c>
       <c r="O21" s="24" t="n">
@@ -6062,24 +6223,24 @@
       </c>
       <c r="P21" s="24" t="n">
         <f aca="false">L21*J21*MAX(0,M21-N21)</f>
-        <v>391.66875</v>
+        <v>353.16875</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="20" t="s">
-        <v>199</v>
+        <v>161</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="E22" s="21" t="n">
-        <v>5.8</v>
+        <v>6.2</v>
       </c>
       <c r="F22" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B22,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C22,Zones!$A$5:$A$14,0)),0))</f>
@@ -6087,22 +6248,22 @@
       </c>
       <c r="G22" s="22" t="n">
         <f aca="false">E22*F22</f>
-        <v>34.8</v>
+        <v>37.2</v>
       </c>
       <c r="H22" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A22,Portes!$H$5:$H$20)</f>
-        <v>0</v>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A22,Portes!$H$5:$H$23)</f>
+        <v>2.94</v>
       </c>
       <c r="I22" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B22,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C22,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B22,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C22,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J22" s="22" t="n">
         <f aca="false">MAX(0,G22-H22)</f>
-        <v>34.8</v>
+        <v>34.26</v>
       </c>
       <c r="K22" s="18" t="n">
-        <f aca="false">IF(I22="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B22,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C22,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I22="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B22,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C22,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>80</v>
       </c>
       <c r="L22" s="32" t="n">
@@ -6110,11 +6271,11 @@
         <v>0.275</v>
       </c>
       <c r="M22" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B22,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B22,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="N22" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C22,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C22,Hypothèses!$A$38:$A$53,0))</f>
         <v>10</v>
       </c>
       <c r="O22" s="24" t="n">
@@ -6123,21 +6284,21 @@
       </c>
       <c r="P22" s="24" t="n">
         <f aca="false">L22*J22*MAX(0,M22-N22)</f>
-        <v>191.4</v>
+        <v>188.43</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="E23" s="21" t="n">
         <v>8.33</v>
@@ -6151,11 +6312,11 @@
         <v>49.98</v>
       </c>
       <c r="H23" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A23,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A23,Portes!$H$5:$H$23)</f>
         <v>0</v>
       </c>
       <c r="I23" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B23,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C23,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B23,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C23,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J23" s="22" t="n">
@@ -6163,7 +6324,7 @@
         <v>49.98</v>
       </c>
       <c r="K23" s="18" t="n">
-        <f aca="false">IF(I23="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B23,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C23,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I23="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B23,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C23,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>80</v>
       </c>
       <c r="L23" s="32" t="n">
@@ -6171,11 +6332,11 @@
         <v>0.275</v>
       </c>
       <c r="M23" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B23,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B23,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="N23" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C23,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C23,Hypothèses!$A$38:$A$53,0))</f>
         <v>10</v>
       </c>
       <c r="O23" s="24" t="n">
@@ -6189,16 +6350,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="E24" s="21" t="n">
         <v>3.93</v>
@@ -6212,11 +6373,11 @@
         <v>23.58</v>
       </c>
       <c r="H24" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A24,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A24,Portes!$H$5:$H$23)</f>
         <v>0</v>
       </c>
       <c r="I24" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B24,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C24,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B24,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C24,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J24" s="22" t="n">
@@ -6224,7 +6385,7 @@
         <v>23.58</v>
       </c>
       <c r="K24" s="18" t="n">
-        <f aca="false">IF(I24="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B24,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C24,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I24="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B24,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C24,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>80</v>
       </c>
       <c r="L24" s="32" t="n">
@@ -6232,11 +6393,11 @@
         <v>0.275</v>
       </c>
       <c r="M24" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B24,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B24,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="N24" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C24,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C24,Hypothèses!$A$38:$A$53,0))</f>
         <v>10</v>
       </c>
       <c r="O24" s="24" t="n">
@@ -6250,16 +6411,16 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="20" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="E25" s="21" t="n">
         <v>2.2</v>
@@ -6273,11 +6434,11 @@
         <v>13.2</v>
       </c>
       <c r="H25" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A25,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A25,Portes!$H$5:$H$23)</f>
         <v>0</v>
       </c>
       <c r="I25" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B25,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C25,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B25,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C25,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J25" s="22" t="n">
@@ -6285,7 +6446,7 @@
         <v>13.2</v>
       </c>
       <c r="K25" s="18" t="n">
-        <f aca="false">IF(I25="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B25,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C25,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I25="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B25,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C25,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>80</v>
       </c>
       <c r="L25" s="32" t="n">
@@ -6293,11 +6454,11 @@
         <v>0.275</v>
       </c>
       <c r="M25" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B25,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B25,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="N25" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C25,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C25,Hypothèses!$A$38:$A$53,0))</f>
         <v>10</v>
       </c>
       <c r="O25" s="24" t="n">
@@ -6311,19 +6472,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="E26" s="21" t="n">
-        <v>8</v>
+        <v>8.4</v>
       </c>
       <c r="F26" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B26,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C26,Zones!$A$5:$A$14,0)),0))</f>
@@ -6331,22 +6492,22 @@
       </c>
       <c r="G26" s="22" t="n">
         <f aca="false">E26*F26</f>
-        <v>48</v>
+        <v>50.4</v>
       </c>
       <c r="H26" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A26,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A26,Portes!$H$5:$H$23)</f>
         <v>0</v>
       </c>
       <c r="I26" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B26,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C26,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B26,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C26,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J26" s="22" t="n">
         <f aca="false">MAX(0,G26-H26)</f>
-        <v>48</v>
+        <v>50.4</v>
       </c>
       <c r="K26" s="18" t="n">
-        <f aca="false">IF(I26="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B26,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C26,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I26="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B26,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C26,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>80</v>
       </c>
       <c r="L26" s="32" t="n">
@@ -6354,16 +6515,16 @@
         <v>0.275</v>
       </c>
       <c r="M26" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B26,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B26,Hypothèses!$A$38:$A$53,0))</f>
         <v>10</v>
       </c>
       <c r="N26" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C26,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C26,Hypothèses!$A$38:$A$53,0))</f>
         <v>40</v>
       </c>
       <c r="O26" s="24" t="n">
         <f aca="false">L26*J26*MAX(0,N26-M26)</f>
-        <v>396</v>
+        <v>415.8</v>
       </c>
       <c r="P26" s="24" t="n">
         <f aca="false">L26*J26*MAX(0,M26-N26)</f>
@@ -6372,16 +6533,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="E27" s="21" t="n">
         <v>9.985</v>
@@ -6395,11 +6556,11 @@
         <v>59.91</v>
       </c>
       <c r="H27" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A27,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A27,Portes!$H$5:$H$23)</f>
         <v>2.94</v>
       </c>
       <c r="I27" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B27,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C27,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B27,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C27,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J27" s="22" t="n">
@@ -6407,7 +6568,7 @@
         <v>56.97</v>
       </c>
       <c r="K27" s="18" t="n">
-        <f aca="false">IF(I27="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B27,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C27,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I27="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B27,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C27,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>80</v>
       </c>
       <c r="L27" s="32" t="n">
@@ -6415,11 +6576,11 @@
         <v>0.275</v>
       </c>
       <c r="M27" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B27,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B27,Hypothèses!$A$38:$A$53,0))</f>
         <v>10</v>
       </c>
       <c r="N27" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C27,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C27,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="O27" s="24" t="n">
@@ -6433,16 +6594,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="20" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="E28" s="21" t="n">
         <v>10.43</v>
@@ -6456,11 +6617,11 @@
         <v>62.58</v>
       </c>
       <c r="H28" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A28,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A28,Portes!$H$5:$H$23)</f>
         <v>0</v>
       </c>
       <c r="I28" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B28,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C28,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B28,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C28,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J28" s="22" t="n">
@@ -6468,7 +6629,7 @@
         <v>62.58</v>
       </c>
       <c r="K28" s="18" t="n">
-        <f aca="false">IF(I28="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B28,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C28,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I28="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B28,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C28,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>60</v>
       </c>
       <c r="L28" s="32" t="n">
@@ -6476,11 +6637,11 @@
         <v>0.366666666666667</v>
       </c>
       <c r="M28" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B28,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B28,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="N28" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C28,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C28,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="O28" s="24" t="n">
@@ -6494,16 +6655,16 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="20" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="E29" s="21" t="n">
         <v>3.93</v>
@@ -6517,11 +6678,11 @@
         <v>23.58</v>
       </c>
       <c r="H29" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A29,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A29,Portes!$H$5:$H$23)</f>
         <v>0</v>
       </c>
       <c r="I29" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B29,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C29,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B29,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C29,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J29" s="22" t="n">
@@ -6529,7 +6690,7 @@
         <v>23.58</v>
       </c>
       <c r="K29" s="18" t="n">
-        <f aca="false">IF(I29="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B29,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C29,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I29="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B29,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C29,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>60</v>
       </c>
       <c r="L29" s="32" t="n">
@@ -6537,11 +6698,11 @@
         <v>0.366666666666667</v>
       </c>
       <c r="M29" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B29,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B29,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="N29" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C29,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C29,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="O29" s="24" t="n">
@@ -6555,16 +6716,16 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="20" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="E30" s="21" t="n">
         <v>2.8</v>
@@ -6578,11 +6739,11 @@
         <v>16.8</v>
       </c>
       <c r="H30" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A30,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A30,Portes!$H$5:$H$23)</f>
         <v>0</v>
       </c>
       <c r="I30" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B30,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C30,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B30,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C30,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J30" s="22" t="n">
@@ -6590,7 +6751,7 @@
         <v>16.8</v>
       </c>
       <c r="K30" s="18" t="n">
-        <f aca="false">IF(I30="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B30,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C30,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I30="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B30,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C30,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>60</v>
       </c>
       <c r="L30" s="32" t="n">
@@ -6598,11 +6759,11 @@
         <v>0.366666666666667</v>
       </c>
       <c r="M30" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B30,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B30,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="N30" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C30,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C30,Hypothèses!$A$38:$A$53,0))</f>
         <v>40</v>
       </c>
       <c r="O30" s="24" t="n">
@@ -6616,16 +6777,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="20" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="E31" s="21" t="n">
         <v>2.8</v>
@@ -6639,11 +6800,11 @@
         <v>16.8</v>
       </c>
       <c r="H31" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A31,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A31,Portes!$H$5:$H$23)</f>
         <v>0</v>
       </c>
       <c r="I31" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B31,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C31,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B31,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C31,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J31" s="22" t="n">
@@ -6651,7 +6812,7 @@
         <v>16.8</v>
       </c>
       <c r="K31" s="18" t="n">
-        <f aca="false">IF(I31="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B31,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C31,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I31="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B31,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C31,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>60</v>
       </c>
       <c r="L31" s="32" t="n">
@@ -6659,11 +6820,11 @@
         <v>0.366666666666667</v>
       </c>
       <c r="M31" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B31,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B31,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="N31" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C31,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C31,Hypothèses!$A$38:$A$53,0))</f>
         <v>40</v>
       </c>
       <c r="O31" s="24" t="n">
@@ -6677,16 +6838,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="20" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="E32" s="21" t="n">
         <v>2.8</v>
@@ -6700,11 +6861,11 @@
         <v>16.8</v>
       </c>
       <c r="H32" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A32,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A32,Portes!$H$5:$H$23)</f>
         <v>2.94</v>
       </c>
       <c r="I32" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B32,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C32,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B32,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C32,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J32" s="22" t="n">
@@ -6712,7 +6873,7 @@
         <v>13.86</v>
       </c>
       <c r="K32" s="18" t="n">
-        <f aca="false">IF(I32="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B32,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C32,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I32="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B32,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C32,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>60</v>
       </c>
       <c r="L32" s="32" t="n">
@@ -6720,11 +6881,11 @@
         <v>0.366666666666667</v>
       </c>
       <c r="M32" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B32,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B32,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="N32" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C32,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C32,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="O32" s="24" t="n">
@@ -6738,16 +6899,16 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="20" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="E33" s="21" t="n">
         <v>19.34</v>
@@ -6761,11 +6922,11 @@
         <v>116.04</v>
       </c>
       <c r="H33" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A33,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A33,Portes!$H$5:$H$23)</f>
         <v>5.88</v>
       </c>
       <c r="I33" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B33,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C33,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B33,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C33,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J33" s="22" t="n">
@@ -6773,7 +6934,7 @@
         <v>110.16</v>
       </c>
       <c r="K33" s="18" t="n">
-        <f aca="false">IF(I33="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B33,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C33,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I33="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B33,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C33,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>150</v>
       </c>
       <c r="L33" s="32" t="n">
@@ -6781,11 +6942,11 @@
         <v>0.146666666666667</v>
       </c>
       <c r="M33" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B33,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B33,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="N33" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C33,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C33,Hypothèses!$A$38:$A$53,0))</f>
         <v>-20</v>
       </c>
       <c r="O33" s="24" t="n">
@@ -6799,16 +6960,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="20" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B34" s="14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="E34" s="21" t="n">
         <v>5</v>
@@ -6822,11 +6983,11 @@
         <v>30</v>
       </c>
       <c r="H34" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A34,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A34,Portes!$H$5:$H$23)</f>
         <v>2.94</v>
       </c>
       <c r="I34" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B34,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C34,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B34,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C34,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J34" s="22" t="n">
@@ -6834,7 +6995,7 @@
         <v>27.06</v>
       </c>
       <c r="K34" s="18" t="n">
-        <f aca="false">IF(I34="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B34,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C34,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I34="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B34,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C34,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>100</v>
       </c>
       <c r="L34" s="32" t="n">
@@ -6842,11 +7003,11 @@
         <v>0.22</v>
       </c>
       <c r="M34" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B34,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B34,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="N34" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C34,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C34,Hypothèses!$A$38:$A$53,0))</f>
         <v>2</v>
       </c>
       <c r="O34" s="24" t="n">
@@ -6860,16 +7021,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="20" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="B35" s="14" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="E35" s="21" t="n">
         <v>15.01</v>
@@ -6883,11 +7044,11 @@
         <v>90.06</v>
       </c>
       <c r="H35" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A35,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A35,Portes!$H$5:$H$23)</f>
         <v>0</v>
       </c>
       <c r="I35" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B35,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C35,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B35,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C35,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J35" s="22" t="n">
@@ -6895,7 +7056,7 @@
         <v>90.06</v>
       </c>
       <c r="K35" s="18" t="n">
-        <f aca="false">IF(I35="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B35,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C35,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I35="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B35,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C35,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>150</v>
       </c>
       <c r="L35" s="32" t="n">
@@ -6903,11 +7064,11 @@
         <v>0.146666666666667</v>
       </c>
       <c r="M35" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B35,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B35,Hypothèses!$A$38:$A$53,0))</f>
         <v>-20</v>
       </c>
       <c r="N35" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C35,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C35,Hypothèses!$A$38:$A$53,0))</f>
         <v>2</v>
       </c>
       <c r="O35" s="24" t="n">
@@ -6921,16 +7082,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="20" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B36" s="14" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="E36" s="21" t="n">
         <v>15.01</v>
@@ -6944,11 +7105,11 @@
         <v>90.06</v>
       </c>
       <c r="H36" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A36,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A36,Portes!$H$5:$H$23)</f>
         <v>8.4</v>
       </c>
       <c r="I36" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B36,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C36,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B36,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C36,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J36" s="22" t="n">
@@ -6956,7 +7117,7 @@
         <v>81.66</v>
       </c>
       <c r="K36" s="18" t="n">
-        <f aca="false">IF(I36="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B36,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C36,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I36="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B36,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C36,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>150</v>
       </c>
       <c r="L36" s="32" t="n">
@@ -6964,11 +7125,11 @@
         <v>0.146666666666667</v>
       </c>
       <c r="M36" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B36,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B36,Hypothèses!$A$38:$A$53,0))</f>
         <v>-20</v>
       </c>
       <c r="N36" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C36,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C36,Hypothèses!$A$38:$A$53,0))</f>
         <v>40</v>
       </c>
       <c r="O36" s="24" t="n">
@@ -6982,16 +7143,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="20" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="B37" s="14" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="E37" s="21" t="n">
         <v>19.34</v>
@@ -7005,11 +7166,11 @@
         <v>116.04</v>
       </c>
       <c r="H37" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A37,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A37,Portes!$H$5:$H$23)</f>
         <v>0</v>
       </c>
       <c r="I37" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B37,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C37,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B37,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C37,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J37" s="22" t="n">
@@ -7017,7 +7178,7 @@
         <v>116.04</v>
       </c>
       <c r="K37" s="18" t="n">
-        <f aca="false">IF(I37="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B37,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C37,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I37="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B37,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C37,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>150</v>
       </c>
       <c r="L37" s="32" t="n">
@@ -7025,11 +7186,11 @@
         <v>0.146666666666667</v>
       </c>
       <c r="M37" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B37,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B37,Hypothèses!$A$38:$A$53,0))</f>
         <v>-20</v>
       </c>
       <c r="N37" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C37,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C37,Hypothèses!$A$38:$A$53,0))</f>
         <v>25</v>
       </c>
       <c r="O37" s="24" t="n">
@@ -7043,16 +7204,16 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="20" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="E38" s="21" t="n">
         <v>5</v>
@@ -7066,11 +7227,11 @@
         <v>30</v>
       </c>
       <c r="H38" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A38,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A38,Portes!$H$5:$H$23)</f>
         <v>0</v>
       </c>
       <c r="I38" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B38,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C38,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B38,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C38,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J38" s="22" t="n">
@@ -7078,7 +7239,7 @@
         <v>30</v>
       </c>
       <c r="K38" s="18" t="n">
-        <f aca="false">IF(I38="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B38,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C38,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I38="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B38,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C38,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>100</v>
       </c>
       <c r="L38" s="32" t="n">
@@ -7086,11 +7247,11 @@
         <v>0.22</v>
       </c>
       <c r="M38" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B38,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B38,Hypothèses!$A$38:$A$53,0))</f>
         <v>2</v>
       </c>
       <c r="N38" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C38,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C38,Hypothèses!$A$38:$A$53,0))</f>
         <v>25</v>
       </c>
       <c r="O38" s="24" t="n">
@@ -7104,16 +7265,16 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="20" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D39" s="14" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="E39" s="21" t="n">
         <v>15.01</v>
@@ -7127,11 +7288,11 @@
         <v>90.06</v>
       </c>
       <c r="H39" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A39,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A39,Portes!$H$5:$H$23)</f>
         <v>0</v>
       </c>
       <c r="I39" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B39,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C39,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B39,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C39,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Oui</v>
       </c>
       <c r="J39" s="22" t="n">
@@ -7139,7 +7300,7 @@
         <v>90.06</v>
       </c>
       <c r="K39" s="18" t="n">
-        <f aca="false">IF(I39="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B39,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C39,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I39="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B39,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C39,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>100</v>
       </c>
       <c r="L39" s="32" t="n">
@@ -7147,11 +7308,11 @@
         <v>0.22</v>
       </c>
       <c r="M39" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B39,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B39,Hypothèses!$A$38:$A$53,0))</f>
         <v>2</v>
       </c>
       <c r="N39" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C39,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C39,Hypothèses!$A$38:$A$53,0))</f>
         <v>40</v>
       </c>
       <c r="O39" s="24" t="n">
@@ -7165,16 +7326,16 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="20" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B40" s="14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D40" s="14" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="E40" s="21" t="n">
         <v>49.5</v>
@@ -7188,11 +7349,11 @@
         <v>297</v>
       </c>
       <c r="H40" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A40,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A40,Portes!$H$5:$H$23)</f>
         <v>5.88</v>
       </c>
       <c r="I40" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B40,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C40,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B40,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C40,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Non</v>
       </c>
       <c r="J40" s="22" t="n">
@@ -7200,7 +7361,7 @@
         <v>291.12</v>
       </c>
       <c r="K40" s="18" t="n">
-        <f aca="false">IF(I40="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B40,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C40,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I40="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B40,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C40,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>0</v>
       </c>
       <c r="L40" s="32" t="n">
@@ -7208,11 +7369,11 @@
         <v>0</v>
       </c>
       <c r="M40" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B40,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B40,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="N40" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C40,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C40,Hypothèses!$A$38:$A$53,0))</f>
         <v>40</v>
       </c>
       <c r="O40" s="24" t="n">
@@ -7226,16 +7387,16 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="20" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B41" s="14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D41" s="14" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="E41" s="21" t="n">
         <v>17.6</v>
@@ -7249,11 +7410,11 @@
         <v>105.6</v>
       </c>
       <c r="H41" s="22" t="n">
-        <f aca="false">SUMIF(Portes!$D$5:$D$20,A41,Portes!$H$5:$H$20)</f>
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A41,Portes!$H$5:$H$23)</f>
         <v>5.88</v>
       </c>
       <c r="I41" s="14" t="str">
-        <f aca="false">IF(OR(INDEX(Hypothèses!$D$37:$D$52,MATCH(B41,Hypothèses!$A$37:$A$52,0))="Oui",INDEX(Hypothèses!$D$37:$D$52,MATCH(C41,Hypothèses!$A$37:$A$52,0))="Oui"),"Oui","Non")</f>
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B41,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C41,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
         <v>Non</v>
       </c>
       <c r="J41" s="22" t="n">
@@ -7261,7 +7422,7 @@
         <v>99.72</v>
       </c>
       <c r="K41" s="18" t="n">
-        <f aca="false">IF(I41="Oui",MAX(INDEX(Hypothèses!$C$37:$C$52,MATCH(B41,Hypothèses!$A$37:$A$52,0)),INDEX(Hypothèses!$C$37:$C$52,MATCH(C41,Hypothèses!$A$37:$A$52,0))),0)</f>
+        <f aca="false">IF(I41="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B41,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C41,Hypothèses!$A$38:$A$53,0))),0)</f>
         <v>0</v>
       </c>
       <c r="L41" s="32" t="n">
@@ -7269,11 +7430,11 @@
         <v>0</v>
       </c>
       <c r="M41" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(B41,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B41,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="N41" s="18" t="n">
-        <f aca="false">INDEX(Hypothèses!$B$37:$B$52,MATCH(C41,Hypothèses!$A$37:$A$52,0))</f>
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C41,Hypothèses!$A$38:$A$53,0))</f>
         <v>30</v>
       </c>
       <c r="O41" s="24" t="n">
@@ -7287,28 +7448,28 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D42" s="28" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E42" s="29" t="n">
         <f aca="false">SUM(E5:E41)</f>
-        <v>446.065</v>
+        <v>445.665</v>
       </c>
       <c r="G42" s="29" t="n">
         <f aca="false">SUM(G5:G41)</f>
-        <v>2676.39</v>
+        <v>2673.99</v>
       </c>
       <c r="H42" s="29" t="n">
         <f aca="false">SUM(H5:H41)</f>
-        <v>52.71</v>
+        <v>64.19</v>
       </c>
       <c r="J42" s="29" t="n">
         <f aca="false">SUM(J5:J41)</f>
-        <v>2623.68</v>
+        <v>2609.8</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D44" s="33" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
     </row>
   </sheetData>
@@ -7328,7 +7489,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -7341,12 +7502,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7354,22 +7515,22 @@
         <v>47</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="F4" s="19" t="s">
         <v>48</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7439,19 +7600,19 @@
       </c>
       <c r="B7" s="22" t="n">
         <f aca="false">SUMIFS(Parois!$J$5:$J$41,Parois!$K$5:$K$41,A7,Parois!$I$5:$I$41,"Oui")</f>
-        <v>356.46</v>
+        <v>349.78</v>
       </c>
       <c r="C7" s="22" t="n">
         <f aca="false">SUMIF(Zones!$L$5:$L$14,A7,Zones!$N$5:$N$14)</f>
-        <v>151.57</v>
+        <v>160.51</v>
       </c>
       <c r="D7" s="22" t="n">
         <f aca="false">B7+C7</f>
-        <v>508.03</v>
+        <v>510.29</v>
       </c>
       <c r="E7" s="22" t="n">
         <f aca="false">D7*(1+Hypothèses!$B$9)</f>
-        <v>533.4315</v>
+        <v>535.8045</v>
       </c>
       <c r="F7" s="34" t="n">
         <f aca="false">Hypothèses!C24</f>
@@ -7459,7 +7620,7 @@
       </c>
       <c r="G7" s="24" t="n">
         <f aca="false">E7*F7</f>
-        <v>154695.135</v>
+        <v>155383.305</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7469,19 +7630,19 @@
       </c>
       <c r="B8" s="22" t="n">
         <f aca="false">SUMIFS(Parois!$J$5:$J$41,Parois!$K$5:$K$41,A8,Parois!$I$5:$I$41,"Oui")</f>
-        <v>1331.34</v>
+        <v>1324.14</v>
       </c>
       <c r="C8" s="22" t="n">
         <f aca="false">SUMIF(Zones!$L$5:$L$14,A8,Zones!$N$5:$N$14)</f>
-        <v>1059.2332</v>
+        <v>1052.4412</v>
       </c>
       <c r="D8" s="22" t="n">
         <f aca="false">B8+C8</f>
-        <v>2390.5732</v>
+        <v>2376.5812</v>
       </c>
       <c r="E8" s="22" t="n">
         <f aca="false">D8*(1+Hypothèses!$B$9)</f>
-        <v>2510.10186</v>
+        <v>2495.41026</v>
       </c>
       <c r="F8" s="34" t="n">
         <f aca="false">Hypothèses!C25</f>
@@ -7489,55 +7650,55 @@
       </c>
       <c r="G8" s="24" t="n">
         <f aca="false">E8*F8</f>
-        <v>627525.465</v>
+        <v>623852.565</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="28" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B9" s="29" t="n">
         <f aca="false">SUM(B5:B8)</f>
-        <v>2232.84</v>
+        <v>2218.96</v>
       </c>
       <c r="C9" s="29" t="n">
         <f aca="false">SUM(C5:C8)</f>
-        <v>1576.1466</v>
+        <v>1578.2946</v>
       </c>
       <c r="D9" s="29" t="n">
         <f aca="false">SUM(D5:D8)</f>
-        <v>3808.9866</v>
+        <v>3797.2546</v>
       </c>
       <c r="E9" s="29" t="n">
         <f aca="false">SUM(E5:E8)</f>
-        <v>3999.43593</v>
+        <v>3987.11733</v>
       </c>
       <c r="G9" s="30" t="n">
         <f aca="false">SUM(G5:G8)</f>
-        <v>1162704.6144</v>
+        <v>1159719.8844</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
       <c r="G10" s="24" t="n">
         <f aca="false">G9*Hypothèses!$B$10</f>
-        <v>174405.69216</v>
+        <v>173957.98266</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="19" t="s">
-        <v>241</v>
+        <v>248</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="C12" s="19" t="s">
         <v>53</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7546,8 +7707,8 @@
         <v>Porte double</v>
       </c>
       <c r="B13" s="18" t="n">
-        <f aca="false">COUNTIF(Portes!$E$5:$E$20,A13)</f>
-        <v>14</v>
+        <f aca="false">COUNTIF(Portes!$E$5:$E$23,A13)</f>
+        <v>16</v>
       </c>
       <c r="C13" s="34" t="n">
         <f aca="false">Hypothèses!C30</f>
@@ -7555,7 +7716,7 @@
       </c>
       <c r="D13" s="24" t="n">
         <f aca="false">B13*C13</f>
-        <v>252000</v>
+        <v>288000</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7564,7 +7725,7 @@
         <v>Porte simple</v>
       </c>
       <c r="B14" s="18" t="n">
-        <f aca="false">COUNTIF(Portes!$E$5:$E$20,A14)</f>
+        <f aca="false">COUNTIF(Portes!$E$5:$E$23,A14)</f>
         <v>1</v>
       </c>
       <c r="C14" s="34" t="n">
@@ -7582,7 +7743,7 @@
         <v>Porte sectionnelle (quai)</v>
       </c>
       <c r="B15" s="18" t="n">
-        <f aca="false">COUNTIF(Portes!$E$5:$E$20,A15)</f>
+        <f aca="false">COUNTIF(Portes!$E$5:$E$23,A15)</f>
         <v>1</v>
       </c>
       <c r="C15" s="34" t="n">
@@ -7595,31 +7756,49 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="28" t="s">
-        <v>244</v>
-      </c>
-      <c r="D16" s="30" t="n">
-        <f aca="false">SUM(D13:D15)</f>
-        <v>306000</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="28" t="s">
-        <v>245</v>
-      </c>
-      <c r="B18" s="28"/>
-      <c r="C18" s="28"/>
-      <c r="D18" s="28"/>
-      <c r="E18" s="28"/>
-      <c r="F18" s="28"/>
-      <c r="G18" s="30" t="n">
-        <f aca="false">G9+G10+D16</f>
-        <v>1643110.30656</v>
+      <c r="A16" s="16" t="str">
+        <f aca="false">Hypothèses!A33</f>
+        <v>Passage tunnel</v>
+      </c>
+      <c r="B16" s="18" t="n">
+        <f aca="false">COUNTIF(Portes!$E$5:$E$23,A16)</f>
+        <v>1</v>
+      </c>
+      <c r="C16" s="34" t="n">
+        <f aca="false">Hypothèses!C33</f>
+        <v>0</v>
+      </c>
+      <c r="D16" s="24" t="n">
+        <f aca="false">B16*C16</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="28" t="s">
+        <v>251</v>
+      </c>
+      <c r="D17" s="30" t="n">
+        <f aca="false">SUM(D13:D16)</f>
+        <v>342000</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="28" t="s">
+        <v>252</v>
+      </c>
+      <c r="B19" s="28"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="28"/>
+      <c r="F19" s="28"/>
+      <c r="G19" s="30" t="n">
+        <f aca="false">G9+G10+D17</f>
+        <v>1675677.86706</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A19:F19"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -7647,101 +7826,101 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>249</v>
+        <v>256</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>250</v>
+        <v>257</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="I4" s="19" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
       <c r="J4" s="19" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="K4" s="19" t="s">
-        <v>254</v>
+        <v>261</v>
       </c>
       <c r="L4" s="19" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
       <c r="M4" s="19" t="s">
-        <v>256</v>
+        <v>263</v>
       </c>
       <c r="N4" s="19" t="s">
-        <v>257</v>
+        <v>264</v>
       </c>
       <c r="O4" s="19" t="s">
-        <v>258</v>
+        <v>265</v>
       </c>
       <c r="P4" s="19" t="s">
-        <v>259</v>
+        <v>266</v>
       </c>
       <c r="Q4" s="19" t="s">
-        <v>260</v>
+        <v>267</v>
       </c>
       <c r="R4" s="19" t="s">
-        <v>261</v>
+        <v>268</v>
       </c>
       <c r="S4" s="19" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
       <c r="T4" s="19" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="U4" s="19" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="V4" s="19" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="W4" s="19" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="X4" s="19" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="Y4" s="19" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="Z4" s="19" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="AA4" s="19" t="s">
-        <v>270</v>
+        <v>277</v>
       </c>
       <c r="AB4" s="19" t="s">
-        <v>271</v>
+        <v>278</v>
       </c>
       <c r="AC4" s="19" t="s">
-        <v>272</v>
+        <v>279</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8075,19 +8254,19 @@
       </c>
       <c r="E8" s="35" t="n">
         <f aca="false">Zones!E8</f>
-        <v>141.299</v>
+        <v>138.501</v>
       </c>
       <c r="F8" s="34" t="n">
         <f aca="false">Zones!H8</f>
-        <v>847.794</v>
+        <v>831.006</v>
       </c>
       <c r="G8" s="24" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A8,Parois!$O$5:$O$41)+SUMIF(Parois!$C$5:$C$41,A8,Parois!$P$5:$P$41)</f>
-        <v>216.81</v>
+        <v>212.41</v>
       </c>
       <c r="H8" s="24" t="n">
         <f aca="false">IF(Zones!L8&gt;0,Hypothèses!$B$4/(Zones!L8/1000),0)*Zones!N8*MAX(0,Hypothèses!$B$14-D8)</f>
-        <v>518.096333333333</v>
+        <v>507.837</v>
       </c>
       <c r="I8" s="24" t="n">
         <f aca="false">IF(D8&lt;0,Hypothèses!$B$6,Hypothèses!$B$7)*E8*MAX(0,Hypothèses!$B$15-D8)</f>
@@ -8150,7 +8329,7 @@
       </c>
       <c r="AA8" s="24" t="n">
         <f aca="false">G8+H8+I8+L8+P8+S8+T8+Z8</f>
-        <v>734.906333333333</v>
+        <v>720.247</v>
       </c>
       <c r="AB8" s="10" t="n">
         <v>18</v>
@@ -8167,7 +8346,7 @@
       </c>
       <c r="B9" s="16" t="str">
         <f aca="false">Zones!B9</f>
-        <v>Zone de refroidissement (2) + cuisson</v>
+        <v>Zone de cuisson / extrusion (ligne JBT)</v>
       </c>
       <c r="C9" s="16" t="str">
         <f aca="false">Zones!J9</f>
@@ -8179,19 +8358,19 @@
       </c>
       <c r="E9" s="35" t="n">
         <f aca="false">Zones!E9</f>
-        <v>201.697</v>
+        <v>197.703</v>
       </c>
       <c r="F9" s="34" t="n">
         <f aca="false">Zones!H9</f>
-        <v>1210.182</v>
+        <v>1186.218</v>
       </c>
       <c r="G9" s="24" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A9,Parois!$O$5:$O$41)+SUMIF(Parois!$C$5:$C$41,A9,Parois!$P$5:$P$41)</f>
-        <v>222.2</v>
+        <v>217.8</v>
       </c>
       <c r="H9" s="24" t="n">
         <f aca="false">IF(Zones!L9&gt;0,Hypothèses!$B$4/(Zones!L9/1000),0)*Zones!N9*MAX(0,Hypothèses!$B$14-D9)</f>
-        <v>369.777833333333</v>
+        <v>362.4555</v>
       </c>
       <c r="I9" s="24" t="n">
         <f aca="false">IF(D9&lt;0,Hypothèses!$B$6,Hypothèses!$B$7)*E9*MAX(0,Hypothèses!$B$15-D9)</f>
@@ -8254,7 +8433,7 @@
       </c>
       <c r="AA9" s="24" t="n">
         <f aca="false">G9+H9+I9+L9+P9+S9+T9+Z9</f>
-        <v>591.977833333333</v>
+        <v>580.2555</v>
       </c>
       <c r="AB9" s="10" t="n">
         <v>18</v>
@@ -8283,23 +8462,23 @@
       </c>
       <c r="E10" s="35" t="n">
         <f aca="false">Zones!E10</f>
-        <v>151.57</v>
+        <v>160.51</v>
       </c>
       <c r="F10" s="34" t="n">
         <f aca="false">Zones!H10</f>
-        <v>909.42</v>
+        <v>963.06</v>
       </c>
       <c r="G10" s="24" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A10,Parois!$O$5:$O$41)+SUMIF(Parois!$C$5:$C$41,A10,Parois!$P$5:$P$41)</f>
-        <v>2170.86375</v>
+        <v>2133.02375</v>
       </c>
       <c r="H10" s="24" t="n">
         <f aca="false">IF(Zones!L10&gt;0,Hypothèses!$B$4/(Zones!L10/1000),0)*Zones!N10*MAX(0,Hypothèses!$B$14-D10)</f>
-        <v>1250.4525</v>
+        <v>1324.2075</v>
       </c>
       <c r="I10" s="24" t="n">
         <f aca="false">IF(D10&lt;0,Hypothèses!$B$6,Hypothèses!$B$7)*E10*MAX(0,Hypothèses!$B$15-D10)</f>
-        <v>909.42</v>
+        <v>963.06</v>
       </c>
       <c r="J10" s="36" t="n">
         <v>10</v>
@@ -8309,7 +8488,7 @@
       </c>
       <c r="L10" s="24" t="n">
         <f aca="false">J10*F10*Hypothèses!$B$5*K10*1000/86400</f>
-        <v>5683.875</v>
+        <v>6019.125</v>
       </c>
       <c r="M10" s="10" t="n">
         <v>6</v>
@@ -8332,7 +8511,7 @@
       </c>
       <c r="S10" s="24" t="n">
         <f aca="false">Q10*E10*R10/24</f>
-        <v>1010.46666666667</v>
+        <v>1070.06666666667</v>
       </c>
       <c r="T10" s="12" t="n">
         <v>2000</v>
@@ -8358,14 +8537,14 @@
       </c>
       <c r="AA10" s="24" t="n">
         <f aca="false">G10+H10+I10+L10+P10+S10+T10+Z10</f>
-        <v>13865.0779166667</v>
+        <v>14349.4829166667</v>
       </c>
       <c r="AB10" s="10" t="n">
         <v>18</v>
       </c>
       <c r="AC10" s="37" t="n">
         <f aca="false">IF(C10="Oui",AA10*(1+Hypothèses!$B$8)*24/AB10/1000,0)</f>
-        <v>22.1841246666667</v>
+        <v>22.9591726666667</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8699,11 +8878,11 @@
       </c>
       <c r="E14" s="35" t="n">
         <f aca="false">Zones!E14</f>
-        <v>316.58</v>
+        <v>314.48</v>
       </c>
       <c r="F14" s="34" t="n">
         <f aca="false">Zones!H14</f>
-        <v>1899.48</v>
+        <v>1886.88</v>
       </c>
       <c r="G14" s="24" t="n">
         <f aca="false">SUMIF(Parois!$B$5:$B$41,A14,Parois!$O$5:$O$41)+SUMIF(Parois!$C$5:$C$41,A14,Parois!$P$5:$P$41)</f>
@@ -8786,41 +8965,41 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="28" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="AC15" s="38" t="n">
         <f aca="false">SUM(AC5:AC14)</f>
-        <v>54.0089330142815</v>
+        <v>54.7839810142815</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="5" t="s">
-        <v>274</v>
+        <v>281</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="39" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="39" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="39" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="39" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="39" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
P1 RDC v5: retorts in 2 facing rows of 3 with central aisle
Stérilisation 20.34 x 8.50 m: strip narrowed to 4.00 m alongside it
(SAS keeps a 1.40 m passage), six Steriflow 1300 retorts east-west in
two rows of 3 facing a 4.50 m north-south basket aisle, door to
refroidissement on the aisle axis. Refroidissement (1) 12.50 m.
Dimensions, areas, surface table, PDF and workbook updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011Ghrdsx3moo1sM21DD7JVm
</commit_message>
<xml_diff>
--- a/DWG_Plan_Modificatif/DWG Plan Modificatif/Unite Humide - dimensions panneaux froid.xlsx
+++ b/DWG_Plan_Modificatif/DWG Plan Modificatif/Unite Humide - dimensions panneaux froid.xlsx
@@ -1203,6 +1203,30 @@
         </r>
       </text>
     </comment>
+    <comment ref="E42" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Mesuré sur P1 RDC v2.dwg (RDC Modifié), entre nus intérieurs des murs</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E43" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Mesuré sur P1 RDC v2.dwg (RDC Modifié), entre nus intérieurs des murs</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="L5" authorId="0">
       <text>
         <r>
@@ -1636,6 +1660,30 @@
       </text>
     </comment>
     <comment ref="L41" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">U ≈ λ / épaisseur (résistances superficielles négligées). Paroi non isolée : 0 (non comptée).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L42" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">U ≈ λ / épaisseur (résistances superficielles négligées). Paroi non isolée : 0 (non comptée).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L43" authorId="0">
       <text>
         <r>
           <rPr>
@@ -1652,7 +1700,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="291">
   <si>
     <t xml:space="preserve">Unité Humide – RDC Modifié (P1 RDC v2) : dimensions, panneaux sandwich et puissance frigorifique</t>
   </si>
@@ -1930,7 +1978,7 @@
     <t xml:space="preserve">Zone de stérilisation</t>
   </si>
   <si>
-    <t xml:space="preserve">6 autoclaves Steriflow 1300 (7 225 × ~1 650 mm, 10,4 t pleins d'eau chacun), allée paniers 4,50 m. Pas de mur entre stérilisation et sertissage sur le plan (espace ouvert sur 7,00 m).</t>
+    <t xml:space="preserve">6 autoclaves Steriflow 1300 en 2 rangées de 3 face à face (7 225 × ~1 650 mm, 10,4 t pleins d'eau chacun), allée centrale nord-sud 4,50 m. Pas de mur entre stérilisation et sertissage sur le plan (espace ouvert sur 7,00 m).</t>
   </si>
   <si>
     <t xml:space="preserve">Z4</t>
@@ -2242,7 +2290,19 @@
     <t xml:space="preserve">P10</t>
   </si>
   <si>
-    <t xml:space="preserve">Stérilisation / circulation</t>
+    <t xml:space="preserve">Stérilisation / circulation (ouest, couloir réduit à 4,00 m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stérilisation / circulation (retour nord)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stérilisation / circulation (retour sud)</t>
   </si>
   <si>
     <t xml:space="preserve">P12</t>
@@ -3952,7 +4012,7 @@
         <v>60</v>
       </c>
       <c r="M5" s="22" t="n">
-        <f aca="false">SUMIF(Parois!$B$5:$B$41,A5,Parois!$J$5:$J$41)+SUMIF(Parois!$C$5:$C$41,A5,Parois!$J$5:$J$41)-SUMIFS(Parois!$J$5:$J$41,Parois!$B$5:$B$41,A5,Parois!$C$5:$C$41,A5)</f>
+        <f aca="false">SUMIF(Parois!$B$5:$B$43,A5,Parois!$J$5:$J$43)+SUMIF(Parois!$C$5:$C$43,A5,Parois!$J$5:$J$43)-SUMIFS(Parois!$J$5:$J$43,Parois!$B$5:$B$43,A5,Parois!$C$5:$C$43,A5)</f>
         <v>428.55</v>
       </c>
       <c r="N5" s="22" t="n">
@@ -3969,25 +4029,25 @@
         <v>89</v>
       </c>
       <c r="C6" s="21" t="n">
-        <v>8.5</v>
+        <v>12.5</v>
       </c>
       <c r="D6" s="21" t="n">
         <v>17.08</v>
       </c>
       <c r="E6" s="22" t="n">
         <f aca="false">C6*D6</f>
-        <v>145.18</v>
+        <v>213.5</v>
       </c>
       <c r="F6" s="23" t="n">
         <f aca="false">2*(C6+D6)</f>
-        <v>51.16</v>
+        <v>59.16</v>
       </c>
       <c r="G6" s="15" t="n">
         <v>6</v>
       </c>
       <c r="H6" s="24" t="n">
         <f aca="false">E6*G6</f>
-        <v>871.08</v>
+        <v>1281</v>
       </c>
       <c r="I6" s="25" t="s">
         <v>87</v>
@@ -4003,12 +4063,12 @@
         <v>60</v>
       </c>
       <c r="M6" s="22" t="n">
-        <f aca="false">SUMIF(Parois!$B$5:$B$41,A6,Parois!$J$5:$J$41)+SUMIF(Parois!$C$5:$C$41,A6,Parois!$J$5:$J$41)-SUMIFS(Parois!$J$5:$J$41,Parois!$B$5:$B$41,A6,Parois!$C$5:$C$41,A6)</f>
-        <v>301.08</v>
+        <f aca="false">SUMIF(Parois!$B$5:$B$43,A6,Parois!$J$5:$J$43)+SUMIF(Parois!$C$5:$C$43,A6,Parois!$J$5:$J$43)-SUMIFS(Parois!$J$5:$J$43,Parois!$B$5:$B$43,A6,Parois!$C$5:$C$43,A6)</f>
+        <v>349.08</v>
       </c>
       <c r="N6" s="22" t="n">
         <f aca="false">IF(I6="Oui",E6,0)</f>
-        <v>145.18</v>
+        <v>213.5</v>
       </c>
       <c r="O6" s="26"/>
     </row>
@@ -4020,25 +4080,25 @@
         <v>91</v>
       </c>
       <c r="C7" s="21" t="n">
-        <v>12.5</v>
+        <v>8.5</v>
       </c>
       <c r="D7" s="21" t="n">
-        <v>17.08</v>
+        <v>20.34</v>
       </c>
       <c r="E7" s="22" t="n">
         <f aca="false">C7*D7</f>
-        <v>213.5</v>
+        <v>172.89</v>
       </c>
       <c r="F7" s="23" t="n">
         <f aca="false">2*(C7+D7)</f>
-        <v>59.16</v>
+        <v>57.68</v>
       </c>
       <c r="G7" s="15" t="n">
         <v>6</v>
       </c>
       <c r="H7" s="24" t="n">
         <f aca="false">E7*G7</f>
-        <v>1281</v>
+        <v>1037.34</v>
       </c>
       <c r="I7" s="25" t="s">
         <v>87</v>
@@ -4054,12 +4114,12 @@
         <v>60</v>
       </c>
       <c r="M7" s="22" t="n">
-        <f aca="false">SUMIF(Parois!$B$5:$B$41,A7,Parois!$J$5:$J$41)+SUMIF(Parois!$C$5:$C$41,A7,Parois!$J$5:$J$41)-SUMIFS(Parois!$J$5:$J$41,Parois!$B$5:$B$41,A7,Parois!$C$5:$C$41,A7)</f>
-        <v>309.45</v>
+        <f aca="false">SUMIF(Parois!$B$5:$B$43,A7,Parois!$J$5:$J$43)+SUMIF(Parois!$C$5:$C$43,A7,Parois!$J$5:$J$43)-SUMIFS(Parois!$J$5:$J$43,Parois!$B$5:$B$43,A7,Parois!$C$5:$C$43,A7)</f>
+        <v>299.37</v>
       </c>
       <c r="N7" s="22" t="n">
         <f aca="false">IF(I7="Oui",E7,0)</f>
-        <v>213.5</v>
+        <v>172.89</v>
       </c>
       <c r="O7" s="26" t="s">
         <v>92</v>
@@ -4107,7 +4167,7 @@
         <v>60</v>
       </c>
       <c r="M8" s="22" t="n">
-        <f aca="false">SUMIF(Parois!$B$5:$B$41,A8,Parois!$J$5:$J$41)+SUMIF(Parois!$C$5:$C$41,A8,Parois!$J$5:$J$41)-SUMIFS(Parois!$J$5:$J$41,Parois!$B$5:$B$41,A8,Parois!$C$5:$C$41,A8)</f>
+        <f aca="false">SUMIF(Parois!$B$5:$B$43,A8,Parois!$J$5:$J$43)+SUMIF(Parois!$C$5:$C$43,A8,Parois!$J$5:$J$43)-SUMIFS(Parois!$J$5:$J$43,Parois!$B$5:$B$43,A8,Parois!$C$5:$C$43,A8)</f>
         <v>270.75</v>
       </c>
       <c r="N8" s="22" t="n">
@@ -4160,7 +4220,7 @@
         <v>60</v>
       </c>
       <c r="M9" s="22" t="n">
-        <f aca="false">SUMIF(Parois!$B$5:$B$41,A9,Parois!$J$5:$J$41)+SUMIF(Parois!$C$5:$C$41,A9,Parois!$J$5:$J$41)-SUMIFS(Parois!$J$5:$J$41,Parois!$B$5:$B$41,A9,Parois!$C$5:$C$41,A9)</f>
+        <f aca="false">SUMIF(Parois!$B$5:$B$43,A9,Parois!$J$5:$J$43)+SUMIF(Parois!$C$5:$C$43,A9,Parois!$J$5:$J$43)-SUMIFS(Parois!$J$5:$J$43,Parois!$B$5:$B$43,A9,Parois!$C$5:$C$43,A9)</f>
         <v>345.94</v>
       </c>
       <c r="N9" s="22" t="n">
@@ -4211,7 +4271,7 @@
         <v>80</v>
       </c>
       <c r="M10" s="22" t="n">
-        <f aca="false">SUMIF(Parois!$B$5:$B$41,A10,Parois!$J$5:$J$41)+SUMIF(Parois!$C$5:$C$41,A10,Parois!$J$5:$J$41)-SUMIFS(Parois!$J$5:$J$41,Parois!$B$5:$B$41,A10,Parois!$C$5:$C$41,A10)</f>
+        <f aca="false">SUMIF(Parois!$B$5:$B$43,A10,Parois!$J$5:$J$43)+SUMIF(Parois!$C$5:$C$43,A10,Parois!$J$5:$J$43)-SUMIFS(Parois!$J$5:$J$43,Parois!$B$5:$B$43,A10,Parois!$C$5:$C$43,A10)</f>
         <v>349.78</v>
       </c>
       <c r="N10" s="22" t="n">
@@ -4264,7 +4324,7 @@
         <v>60</v>
       </c>
       <c r="M11" s="22" t="n">
-        <f aca="false">SUMIF(Parois!$B$5:$B$41,A11,Parois!$J$5:$J$41)+SUMIF(Parois!$C$5:$C$41,A11,Parois!$J$5:$J$41)-SUMIFS(Parois!$J$5:$J$41,Parois!$B$5:$B$41,A11,Parois!$C$5:$C$41,A11)</f>
+        <f aca="false">SUMIF(Parois!$B$5:$B$43,A11,Parois!$J$5:$J$43)+SUMIF(Parois!$C$5:$C$43,A11,Parois!$J$5:$J$43)-SUMIFS(Parois!$J$5:$J$43,Parois!$B$5:$B$43,A11,Parois!$C$5:$C$43,A11)</f>
         <v>327.81</v>
       </c>
       <c r="N11" s="22" t="n">
@@ -4317,7 +4377,7 @@
         <v>150</v>
       </c>
       <c r="M12" s="22" t="n">
-        <f aca="false">SUMIF(Parois!$B$5:$B$41,A12,Parois!$J$5:$J$41)+SUMIF(Parois!$C$5:$C$41,A12,Parois!$J$5:$J$41)-SUMIFS(Parois!$J$5:$J$41,Parois!$B$5:$B$41,A12,Parois!$C$5:$C$41,A12)</f>
+        <f aca="false">SUMIF(Parois!$B$5:$B$43,A12,Parois!$J$5:$J$43)+SUMIF(Parois!$C$5:$C$43,A12,Parois!$J$5:$J$43)-SUMIFS(Parois!$J$5:$J$43,Parois!$B$5:$B$43,A12,Parois!$C$5:$C$43,A12)</f>
         <v>397.92</v>
       </c>
       <c r="N12" s="22" t="n">
@@ -4370,7 +4430,7 @@
         <v>100</v>
       </c>
       <c r="M13" s="22" t="n">
-        <f aca="false">SUMIF(Parois!$B$5:$B$41,A13,Parois!$J$5:$J$41)+SUMIF(Parois!$C$5:$C$41,A13,Parois!$J$5:$J$41)-SUMIFS(Parois!$J$5:$J$41,Parois!$B$5:$B$41,A13,Parois!$C$5:$C$41,A13)</f>
+        <f aca="false">SUMIF(Parois!$B$5:$B$43,A13,Parois!$J$5:$J$43)+SUMIF(Parois!$C$5:$C$43,A13,Parois!$J$5:$J$43)-SUMIFS(Parois!$J$5:$J$43,Parois!$B$5:$B$43,A13,Parois!$C$5:$C$43,A13)</f>
         <v>237.18</v>
       </c>
       <c r="N13" s="22" t="n">
@@ -4393,17 +4453,17 @@
         <v>101</v>
       </c>
       <c r="E14" s="27" t="n">
-        <v>314.48</v>
+        <v>286.11</v>
       </c>
       <c r="F14" s="21" t="n">
-        <v>130.38</v>
+        <v>136.9</v>
       </c>
       <c r="G14" s="15" t="n">
         <v>6</v>
       </c>
       <c r="H14" s="24" t="n">
         <f aca="false">E14*G14</f>
-        <v>1886.88</v>
+        <v>1716.66</v>
       </c>
       <c r="I14" s="25" t="s">
         <v>64</v>
@@ -4419,8 +4479,8 @@
         <v>0</v>
       </c>
       <c r="M14" s="22" t="n">
-        <f aca="false">SUMIF(Parois!$B$5:$B$41,A14,Parois!$J$5:$J$41)+SUMIF(Parois!$C$5:$C$41,A14,Parois!$J$5:$J$41)-SUMIFS(Parois!$J$5:$J$41,Parois!$B$5:$B$41,A14,Parois!$C$5:$C$41,A14)</f>
-        <v>854.07</v>
+        <f aca="false">SUMIF(Parois!$B$5:$B$43,A14,Parois!$J$5:$J$43)+SUMIF(Parois!$C$5:$C$43,A14,Parois!$J$5:$J$43)-SUMIFS(Parois!$J$5:$J$43,Parois!$B$5:$B$43,A14,Parois!$C$5:$C$43,A14)</f>
+        <v>891.99</v>
       </c>
       <c r="N14" s="22" t="n">
         <f aca="false">IF(I14="Oui",E14,0)</f>
@@ -4436,19 +4496,19 @@
       </c>
       <c r="E15" s="29" t="n">
         <f aca="false">SUM(E5:E14)</f>
-        <v>1892.7746</v>
+        <v>1892.1146</v>
       </c>
       <c r="H15" s="30" t="n">
         <f aca="false">SUM(H5:H14)</f>
-        <v>11356.6476</v>
+        <v>11352.6876</v>
       </c>
       <c r="M15" s="29" t="n">
         <f aca="false">SUM(M5:M14)</f>
-        <v>3822.53</v>
+        <v>3898.37</v>
       </c>
       <c r="N15" s="29" t="n">
         <f aca="false">SUM(N5:N14)</f>
-        <v>1578.2946</v>
+        <v>1606.0046</v>
       </c>
     </row>
   </sheetData>
@@ -5115,7 +5175,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P44"/>
+  <dimension ref="A1:P46"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -5508,7 +5568,7 @@
         <v>189</v>
       </c>
       <c r="E10" s="21" t="n">
-        <v>8.5</v>
+        <v>12.5</v>
       </c>
       <c r="F10" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B10,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C10,Zones!$A$5:$A$14,0)),0))</f>
@@ -5516,7 +5576,7 @@
       </c>
       <c r="G10" s="22" t="n">
         <f aca="false">E10*F10</f>
-        <v>51</v>
+        <v>75</v>
       </c>
       <c r="H10" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A10,Portes!$H$5:$H$23)</f>
@@ -5528,7 +5588,7 @@
       </c>
       <c r="J10" s="22" t="n">
         <f aca="false">MAX(0,G10-H10)</f>
-        <v>51</v>
+        <v>75</v>
       </c>
       <c r="K10" s="18" t="n">
         <f aca="false">IF(I10="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B10,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C10,Hypothèses!$A$38:$A$53,0))),0)</f>
@@ -5548,7 +5608,7 @@
       </c>
       <c r="O10" s="24" t="n">
         <f aca="false">L10*J10*MAX(0,N10-M10)</f>
-        <v>187</v>
+        <v>275</v>
       </c>
       <c r="P10" s="24" t="n">
         <f aca="false">L10*J10*MAX(0,M10-N10)</f>
@@ -5630,7 +5690,7 @@
         <v>192</v>
       </c>
       <c r="E12" s="21" t="n">
-        <v>8.5</v>
+        <v>12.5</v>
       </c>
       <c r="F12" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B12,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C12,Zones!$A$5:$A$14,0)),0))</f>
@@ -5638,7 +5698,7 @@
       </c>
       <c r="G12" s="22" t="n">
         <f aca="false">E12*F12</f>
-        <v>51</v>
+        <v>75</v>
       </c>
       <c r="H12" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A12,Portes!$H$5:$H$23)</f>
@@ -5650,7 +5710,7 @@
       </c>
       <c r="J12" s="22" t="n">
         <f aca="false">MAX(0,G12-H12)</f>
-        <v>51</v>
+        <v>75</v>
       </c>
       <c r="K12" s="18" t="n">
         <f aca="false">IF(I12="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B12,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C12,Hypothèses!$A$38:$A$53,0))),0)</f>
@@ -5691,7 +5751,7 @@
         <v>194</v>
       </c>
       <c r="E13" s="21" t="n">
-        <v>12.5</v>
+        <v>8.5</v>
       </c>
       <c r="F13" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B13,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C13,Zones!$A$5:$A$14,0)),0))</f>
@@ -5699,7 +5759,7 @@
       </c>
       <c r="G13" s="22" t="n">
         <f aca="false">E13*F13</f>
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="H13" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A13,Portes!$H$5:$H$23)</f>
@@ -5711,7 +5771,7 @@
       </c>
       <c r="J13" s="22" t="n">
         <f aca="false">MAX(0,G13-H13)</f>
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="K13" s="18" t="n">
         <f aca="false">IF(I13="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B13,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C13,Hypothèses!$A$38:$A$53,0))),0)</f>
@@ -5731,7 +5791,7 @@
       </c>
       <c r="O13" s="24" t="n">
         <f aca="false">L13*J13*MAX(0,N13-M13)</f>
-        <v>137.5</v>
+        <v>93.5</v>
       </c>
       <c r="P13" s="24" t="n">
         <f aca="false">L13*J13*MAX(0,M13-N13)</f>
@@ -5752,7 +5812,7 @@
         <v>196</v>
       </c>
       <c r="E14" s="21" t="n">
-        <v>12.5</v>
+        <v>8.5</v>
       </c>
       <c r="F14" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B14,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C14,Zones!$A$5:$A$14,0)),0))</f>
@@ -5760,7 +5820,7 @@
       </c>
       <c r="G14" s="22" t="n">
         <f aca="false">E14*F14</f>
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="H14" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A14,Portes!$H$5:$H$23)</f>
@@ -5772,7 +5832,7 @@
       </c>
       <c r="J14" s="22" t="n">
         <f aca="false">MAX(0,G14-H14)</f>
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="K14" s="18" t="n">
         <f aca="false">IF(I14="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B14,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C14,Hypothèses!$A$38:$A$53,0))),0)</f>
@@ -5796,7 +5856,7 @@
       </c>
       <c r="P14" s="24" t="n">
         <f aca="false">L14*J14*MAX(0,M14-N14)</f>
-        <v>137.5</v>
+        <v>93.5</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5807,13 +5867,13 @@
         <v>90</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>96</v>
+        <v>111</v>
       </c>
       <c r="D15" s="14" t="s">
         <v>198</v>
       </c>
       <c r="E15" s="21" t="n">
-        <v>9.985</v>
+        <v>3.16</v>
       </c>
       <c r="F15" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B15,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C15,Zones!$A$5:$A$14,0)),0))</f>
@@ -5821,7 +5881,7 @@
       </c>
       <c r="G15" s="22" t="n">
         <f aca="false">E15*F15</f>
-        <v>59.91</v>
+        <v>18.96</v>
       </c>
       <c r="H15" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A15,Portes!$H$5:$H$23)</f>
@@ -5833,7 +5893,7 @@
       </c>
       <c r="J15" s="22" t="n">
         <f aca="false">MAX(0,G15-H15)</f>
-        <v>59.91</v>
+        <v>18.96</v>
       </c>
       <c r="K15" s="18" t="n">
         <f aca="false">IF(I15="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B15,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C15,Hypothèses!$A$38:$A$53,0))),0)</f>
@@ -5849,7 +5909,7 @@
       </c>
       <c r="N15" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C15,Hypothèses!$A$38:$A$53,0))</f>
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="O15" s="24" t="n">
         <f aca="false">L15*J15*MAX(0,N15-M15)</f>
@@ -5857,24 +5917,24 @@
       </c>
       <c r="P15" s="24" t="n">
         <f aca="false">L15*J15*MAX(0,M15-N15)</f>
-        <v>0</v>
+        <v>34.76</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="20" t="s">
-        <v>132</v>
+        <v>199</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C16" s="14" t="s">
         <v>111</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E16" s="21" t="n">
-        <v>19.8</v>
+        <v>3.16</v>
       </c>
       <c r="F16" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B16,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C16,Zones!$A$5:$A$14,0)),0))</f>
@@ -5882,11 +5942,11 @@
       </c>
       <c r="G16" s="22" t="n">
         <f aca="false">E16*F16</f>
-        <v>118.8</v>
+        <v>18.96</v>
       </c>
       <c r="H16" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A16,Portes!$H$5:$H$23)</f>
-        <v>2.94</v>
+        <v>0</v>
       </c>
       <c r="I16" s="14" t="str">
         <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B16,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C16,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
@@ -5894,7 +5954,7 @@
       </c>
       <c r="J16" s="22" t="n">
         <f aca="false">MAX(0,G16-H16)</f>
-        <v>115.86</v>
+        <v>18.96</v>
       </c>
       <c r="K16" s="18" t="n">
         <f aca="false">IF(I16="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B16,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C16,Hypothèses!$A$38:$A$53,0))),0)</f>
@@ -5906,7 +5966,7 @@
       </c>
       <c r="M16" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B16,Hypothèses!$A$38:$A$53,0))</f>
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="N16" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C16,Hypothèses!$A$38:$A$53,0))</f>
@@ -5918,24 +5978,24 @@
       </c>
       <c r="P16" s="24" t="n">
         <f aca="false">L16*J16*MAX(0,M16-N16)</f>
-        <v>0</v>
+        <v>34.76</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="s">
-        <v>130</v>
+        <v>201</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C17" s="14" t="s">
         <v>96</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="E17" s="21" t="n">
-        <v>19.8</v>
+        <v>9.985</v>
       </c>
       <c r="F17" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B17,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C17,Zones!$A$5:$A$14,0)),0))</f>
@@ -5943,11 +6003,11 @@
       </c>
       <c r="G17" s="22" t="n">
         <f aca="false">E17*F17</f>
-        <v>118.8</v>
+        <v>59.91</v>
       </c>
       <c r="H17" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A17,Portes!$H$5:$H$23)</f>
-        <v>2.94</v>
+        <v>0</v>
       </c>
       <c r="I17" s="14" t="str">
         <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B17,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C17,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
@@ -5955,7 +6015,7 @@
       </c>
       <c r="J17" s="22" t="n">
         <f aca="false">MAX(0,G17-H17)</f>
-        <v>115.86</v>
+        <v>59.91</v>
       </c>
       <c r="K17" s="18" t="n">
         <f aca="false">IF(I17="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B17,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C17,Hypothèses!$A$38:$A$53,0))),0)</f>
@@ -5967,7 +6027,7 @@
       </c>
       <c r="M17" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B17,Hypothèses!$A$38:$A$53,0))</f>
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="N17" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C17,Hypothèses!$A$38:$A$53,0))</f>
@@ -5975,7 +6035,7 @@
       </c>
       <c r="O17" s="24" t="n">
         <f aca="false">L17*J17*MAX(0,N17-M17)</f>
-        <v>212.41</v>
+        <v>0</v>
       </c>
       <c r="P17" s="24" t="n">
         <f aca="false">L17*J17*MAX(0,M17-N17)</f>
@@ -5984,16 +6044,16 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="20" t="s">
-        <v>201</v>
+        <v>132</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>63</v>
+        <v>111</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E18" s="21" t="n">
         <v>19.8</v>
@@ -6008,7 +6068,7 @@
       </c>
       <c r="H18" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A18,Portes!$H$5:$H$23)</f>
-        <v>0</v>
+        <v>2.94</v>
       </c>
       <c r="I18" s="14" t="str">
         <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B18,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C18,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
@@ -6016,7 +6076,7 @@
       </c>
       <c r="J18" s="22" t="n">
         <f aca="false">MAX(0,G18-H18)</f>
-        <v>118.8</v>
+        <v>115.86</v>
       </c>
       <c r="K18" s="18" t="n">
         <f aca="false">IF(I18="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B18,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C18,Hypothèses!$A$38:$A$53,0))),0)</f>
@@ -6028,15 +6088,15 @@
       </c>
       <c r="M18" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B18,Hypothèses!$A$38:$A$53,0))</f>
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="N18" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C18,Hypothèses!$A$38:$A$53,0))</f>
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O18" s="24" t="n">
         <f aca="false">L18*J18*MAX(0,N18-M18)</f>
-        <v>217.8</v>
+        <v>0</v>
       </c>
       <c r="P18" s="24" t="n">
         <f aca="false">L18*J18*MAX(0,M18-N18)</f>
@@ -6045,19 +6105,19 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="20" t="s">
-        <v>164</v>
+        <v>130</v>
       </c>
       <c r="B19" s="14" t="s">
         <v>93</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E19" s="21" t="n">
-        <v>6.995</v>
+        <v>19.8</v>
       </c>
       <c r="F19" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B19,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C19,Zones!$A$5:$A$14,0)),0))</f>
@@ -6065,7 +6125,7 @@
       </c>
       <c r="G19" s="22" t="n">
         <f aca="false">E19*F19</f>
-        <v>41.97</v>
+        <v>118.8</v>
       </c>
       <c r="H19" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A19,Portes!$H$5:$H$23)</f>
@@ -6077,15 +6137,15 @@
       </c>
       <c r="J19" s="22" t="n">
         <f aca="false">MAX(0,G19-H19)</f>
-        <v>39.03</v>
+        <v>115.86</v>
       </c>
       <c r="K19" s="18" t="n">
         <f aca="false">IF(I19="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B19,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C19,Hypothèses!$A$38:$A$53,0))),0)</f>
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="L19" s="32" t="n">
         <f aca="false">IF(K19&gt;0,Hypothèses!$B$4/(K19/1000),0)</f>
-        <v>0.275</v>
+        <v>0.366666666666667</v>
       </c>
       <c r="M19" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B19,Hypothèses!$A$38:$A$53,0))</f>
@@ -6093,32 +6153,32 @@
       </c>
       <c r="N19" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C19,Hypothèses!$A$38:$A$53,0))</f>
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="O19" s="24" t="n">
         <f aca="false">L19*J19*MAX(0,N19-M19)</f>
-        <v>0</v>
+        <v>212.41</v>
       </c>
       <c r="P19" s="24" t="n">
         <f aca="false">L19*J19*MAX(0,M19-N19)</f>
-        <v>214.665</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>111</v>
+        <v>96</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>99</v>
+        <v>63</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E20" s="21" t="n">
-        <v>5.165</v>
+        <v>19.8</v>
       </c>
       <c r="F20" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B20,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C20,Zones!$A$5:$A$14,0)),0))</f>
@@ -6126,7 +6186,7 @@
       </c>
       <c r="G20" s="22" t="n">
         <f aca="false">E20*F20</f>
-        <v>30.99</v>
+        <v>118.8</v>
       </c>
       <c r="H20" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A20,Portes!$H$5:$H$23)</f>
@@ -6138,48 +6198,48 @@
       </c>
       <c r="J20" s="22" t="n">
         <f aca="false">MAX(0,G20-H20)</f>
-        <v>30.99</v>
+        <v>118.8</v>
       </c>
       <c r="K20" s="18" t="n">
         <f aca="false">IF(I20="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B20,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C20,Hypothèses!$A$38:$A$53,0))),0)</f>
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="L20" s="32" t="n">
         <f aca="false">IF(K20&gt;0,Hypothèses!$B$4/(K20/1000),0)</f>
-        <v>0.275</v>
+        <v>0.366666666666667</v>
       </c>
       <c r="M20" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B20,Hypothèses!$A$38:$A$53,0))</f>
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="N20" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C20,Hypothèses!$A$38:$A$53,0))</f>
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="O20" s="24" t="n">
         <f aca="false">L20*J20*MAX(0,N20-M20)</f>
-        <v>0</v>
+        <v>217.8</v>
       </c>
       <c r="P20" s="24" t="n">
         <f aca="false">L20*J20*MAX(0,M20-N20)</f>
-        <v>170.445</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="s">
-        <v>134</v>
+        <v>164</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C21" s="14" t="s">
         <v>99</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E21" s="21" t="n">
-        <v>9.985</v>
+        <v>6.995</v>
       </c>
       <c r="F21" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B21,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C21,Zones!$A$5:$A$14,0)),0))</f>
@@ -6187,11 +6247,11 @@
       </c>
       <c r="G21" s="22" t="n">
         <f aca="false">E21*F21</f>
-        <v>59.91</v>
+        <v>41.97</v>
       </c>
       <c r="H21" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A21,Portes!$H$5:$H$23)</f>
-        <v>8.54</v>
+        <v>2.94</v>
       </c>
       <c r="I21" s="14" t="str">
         <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B21,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C21,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
@@ -6199,7 +6259,7 @@
       </c>
       <c r="J21" s="22" t="n">
         <f aca="false">MAX(0,G21-H21)</f>
-        <v>51.37</v>
+        <v>39.03</v>
       </c>
       <c r="K21" s="18" t="n">
         <f aca="false">IF(I21="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B21,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C21,Hypothèses!$A$38:$A$53,0))),0)</f>
@@ -6211,7 +6271,7 @@
       </c>
       <c r="M21" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B21,Hypothèses!$A$38:$A$53,0))</f>
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="N21" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C21,Hypothèses!$A$38:$A$53,0))</f>
@@ -6223,12 +6283,12 @@
       </c>
       <c r="P21" s="24" t="n">
         <f aca="false">L21*J21*MAX(0,M21-N21)</f>
-        <v>353.16875</v>
+        <v>214.665</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="20" t="s">
-        <v>161</v>
+        <v>208</v>
       </c>
       <c r="B22" s="14" t="s">
         <v>111</v>
@@ -6237,10 +6297,10 @@
         <v>99</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E22" s="21" t="n">
-        <v>6.2</v>
+        <v>5.165</v>
       </c>
       <c r="F22" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B22,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C22,Zones!$A$5:$A$14,0)),0))</f>
@@ -6248,11 +6308,11 @@
       </c>
       <c r="G22" s="22" t="n">
         <f aca="false">E22*F22</f>
-        <v>37.2</v>
+        <v>30.99</v>
       </c>
       <c r="H22" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A22,Portes!$H$5:$H$23)</f>
-        <v>2.94</v>
+        <v>0</v>
       </c>
       <c r="I22" s="14" t="str">
         <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B22,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C22,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
@@ -6260,7 +6320,7 @@
       </c>
       <c r="J22" s="22" t="n">
         <f aca="false">MAX(0,G22-H22)</f>
-        <v>34.26</v>
+        <v>30.99</v>
       </c>
       <c r="K22" s="18" t="n">
         <f aca="false">IF(I22="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B22,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C22,Hypothèses!$A$38:$A$53,0))),0)</f>
@@ -6284,24 +6344,24 @@
       </c>
       <c r="P22" s="24" t="n">
         <f aca="false">L22*J22*MAX(0,M22-N22)</f>
-        <v>188.43</v>
+        <v>170.445</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="s">
-        <v>208</v>
+        <v>134</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>111</v>
+        <v>96</v>
       </c>
       <c r="C23" s="14" t="s">
         <v>99</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E23" s="21" t="n">
-        <v>8.33</v>
+        <v>9.985</v>
       </c>
       <c r="F23" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B23,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C23,Zones!$A$5:$A$14,0)),0))</f>
@@ -6309,11 +6369,11 @@
       </c>
       <c r="G23" s="22" t="n">
         <f aca="false">E23*F23</f>
-        <v>49.98</v>
+        <v>59.91</v>
       </c>
       <c r="H23" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A23,Portes!$H$5:$H$23)</f>
-        <v>0</v>
+        <v>8.54</v>
       </c>
       <c r="I23" s="14" t="str">
         <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B23,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C23,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
@@ -6321,7 +6381,7 @@
       </c>
       <c r="J23" s="22" t="n">
         <f aca="false">MAX(0,G23-H23)</f>
-        <v>49.98</v>
+        <v>51.37</v>
       </c>
       <c r="K23" s="18" t="n">
         <f aca="false">IF(I23="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B23,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C23,Hypothèses!$A$38:$A$53,0))),0)</f>
@@ -6333,7 +6393,7 @@
       </c>
       <c r="M23" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B23,Hypothèses!$A$38:$A$53,0))</f>
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="N23" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C23,Hypothèses!$A$38:$A$53,0))</f>
@@ -6345,15 +6405,15 @@
       </c>
       <c r="P23" s="24" t="n">
         <f aca="false">L23*J23*MAX(0,M23-N23)</f>
-        <v>274.89</v>
+        <v>353.16875</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="s">
-        <v>210</v>
+        <v>161</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>69</v>
+        <v>111</v>
       </c>
       <c r="C24" s="14" t="s">
         <v>99</v>
@@ -6362,7 +6422,7 @@
         <v>211</v>
       </c>
       <c r="E24" s="21" t="n">
-        <v>3.93</v>
+        <v>6.2</v>
       </c>
       <c r="F24" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B24,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C24,Zones!$A$5:$A$14,0)),0))</f>
@@ -6370,11 +6430,11 @@
       </c>
       <c r="G24" s="22" t="n">
         <f aca="false">E24*F24</f>
-        <v>23.58</v>
+        <v>37.2</v>
       </c>
       <c r="H24" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A24,Portes!$H$5:$H$23)</f>
-        <v>0</v>
+        <v>2.94</v>
       </c>
       <c r="I24" s="14" t="str">
         <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B24,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C24,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
@@ -6382,7 +6442,7 @@
       </c>
       <c r="J24" s="22" t="n">
         <f aca="false">MAX(0,G24-H24)</f>
-        <v>23.58</v>
+        <v>34.26</v>
       </c>
       <c r="K24" s="18" t="n">
         <f aca="false">IF(I24="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B24,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C24,Hypothèses!$A$38:$A$53,0))),0)</f>
@@ -6406,7 +6466,7 @@
       </c>
       <c r="P24" s="24" t="n">
         <f aca="false">L24*J24*MAX(0,M24-N24)</f>
-        <v>129.69</v>
+        <v>188.43</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6414,7 +6474,7 @@
         <v>212</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>69</v>
+        <v>111</v>
       </c>
       <c r="C25" s="14" t="s">
         <v>99</v>
@@ -6423,7 +6483,7 @@
         <v>213</v>
       </c>
       <c r="E25" s="21" t="n">
-        <v>2.2</v>
+        <v>8.33</v>
       </c>
       <c r="F25" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B25,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C25,Zones!$A$5:$A$14,0)),0))</f>
@@ -6431,7 +6491,7 @@
       </c>
       <c r="G25" s="22" t="n">
         <f aca="false">E25*F25</f>
-        <v>13.2</v>
+        <v>49.98</v>
       </c>
       <c r="H25" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A25,Portes!$H$5:$H$23)</f>
@@ -6443,7 +6503,7 @@
       </c>
       <c r="J25" s="22" t="n">
         <f aca="false">MAX(0,G25-H25)</f>
-        <v>13.2</v>
+        <v>49.98</v>
       </c>
       <c r="K25" s="18" t="n">
         <f aca="false">IF(I25="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B25,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C25,Hypothèses!$A$38:$A$53,0))),0)</f>
@@ -6467,7 +6527,7 @@
       </c>
       <c r="P25" s="24" t="n">
         <f aca="false">L25*J25*MAX(0,M25-N25)</f>
-        <v>72.6</v>
+        <v>274.89</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6475,16 +6535,16 @@
         <v>214</v>
       </c>
       <c r="B26" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="C26" s="14" t="s">
         <v>99</v>
-      </c>
-      <c r="C26" s="14" t="s">
-        <v>63</v>
       </c>
       <c r="D26" s="14" t="s">
         <v>215</v>
       </c>
       <c r="E26" s="21" t="n">
-        <v>8.4</v>
+        <v>3.93</v>
       </c>
       <c r="F26" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B26,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C26,Zones!$A$5:$A$14,0)),0))</f>
@@ -6492,7 +6552,7 @@
       </c>
       <c r="G26" s="22" t="n">
         <f aca="false">E26*F26</f>
-        <v>50.4</v>
+        <v>23.58</v>
       </c>
       <c r="H26" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A26,Portes!$H$5:$H$23)</f>
@@ -6504,7 +6564,7 @@
       </c>
       <c r="J26" s="22" t="n">
         <f aca="false">MAX(0,G26-H26)</f>
-        <v>50.4</v>
+        <v>23.58</v>
       </c>
       <c r="K26" s="18" t="n">
         <f aca="false">IF(I26="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B26,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C26,Hypothèses!$A$38:$A$53,0))),0)</f>
@@ -6516,36 +6576,36 @@
       </c>
       <c r="M26" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B26,Hypothèses!$A$38:$A$53,0))</f>
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="N26" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C26,Hypothèses!$A$38:$A$53,0))</f>
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="O26" s="24" t="n">
         <f aca="false">L26*J26*MAX(0,N26-M26)</f>
-        <v>415.8</v>
+        <v>0</v>
       </c>
       <c r="P26" s="24" t="n">
         <f aca="false">L26*J26*MAX(0,M26-N26)</f>
-        <v>0</v>
+        <v>129.69</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="s">
-        <v>136</v>
+        <v>216</v>
       </c>
       <c r="B27" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="C27" s="14" t="s">
         <v>99</v>
       </c>
-      <c r="C27" s="14" t="s">
-        <v>103</v>
-      </c>
       <c r="D27" s="14" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E27" s="21" t="n">
-        <v>9.985</v>
+        <v>2.2</v>
       </c>
       <c r="F27" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B27,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C27,Zones!$A$5:$A$14,0)),0))</f>
@@ -6553,11 +6613,11 @@
       </c>
       <c r="G27" s="22" t="n">
         <f aca="false">E27*F27</f>
-        <v>59.91</v>
+        <v>13.2</v>
       </c>
       <c r="H27" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A27,Portes!$H$5:$H$23)</f>
-        <v>2.94</v>
+        <v>0</v>
       </c>
       <c r="I27" s="14" t="str">
         <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B27,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C27,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
@@ -6565,7 +6625,7 @@
       </c>
       <c r="J27" s="22" t="n">
         <f aca="false">MAX(0,G27-H27)</f>
-        <v>56.97</v>
+        <v>13.2</v>
       </c>
       <c r="K27" s="18" t="n">
         <f aca="false">IF(I27="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B27,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C27,Hypothèses!$A$38:$A$53,0))),0)</f>
@@ -6577,36 +6637,36 @@
       </c>
       <c r="M27" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B27,Hypothèses!$A$38:$A$53,0))</f>
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="N27" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C27,Hypothèses!$A$38:$A$53,0))</f>
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="O27" s="24" t="n">
         <f aca="false">L27*J27*MAX(0,N27-M27)</f>
-        <v>313.335</v>
+        <v>0</v>
       </c>
       <c r="P27" s="24" t="n">
         <f aca="false">L27*J27*MAX(0,M27-N27)</f>
-        <v>0</v>
+        <v>72.6</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="20" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>103</v>
+        <v>63</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E28" s="21" t="n">
-        <v>10.43</v>
+        <v>8.4</v>
       </c>
       <c r="F28" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B28,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C28,Zones!$A$5:$A$14,0)),0))</f>
@@ -6614,7 +6674,7 @@
       </c>
       <c r="G28" s="22" t="n">
         <f aca="false">E28*F28</f>
-        <v>62.58</v>
+        <v>50.4</v>
       </c>
       <c r="H28" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A28,Portes!$H$5:$H$23)</f>
@@ -6626,27 +6686,27 @@
       </c>
       <c r="J28" s="22" t="n">
         <f aca="false">MAX(0,G28-H28)</f>
-        <v>62.58</v>
+        <v>50.4</v>
       </c>
       <c r="K28" s="18" t="n">
         <f aca="false">IF(I28="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B28,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C28,Hypothèses!$A$38:$A$53,0))),0)</f>
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="L28" s="32" t="n">
         <f aca="false">IF(K28&gt;0,Hypothèses!$B$4/(K28/1000),0)</f>
-        <v>0.366666666666667</v>
+        <v>0.275</v>
       </c>
       <c r="M28" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B28,Hypothèses!$A$38:$A$53,0))</f>
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="N28" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C28,Hypothèses!$A$38:$A$53,0))</f>
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O28" s="24" t="n">
         <f aca="false">L28*J28*MAX(0,N28-M28)</f>
-        <v>0</v>
+        <v>415.8</v>
       </c>
       <c r="P28" s="24" t="n">
         <f aca="false">L28*J28*MAX(0,M28-N28)</f>
@@ -6655,10 +6715,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="20" t="s">
-        <v>219</v>
+        <v>136</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>69</v>
+        <v>99</v>
       </c>
       <c r="C29" s="14" t="s">
         <v>103</v>
@@ -6667,7 +6727,7 @@
         <v>220</v>
       </c>
       <c r="E29" s="21" t="n">
-        <v>3.93</v>
+        <v>9.985</v>
       </c>
       <c r="F29" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B29,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C29,Zones!$A$5:$A$14,0)),0))</f>
@@ -6675,11 +6735,11 @@
       </c>
       <c r="G29" s="22" t="n">
         <f aca="false">E29*F29</f>
-        <v>23.58</v>
+        <v>59.91</v>
       </c>
       <c r="H29" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A29,Portes!$H$5:$H$23)</f>
-        <v>0</v>
+        <v>2.94</v>
       </c>
       <c r="I29" s="14" t="str">
         <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B29,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C29,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
@@ -6687,19 +6747,19 @@
       </c>
       <c r="J29" s="22" t="n">
         <f aca="false">MAX(0,G29-H29)</f>
-        <v>23.58</v>
+        <v>56.97</v>
       </c>
       <c r="K29" s="18" t="n">
         <f aca="false">IF(I29="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B29,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C29,Hypothèses!$A$38:$A$53,0))),0)</f>
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="L29" s="32" t="n">
         <f aca="false">IF(K29&gt;0,Hypothèses!$B$4/(K29/1000),0)</f>
-        <v>0.366666666666667</v>
+        <v>0.275</v>
       </c>
       <c r="M29" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B29,Hypothèses!$A$38:$A$53,0))</f>
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="N29" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C29,Hypothèses!$A$38:$A$53,0))</f>
@@ -6707,7 +6767,7 @@
       </c>
       <c r="O29" s="24" t="n">
         <f aca="false">L29*J29*MAX(0,N29-M29)</f>
-        <v>0</v>
+        <v>313.335</v>
       </c>
       <c r="P29" s="24" t="n">
         <f aca="false">L29*J29*MAX(0,M29-N29)</f>
@@ -6719,16 +6779,16 @@
         <v>221</v>
       </c>
       <c r="B30" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="C30" s="14" t="s">
         <v>103</v>
-      </c>
-      <c r="C30" s="14" t="s">
-        <v>63</v>
       </c>
       <c r="D30" s="14" t="s">
         <v>222</v>
       </c>
       <c r="E30" s="21" t="n">
-        <v>2.8</v>
+        <v>10.43</v>
       </c>
       <c r="F30" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B30,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C30,Zones!$A$5:$A$14,0)),0))</f>
@@ -6736,7 +6796,7 @@
       </c>
       <c r="G30" s="22" t="n">
         <f aca="false">E30*F30</f>
-        <v>16.8</v>
+        <v>62.58</v>
       </c>
       <c r="H30" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A30,Portes!$H$5:$H$23)</f>
@@ -6748,7 +6808,7 @@
       </c>
       <c r="J30" s="22" t="n">
         <f aca="false">MAX(0,G30-H30)</f>
-        <v>16.8</v>
+        <v>62.58</v>
       </c>
       <c r="K30" s="18" t="n">
         <f aca="false">IF(I30="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B30,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C30,Hypothèses!$A$38:$A$53,0))),0)</f>
@@ -6764,11 +6824,11 @@
       </c>
       <c r="N30" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C30,Hypothèses!$A$38:$A$53,0))</f>
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O30" s="24" t="n">
         <f aca="false">L30*J30*MAX(0,N30-M30)</f>
-        <v>61.6</v>
+        <v>0</v>
       </c>
       <c r="P30" s="24" t="n">
         <f aca="false">L30*J30*MAX(0,M30-N30)</f>
@@ -6780,16 +6840,16 @@
         <v>223</v>
       </c>
       <c r="B31" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="C31" s="14" t="s">
         <v>103</v>
-      </c>
-      <c r="C31" s="14" t="s">
-        <v>63</v>
       </c>
       <c r="D31" s="14" t="s">
         <v>224</v>
       </c>
       <c r="E31" s="21" t="n">
-        <v>2.8</v>
+        <v>3.93</v>
       </c>
       <c r="F31" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B31,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C31,Zones!$A$5:$A$14,0)),0))</f>
@@ -6797,7 +6857,7 @@
       </c>
       <c r="G31" s="22" t="n">
         <f aca="false">E31*F31</f>
-        <v>16.8</v>
+        <v>23.58</v>
       </c>
       <c r="H31" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A31,Portes!$H$5:$H$23)</f>
@@ -6809,7 +6869,7 @@
       </c>
       <c r="J31" s="22" t="n">
         <f aca="false">MAX(0,G31-H31)</f>
-        <v>16.8</v>
+        <v>23.58</v>
       </c>
       <c r="K31" s="18" t="n">
         <f aca="false">IF(I31="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B31,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C31,Hypothèses!$A$38:$A$53,0))),0)</f>
@@ -6825,11 +6885,11 @@
       </c>
       <c r="N31" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C31,Hypothèses!$A$38:$A$53,0))</f>
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O31" s="24" t="n">
         <f aca="false">L31*J31*MAX(0,N31-M31)</f>
-        <v>61.6</v>
+        <v>0</v>
       </c>
       <c r="P31" s="24" t="n">
         <f aca="false">L31*J31*MAX(0,M31-N31)</f>
@@ -6838,16 +6898,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="20" t="s">
-        <v>138</v>
+        <v>225</v>
       </c>
       <c r="B32" s="14" t="s">
         <v>103</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>103</v>
+        <v>63</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E32" s="21" t="n">
         <v>2.8</v>
@@ -6862,7 +6922,7 @@
       </c>
       <c r="H32" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A32,Portes!$H$5:$H$23)</f>
-        <v>2.94</v>
+        <v>0</v>
       </c>
       <c r="I32" s="14" t="str">
         <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B32,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C32,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
@@ -6870,7 +6930,7 @@
       </c>
       <c r="J32" s="22" t="n">
         <f aca="false">MAX(0,G32-H32)</f>
-        <v>13.86</v>
+        <v>16.8</v>
       </c>
       <c r="K32" s="18" t="n">
         <f aca="false">IF(I32="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B32,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C32,Hypothèses!$A$38:$A$53,0))),0)</f>
@@ -6886,11 +6946,11 @@
       </c>
       <c r="N32" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C32,Hypothèses!$A$38:$A$53,0))</f>
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O32" s="24" t="n">
         <f aca="false">L32*J32*MAX(0,N32-M32)</f>
-        <v>0</v>
+        <v>61.6</v>
       </c>
       <c r="P32" s="24" t="n">
         <f aca="false">L32*J32*MAX(0,M32-N32)</f>
@@ -6899,19 +6959,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="20" t="s">
-        <v>141</v>
+        <v>227</v>
       </c>
       <c r="B33" s="14" t="s">
         <v>103</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>106</v>
+        <v>63</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="E33" s="21" t="n">
-        <v>19.34</v>
+        <v>2.8</v>
       </c>
       <c r="F33" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B33,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C33,Zones!$A$5:$A$14,0)),0))</f>
@@ -6919,11 +6979,11 @@
       </c>
       <c r="G33" s="22" t="n">
         <f aca="false">E33*F33</f>
-        <v>116.04</v>
+        <v>16.8</v>
       </c>
       <c r="H33" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A33,Portes!$H$5:$H$23)</f>
-        <v>5.88</v>
+        <v>0</v>
       </c>
       <c r="I33" s="14" t="str">
         <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B33,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C33,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
@@ -6931,15 +6991,15 @@
       </c>
       <c r="J33" s="22" t="n">
         <f aca="false">MAX(0,G33-H33)</f>
-        <v>110.16</v>
+        <v>16.8</v>
       </c>
       <c r="K33" s="18" t="n">
         <f aca="false">IF(I33="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B33,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C33,Hypothèses!$A$38:$A$53,0))),0)</f>
-        <v>150</v>
+        <v>60</v>
       </c>
       <c r="L33" s="32" t="n">
         <f aca="false">IF(K33&gt;0,Hypothèses!$B$4/(K33/1000),0)</f>
-        <v>0.146666666666667</v>
+        <v>0.366666666666667</v>
       </c>
       <c r="M33" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B33,Hypothèses!$A$38:$A$53,0))</f>
@@ -6947,32 +7007,32 @@
       </c>
       <c r="N33" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C33,Hypothèses!$A$38:$A$53,0))</f>
-        <v>-20</v>
+        <v>40</v>
       </c>
       <c r="O33" s="24" t="n">
         <f aca="false">L33*J33*MAX(0,N33-M33)</f>
-        <v>0</v>
+        <v>61.6</v>
       </c>
       <c r="P33" s="24" t="n">
         <f aca="false">L33*J33*MAX(0,M33-N33)</f>
-        <v>807.84</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="20" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="B34" s="14" t="s">
         <v>103</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="E34" s="21" t="n">
-        <v>5</v>
+        <v>2.8</v>
       </c>
       <c r="F34" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B34,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C34,Zones!$A$5:$A$14,0)),0))</f>
@@ -6980,7 +7040,7 @@
       </c>
       <c r="G34" s="22" t="n">
         <f aca="false">E34*F34</f>
-        <v>30</v>
+        <v>16.8</v>
       </c>
       <c r="H34" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A34,Portes!$H$5:$H$23)</f>
@@ -6992,15 +7052,15 @@
       </c>
       <c r="J34" s="22" t="n">
         <f aca="false">MAX(0,G34-H34)</f>
-        <v>27.06</v>
+        <v>13.86</v>
       </c>
       <c r="K34" s="18" t="n">
         <f aca="false">IF(I34="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B34,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C34,Hypothèses!$A$38:$A$53,0))),0)</f>
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="L34" s="32" t="n">
         <f aca="false">IF(K34&gt;0,Hypothèses!$B$4/(K34/1000),0)</f>
-        <v>0.22</v>
+        <v>0.366666666666667</v>
       </c>
       <c r="M34" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B34,Hypothèses!$A$38:$A$53,0))</f>
@@ -7008,7 +7068,7 @@
       </c>
       <c r="N34" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C34,Hypothèses!$A$38:$A$53,0))</f>
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="O34" s="24" t="n">
         <f aca="false">L34*J34*MAX(0,N34-M34)</f>
@@ -7016,24 +7076,24 @@
       </c>
       <c r="P34" s="24" t="n">
         <f aca="false">L34*J34*MAX(0,M34-N34)</f>
-        <v>166.6896</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="20" t="s">
-        <v>228</v>
+        <v>141</v>
       </c>
       <c r="B35" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="C35" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="C35" s="14" t="s">
-        <v>109</v>
-      </c>
       <c r="D35" s="14" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E35" s="21" t="n">
-        <v>15.01</v>
+        <v>19.34</v>
       </c>
       <c r="F35" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B35,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C35,Zones!$A$5:$A$14,0)),0))</f>
@@ -7041,11 +7101,11 @@
       </c>
       <c r="G35" s="22" t="n">
         <f aca="false">E35*F35</f>
-        <v>90.06</v>
+        <v>116.04</v>
       </c>
       <c r="H35" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A35,Portes!$H$5:$H$23)</f>
-        <v>0</v>
+        <v>5.88</v>
       </c>
       <c r="I35" s="14" t="str">
         <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B35,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C35,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
@@ -7053,7 +7113,7 @@
       </c>
       <c r="J35" s="22" t="n">
         <f aca="false">MAX(0,G35-H35)</f>
-        <v>90.06</v>
+        <v>110.16</v>
       </c>
       <c r="K35" s="18" t="n">
         <f aca="false">IF(I35="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B35,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C35,Hypothèses!$A$38:$A$53,0))),0)</f>
@@ -7065,36 +7125,36 @@
       </c>
       <c r="M35" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B35,Hypothèses!$A$38:$A$53,0))</f>
-        <v>-20</v>
+        <v>30</v>
       </c>
       <c r="N35" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C35,Hypothèses!$A$38:$A$53,0))</f>
-        <v>2</v>
+        <v>-20</v>
       </c>
       <c r="O35" s="24" t="n">
         <f aca="false">L35*J35*MAX(0,N35-M35)</f>
-        <v>290.5936</v>
+        <v>0</v>
       </c>
       <c r="P35" s="24" t="n">
         <f aca="false">L35*J35*MAX(0,M35-N35)</f>
-        <v>0</v>
+        <v>807.84</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="20" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="B36" s="14" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>63</v>
+        <v>109</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E36" s="21" t="n">
-        <v>15.01</v>
+        <v>5</v>
       </c>
       <c r="F36" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B36,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C36,Zones!$A$5:$A$14,0)),0))</f>
@@ -7102,11 +7162,11 @@
       </c>
       <c r="G36" s="22" t="n">
         <f aca="false">E36*F36</f>
-        <v>90.06</v>
+        <v>30</v>
       </c>
       <c r="H36" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A36,Portes!$H$5:$H$23)</f>
-        <v>8.4</v>
+        <v>2.94</v>
       </c>
       <c r="I36" s="14" t="str">
         <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B36,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C36,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
@@ -7114,48 +7174,48 @@
       </c>
       <c r="J36" s="22" t="n">
         <f aca="false">MAX(0,G36-H36)</f>
-        <v>81.66</v>
+        <v>27.06</v>
       </c>
       <c r="K36" s="18" t="n">
         <f aca="false">IF(I36="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B36,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C36,Hypothèses!$A$38:$A$53,0))),0)</f>
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="L36" s="32" t="n">
         <f aca="false">IF(K36&gt;0,Hypothèses!$B$4/(K36/1000),0)</f>
-        <v>0.146666666666667</v>
+        <v>0.22</v>
       </c>
       <c r="M36" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B36,Hypothèses!$A$38:$A$53,0))</f>
-        <v>-20</v>
+        <v>30</v>
       </c>
       <c r="N36" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C36,Hypothèses!$A$38:$A$53,0))</f>
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="O36" s="24" t="n">
         <f aca="false">L36*J36*MAX(0,N36-M36)</f>
-        <v>718.608</v>
+        <v>0</v>
       </c>
       <c r="P36" s="24" t="n">
         <f aca="false">L36*J36*MAX(0,M36-N36)</f>
-        <v>0</v>
+        <v>166.6896</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="20" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B37" s="14" t="s">
         <v>106</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>68</v>
+        <v>109</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E37" s="21" t="n">
-        <v>19.34</v>
+        <v>15.01</v>
       </c>
       <c r="F37" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B37,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C37,Zones!$A$5:$A$14,0)),0))</f>
@@ -7163,7 +7223,7 @@
       </c>
       <c r="G37" s="22" t="n">
         <f aca="false">E37*F37</f>
-        <v>116.04</v>
+        <v>90.06</v>
       </c>
       <c r="H37" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A37,Portes!$H$5:$H$23)</f>
@@ -7175,7 +7235,7 @@
       </c>
       <c r="J37" s="22" t="n">
         <f aca="false">MAX(0,G37-H37)</f>
-        <v>116.04</v>
+        <v>90.06</v>
       </c>
       <c r="K37" s="18" t="n">
         <f aca="false">IF(I37="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B37,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C37,Hypothèses!$A$38:$A$53,0))),0)</f>
@@ -7191,11 +7251,11 @@
       </c>
       <c r="N37" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C37,Hypothèses!$A$38:$A$53,0))</f>
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="O37" s="24" t="n">
         <f aca="false">L37*J37*MAX(0,N37-M37)</f>
-        <v>765.864</v>
+        <v>290.5936</v>
       </c>
       <c r="P37" s="24" t="n">
         <f aca="false">L37*J37*MAX(0,M37-N37)</f>
@@ -7204,19 +7264,19 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="20" t="s">
-        <v>233</v>
+        <v>158</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="D38" s="14" t="s">
         <v>234</v>
       </c>
       <c r="E38" s="21" t="n">
-        <v>5</v>
+        <v>15.01</v>
       </c>
       <c r="F38" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B38,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C38,Zones!$A$5:$A$14,0)),0))</f>
@@ -7224,11 +7284,11 @@
       </c>
       <c r="G38" s="22" t="n">
         <f aca="false">E38*F38</f>
-        <v>30</v>
+        <v>90.06</v>
       </c>
       <c r="H38" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A38,Portes!$H$5:$H$23)</f>
-        <v>0</v>
+        <v>8.4</v>
       </c>
       <c r="I38" s="14" t="str">
         <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B38,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C38,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
@@ -7236,27 +7296,27 @@
       </c>
       <c r="J38" s="22" t="n">
         <f aca="false">MAX(0,G38-H38)</f>
-        <v>30</v>
+        <v>81.66</v>
       </c>
       <c r="K38" s="18" t="n">
         <f aca="false">IF(I38="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B38,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C38,Hypothèses!$A$38:$A$53,0))),0)</f>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="L38" s="32" t="n">
         <f aca="false">IF(K38&gt;0,Hypothèses!$B$4/(K38/1000),0)</f>
-        <v>0.22</v>
+        <v>0.146666666666667</v>
       </c>
       <c r="M38" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B38,Hypothèses!$A$38:$A$53,0))</f>
-        <v>2</v>
+        <v>-20</v>
       </c>
       <c r="N38" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C38,Hypothèses!$A$38:$A$53,0))</f>
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="O38" s="24" t="n">
         <f aca="false">L38*J38*MAX(0,N38-M38)</f>
-        <v>151.8</v>
+        <v>718.608</v>
       </c>
       <c r="P38" s="24" t="n">
         <f aca="false">L38*J38*MAX(0,M38-N38)</f>
@@ -7268,16 +7328,16 @@
         <v>235</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="D39" s="14" t="s">
         <v>236</v>
       </c>
       <c r="E39" s="21" t="n">
-        <v>15.01</v>
+        <v>19.34</v>
       </c>
       <c r="F39" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B39,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C39,Zones!$A$5:$A$14,0)),0))</f>
@@ -7285,7 +7345,7 @@
       </c>
       <c r="G39" s="22" t="n">
         <f aca="false">E39*F39</f>
-        <v>90.06</v>
+        <v>116.04</v>
       </c>
       <c r="H39" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A39,Portes!$H$5:$H$23)</f>
@@ -7297,27 +7357,27 @@
       </c>
       <c r="J39" s="22" t="n">
         <f aca="false">MAX(0,G39-H39)</f>
-        <v>90.06</v>
+        <v>116.04</v>
       </c>
       <c r="K39" s="18" t="n">
         <f aca="false">IF(I39="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B39,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C39,Hypothèses!$A$38:$A$53,0))),0)</f>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="L39" s="32" t="n">
         <f aca="false">IF(K39&gt;0,Hypothèses!$B$4/(K39/1000),0)</f>
-        <v>0.22</v>
+        <v>0.146666666666667</v>
       </c>
       <c r="M39" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B39,Hypothèses!$A$38:$A$53,0))</f>
-        <v>2</v>
+        <v>-20</v>
       </c>
       <c r="N39" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C39,Hypothèses!$A$38:$A$53,0))</f>
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="O39" s="24" t="n">
         <f aca="false">L39*J39*MAX(0,N39-M39)</f>
-        <v>752.9016</v>
+        <v>765.864</v>
       </c>
       <c r="P39" s="24" t="n">
         <f aca="false">L39*J39*MAX(0,M39-N39)</f>
@@ -7326,19 +7386,19 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="20" t="s">
-        <v>148</v>
+        <v>237</v>
       </c>
       <c r="B40" s="14" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="D40" s="14" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E40" s="21" t="n">
-        <v>49.5</v>
+        <v>5</v>
       </c>
       <c r="F40" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B40,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C40,Zones!$A$5:$A$14,0)),0))</f>
@@ -7346,39 +7406,39 @@
       </c>
       <c r="G40" s="22" t="n">
         <f aca="false">E40*F40</f>
-        <v>297</v>
+        <v>30</v>
       </c>
       <c r="H40" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A40,Portes!$H$5:$H$23)</f>
-        <v>5.88</v>
+        <v>0</v>
       </c>
       <c r="I40" s="14" t="str">
         <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B40,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C40,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
-        <v>Non</v>
+        <v>Oui</v>
       </c>
       <c r="J40" s="22" t="n">
         <f aca="false">MAX(0,G40-H40)</f>
-        <v>291.12</v>
+        <v>30</v>
       </c>
       <c r="K40" s="18" t="n">
         <f aca="false">IF(I40="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B40,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C40,Hypothèses!$A$38:$A$53,0))),0)</f>
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="L40" s="32" t="n">
         <f aca="false">IF(K40&gt;0,Hypothèses!$B$4/(K40/1000),0)</f>
-        <v>0</v>
+        <v>0.22</v>
       </c>
       <c r="M40" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B40,Hypothèses!$A$38:$A$53,0))</f>
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="N40" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C40,Hypothèses!$A$38:$A$53,0))</f>
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="O40" s="24" t="n">
         <f aca="false">L40*J40*MAX(0,N40-M40)</f>
-        <v>0</v>
+        <v>151.8</v>
       </c>
       <c r="P40" s="24" t="n">
         <f aca="false">L40*J40*MAX(0,M40-N40)</f>
@@ -7387,19 +7447,19 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="20" t="s">
-        <v>153</v>
+        <v>239</v>
       </c>
       <c r="B41" s="14" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>111</v>
+        <v>63</v>
       </c>
       <c r="D41" s="14" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E41" s="21" t="n">
-        <v>17.6</v>
+        <v>15.01</v>
       </c>
       <c r="F41" s="23" t="n">
         <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B41,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C41,Zones!$A$5:$A$14,0)),0))</f>
@@ -7407,39 +7467,39 @@
       </c>
       <c r="G41" s="22" t="n">
         <f aca="false">E41*F41</f>
-        <v>105.6</v>
+        <v>90.06</v>
       </c>
       <c r="H41" s="22" t="n">
         <f aca="false">SUMIF(Portes!$D$5:$D$23,A41,Portes!$H$5:$H$23)</f>
-        <v>5.88</v>
+        <v>0</v>
       </c>
       <c r="I41" s="14" t="str">
         <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B41,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C41,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
-        <v>Non</v>
+        <v>Oui</v>
       </c>
       <c r="J41" s="22" t="n">
         <f aca="false">MAX(0,G41-H41)</f>
-        <v>99.72</v>
+        <v>90.06</v>
       </c>
       <c r="K41" s="18" t="n">
         <f aca="false">IF(I41="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B41,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C41,Hypothèses!$A$38:$A$53,0))),0)</f>
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="L41" s="32" t="n">
         <f aca="false">IF(K41&gt;0,Hypothèses!$B$4/(K41/1000),0)</f>
-        <v>0</v>
+        <v>0.22</v>
       </c>
       <c r="M41" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B41,Hypothèses!$A$38:$A$53,0))</f>
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="N41" s="18" t="n">
         <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C41,Hypothèses!$A$38:$A$53,0))</f>
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O41" s="24" t="n">
         <f aca="false">L41*J41*MAX(0,N41-M41)</f>
-        <v>0</v>
+        <v>752.9016</v>
       </c>
       <c r="P41" s="24" t="n">
         <f aca="false">L41*J41*MAX(0,M41-N41)</f>
@@ -7447,29 +7507,151 @@
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D42" s="28" t="s">
+      <c r="A42" s="20" t="s">
+        <v>148</v>
+      </c>
+      <c r="B42" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="C42" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="D42" s="14" t="s">
+        <v>241</v>
+      </c>
+      <c r="E42" s="21" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="F42" s="23" t="n">
+        <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B42,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C42,Zones!$A$5:$A$14,0)),0))</f>
+        <v>6</v>
+      </c>
+      <c r="G42" s="22" t="n">
+        <f aca="false">E42*F42</f>
+        <v>297</v>
+      </c>
+      <c r="H42" s="22" t="n">
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A42,Portes!$H$5:$H$23)</f>
+        <v>5.88</v>
+      </c>
+      <c r="I42" s="14" t="str">
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B42,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C42,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
+        <v>Non</v>
+      </c>
+      <c r="J42" s="22" t="n">
+        <f aca="false">MAX(0,G42-H42)</f>
+        <v>291.12</v>
+      </c>
+      <c r="K42" s="18" t="n">
+        <f aca="false">IF(I42="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B42,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C42,Hypothèses!$A$38:$A$53,0))),0)</f>
+        <v>0</v>
+      </c>
+      <c r="L42" s="32" t="n">
+        <f aca="false">IF(K42&gt;0,Hypothèses!$B$4/(K42/1000),0)</f>
+        <v>0</v>
+      </c>
+      <c r="M42" s="18" t="n">
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B42,Hypothèses!$A$38:$A$53,0))</f>
+        <v>30</v>
+      </c>
+      <c r="N42" s="18" t="n">
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C42,Hypothèses!$A$38:$A$53,0))</f>
+        <v>40</v>
+      </c>
+      <c r="O42" s="24" t="n">
+        <f aca="false">L42*J42*MAX(0,N42-M42)</f>
+        <v>0</v>
+      </c>
+      <c r="P42" s="24" t="n">
+        <f aca="false">L42*J42*MAX(0,M42-N42)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="20" t="s">
+        <v>153</v>
+      </c>
+      <c r="B43" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="C43" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="D43" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="E43" s="21" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="F43" s="23" t="n">
+        <f aca="false">MAX(IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(B43,Zones!$A$5:$A$14,0)),0),IFERROR(INDEX(Zones!$G$5:$G$14,MATCH(C43,Zones!$A$5:$A$14,0)),0))</f>
+        <v>6</v>
+      </c>
+      <c r="G43" s="22" t="n">
+        <f aca="false">E43*F43</f>
+        <v>105.6</v>
+      </c>
+      <c r="H43" s="22" t="n">
+        <f aca="false">SUMIF(Portes!$D$5:$D$23,A43,Portes!$H$5:$H$23)</f>
+        <v>5.88</v>
+      </c>
+      <c r="I43" s="14" t="str">
+        <f aca="false">IF(OR(INDEX(Hypothèses!$D$38:$D$53,MATCH(B43,Hypothèses!$A$38:$A$53,0))="Oui",INDEX(Hypothèses!$D$38:$D$53,MATCH(C43,Hypothèses!$A$38:$A$53,0))="Oui"),"Oui","Non")</f>
+        <v>Non</v>
+      </c>
+      <c r="J43" s="22" t="n">
+        <f aca="false">MAX(0,G43-H43)</f>
+        <v>99.72</v>
+      </c>
+      <c r="K43" s="18" t="n">
+        <f aca="false">IF(I43="Oui",MAX(INDEX(Hypothèses!$C$38:$C$53,MATCH(B43,Hypothèses!$A$38:$A$53,0)),INDEX(Hypothèses!$C$38:$C$53,MATCH(C43,Hypothèses!$A$38:$A$53,0))),0)</f>
+        <v>0</v>
+      </c>
+      <c r="L43" s="32" t="n">
+        <f aca="false">IF(K43&gt;0,Hypothèses!$B$4/(K43/1000),0)</f>
+        <v>0</v>
+      </c>
+      <c r="M43" s="18" t="n">
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(B43,Hypothèses!$A$38:$A$53,0))</f>
+        <v>30</v>
+      </c>
+      <c r="N43" s="18" t="n">
+        <f aca="false">INDEX(Hypothèses!$B$38:$B$53,MATCH(C43,Hypothèses!$A$38:$A$53,0))</f>
+        <v>30</v>
+      </c>
+      <c r="O43" s="24" t="n">
+        <f aca="false">L43*J43*MAX(0,N43-M43)</f>
+        <v>0</v>
+      </c>
+      <c r="P43" s="24" t="n">
+        <f aca="false">L43*J43*MAX(0,M43-N43)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D44" s="28" t="s">
         <v>114</v>
       </c>
-      <c r="E42" s="29" t="n">
-        <f aca="false">SUM(E5:E41)</f>
-        <v>445.665</v>
-      </c>
-      <c r="G42" s="29" t="n">
-        <f aca="false">SUM(G5:G41)</f>
-        <v>2673.99</v>
-      </c>
-      <c r="H42" s="29" t="n">
-        <f aca="false">SUM(H5:H41)</f>
+      <c r="E44" s="29" t="n">
+        <f aca="false">SUM(E5:E43)</f>
+        <v>451.985</v>
+      </c>
+      <c r="G44" s="29" t="n">
+        <f aca="false">SUM(G5:G43)</f>
+        <v>2711.91</v>
+      </c>
+      <c r="H44" s="29" t="n">
+        <f aca="false">SUM(H5:H43)</f>
         <v>64.19</v>
       </c>
-      <c r="J42" s="29" t="n">
-        <f aca="false">SUM(J5:J41)</f>
-        <v>2609.8</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D44" s="33" t="s">
-        <v>239</v>
+      <c r="J44" s="29" t="n">
+        <f aca="false">SUM(J5:J43)</f>
+        <v>2647.72</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D46" s="33" t="s">
+        <v>243</v>
       </c>
     </row>
   </sheetData>
@@ -7502,12 +7684,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7515,22 +7697,22 @@
         <v>47</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="F4" s="19" t="s">
         <v>48</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7539,7 +7721,7 @@
         <v>150</v>
       </c>
       <c r="B5" s="22" t="n">
-        <f aca="false">SUMIFS(Parois!$J$5:$J$41,Parois!$K$5:$K$41,A5,Parois!$I$5:$I$41,"Oui")</f>
+        <f aca="false">SUMIFS(Parois!$J$5:$J$43,Parois!$K$5:$K$43,A5,Parois!$I$5:$I$43,"Oui")</f>
         <v>397.92</v>
       </c>
       <c r="C5" s="22" t="n">
@@ -7569,7 +7751,7 @@
         <v>100</v>
       </c>
       <c r="B6" s="22" t="n">
-        <f aca="false">SUMIFS(Parois!$J$5:$J$41,Parois!$K$5:$K$41,A6,Parois!$I$5:$I$41,"Oui")</f>
+        <f aca="false">SUMIFS(Parois!$J$5:$J$43,Parois!$K$5:$K$43,A6,Parois!$I$5:$I$43,"Oui")</f>
         <v>147.12</v>
       </c>
       <c r="C6" s="22" t="n">
@@ -7599,7 +7781,7 @@
         <v>80</v>
       </c>
       <c r="B7" s="22" t="n">
-        <f aca="false">SUMIFS(Parois!$J$5:$J$41,Parois!$K$5:$K$41,A7,Parois!$I$5:$I$41,"Oui")</f>
+        <f aca="false">SUMIFS(Parois!$J$5:$J$43,Parois!$K$5:$K$43,A7,Parois!$I$5:$I$43,"Oui")</f>
         <v>349.78</v>
       </c>
       <c r="C7" s="22" t="n">
@@ -7629,20 +7811,20 @@
         <v>60</v>
       </c>
       <c r="B8" s="22" t="n">
-        <f aca="false">SUMIFS(Parois!$J$5:$J$41,Parois!$K$5:$K$41,A8,Parois!$I$5:$I$41,"Oui")</f>
-        <v>1324.14</v>
+        <f aca="false">SUMIFS(Parois!$J$5:$J$43,Parois!$K$5:$K$43,A8,Parois!$I$5:$I$43,"Oui")</f>
+        <v>1362.06</v>
       </c>
       <c r="C8" s="22" t="n">
         <f aca="false">SUMIF(Zones!$L$5:$L$14,A8,Zones!$N$5:$N$14)</f>
-        <v>1052.4412</v>
+        <v>1080.1512</v>
       </c>
       <c r="D8" s="22" t="n">
         <f aca="false">B8+C8</f>
-        <v>2376.5812</v>
+        <v>2442.2112</v>
       </c>
       <c r="E8" s="22" t="n">
         <f aca="false">D8*(1+Hypothèses!$B$9)</f>
-        <v>2495.41026</v>
+        <v>2564.32176</v>
       </c>
       <c r="F8" s="34" t="n">
         <f aca="false">Hypothèses!C25</f>
@@ -7650,7 +7832,7 @@
       </c>
       <c r="G8" s="24" t="n">
         <f aca="false">E8*F8</f>
-        <v>623852.565</v>
+        <v>641080.44</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7659,46 +7841,46 @@
       </c>
       <c r="B9" s="29" t="n">
         <f aca="false">SUM(B5:B8)</f>
-        <v>2218.96</v>
+        <v>2256.88</v>
       </c>
       <c r="C9" s="29" t="n">
         <f aca="false">SUM(C5:C8)</f>
-        <v>1578.2946</v>
+        <v>1606.0046</v>
       </c>
       <c r="D9" s="29" t="n">
         <f aca="false">SUM(D5:D8)</f>
-        <v>3797.2546</v>
+        <v>3862.8846</v>
       </c>
       <c r="E9" s="29" t="n">
         <f aca="false">SUM(E5:E8)</f>
-        <v>3987.11733</v>
+        <v>4056.02883</v>
       </c>
       <c r="G9" s="30" t="n">
         <f aca="false">SUM(G5:G8)</f>
-        <v>1159719.8844</v>
+        <v>1176947.7594</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="G10" s="24" t="n">
         <f aca="false">G9*Hypothèses!$B$10</f>
-        <v>173957.98266</v>
+        <v>176542.16391</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="19" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="C12" s="19" t="s">
         <v>53</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7775,7 +7957,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="28" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="D17" s="30" t="n">
         <f aca="false">SUM(D13:D16)</f>
@@ -7784,7 +7966,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="28" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="B19" s="28"/>
       <c r="C19" s="28"/>
@@ -7793,7 +7975,7 @@
       <c r="F19" s="28"/>
       <c r="G19" s="30" t="n">
         <f aca="false">G9+G10+D17</f>
-        <v>1675677.86706</v>
+        <v>1695489.92331</v>
       </c>
     </row>
   </sheetData>
@@ -7826,12 +8008,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7842,10 +8024,10 @@
         <v>72</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="E4" s="19" t="s">
         <v>75</v>
@@ -7854,73 +8036,73 @@
         <v>78</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="I4" s="19" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="J4" s="19" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="K4" s="19" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="L4" s="19" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="M4" s="19" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="N4" s="19" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="O4" s="19" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="P4" s="19" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="Q4" s="19" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="R4" s="19" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="S4" s="19" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="T4" s="19" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="U4" s="19" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="V4" s="19" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="W4" s="19" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="X4" s="19" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="Y4" s="19" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="Z4" s="19" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="AA4" s="19" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="AB4" s="19" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="AC4" s="19" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7949,7 +8131,7 @@
         <v>1734.7512</v>
       </c>
       <c r="G5" s="24" t="n">
-        <f aca="false">SUMIF(Parois!$B$5:$B$41,A5,Parois!$O$5:$O$41)+SUMIF(Parois!$C$5:$C$41,A5,Parois!$P$5:$P$41)</f>
+        <f aca="false">SUMIF(Parois!$B$5:$B$43,A5,Parois!$O$5:$O$43)+SUMIF(Parois!$C$5:$C$43,A5,Parois!$P$5:$P$43)</f>
         <v>797.94</v>
       </c>
       <c r="H5" s="24" t="n">
@@ -8046,19 +8228,19 @@
       </c>
       <c r="E6" s="35" t="n">
         <f aca="false">Zones!E6</f>
-        <v>145.18</v>
+        <v>213.5</v>
       </c>
       <c r="F6" s="34" t="n">
         <f aca="false">Zones!H6</f>
-        <v>871.08</v>
+        <v>1281</v>
       </c>
       <c r="G6" s="24" t="n">
-        <f aca="false">SUMIF(Parois!$B$5:$B$41,A6,Parois!$O$5:$O$41)+SUMIF(Parois!$C$5:$C$41,A6,Parois!$P$5:$P$41)</f>
-        <v>369.49</v>
+        <f aca="false">SUMIF(Parois!$B$5:$B$43,A6,Parois!$O$5:$O$43)+SUMIF(Parois!$C$5:$C$43,A6,Parois!$P$5:$P$43)</f>
+        <v>457.49</v>
       </c>
       <c r="H6" s="24" t="n">
         <f aca="false">IF(Zones!L6&gt;0,Hypothèses!$B$4/(Zones!L6/1000),0)*Zones!N6*MAX(0,Hypothèses!$B$14-D6)</f>
-        <v>532.326666666667</v>
+        <v>782.833333333333</v>
       </c>
       <c r="I6" s="24" t="n">
         <f aca="false">IF(D6&lt;0,Hypothèses!$B$6,Hypothèses!$B$7)*E6*MAX(0,Hypothèses!$B$15-D6)</f>
@@ -8121,7 +8303,7 @@
       </c>
       <c r="AA6" s="24" t="n">
         <f aca="false">G6+H6+I6+L6+P6+S6+T6+Z6</f>
-        <v>901.816666666667</v>
+        <v>1240.32333333333</v>
       </c>
       <c r="AB6" s="10" t="n">
         <v>18</v>
@@ -8150,19 +8332,19 @@
       </c>
       <c r="E7" s="35" t="n">
         <f aca="false">Zones!E7</f>
-        <v>213.5</v>
+        <v>172.89</v>
       </c>
       <c r="F7" s="34" t="n">
         <f aca="false">Zones!H7</f>
-        <v>1281</v>
+        <v>1037.34</v>
       </c>
       <c r="G7" s="24" t="n">
-        <f aca="false">SUMIF(Parois!$B$5:$B$41,A7,Parois!$O$5:$O$41)+SUMIF(Parois!$C$5:$C$41,A7,Parois!$P$5:$P$41)</f>
-        <v>137.5</v>
+        <f aca="false">SUMIF(Parois!$B$5:$B$43,A7,Parois!$O$5:$O$43)+SUMIF(Parois!$C$5:$C$43,A7,Parois!$P$5:$P$43)</f>
+        <v>93.5</v>
       </c>
       <c r="H7" s="24" t="n">
         <f aca="false">IF(Zones!L7&gt;0,Hypothèses!$B$4/(Zones!L7/1000),0)*Zones!N7*MAX(0,Hypothèses!$B$14-D7)</f>
-        <v>391.416666666667</v>
+        <v>316.965</v>
       </c>
       <c r="I7" s="24" t="n">
         <f aca="false">IF(D7&lt;0,Hypothèses!$B$6,Hypothèses!$B$7)*E7*MAX(0,Hypothèses!$B$15-D7)</f>
@@ -8225,7 +8407,7 @@
       </c>
       <c r="AA7" s="24" t="n">
         <f aca="false">G7+H7+I7+L7+P7+S7+T7+Z7</f>
-        <v>528.916666666667</v>
+        <v>410.465</v>
       </c>
       <c r="AB7" s="10" t="n">
         <v>18</v>
@@ -8261,7 +8443,7 @@
         <v>831.006</v>
       </c>
       <c r="G8" s="24" t="n">
-        <f aca="false">SUMIF(Parois!$B$5:$B$41,A8,Parois!$O$5:$O$41)+SUMIF(Parois!$C$5:$C$41,A8,Parois!$P$5:$P$41)</f>
+        <f aca="false">SUMIF(Parois!$B$5:$B$43,A8,Parois!$O$5:$O$43)+SUMIF(Parois!$C$5:$C$43,A8,Parois!$P$5:$P$43)</f>
         <v>212.41</v>
       </c>
       <c r="H8" s="24" t="n">
@@ -8365,7 +8547,7 @@
         <v>1186.218</v>
       </c>
       <c r="G9" s="24" t="n">
-        <f aca="false">SUMIF(Parois!$B$5:$B$41,A9,Parois!$O$5:$O$41)+SUMIF(Parois!$C$5:$C$41,A9,Parois!$P$5:$P$41)</f>
+        <f aca="false">SUMIF(Parois!$B$5:$B$43,A9,Parois!$O$5:$O$43)+SUMIF(Parois!$C$5:$C$43,A9,Parois!$P$5:$P$43)</f>
         <v>217.8</v>
       </c>
       <c r="H9" s="24" t="n">
@@ -8469,7 +8651,7 @@
         <v>963.06</v>
       </c>
       <c r="G10" s="24" t="n">
-        <f aca="false">SUMIF(Parois!$B$5:$B$41,A10,Parois!$O$5:$O$41)+SUMIF(Parois!$C$5:$C$41,A10,Parois!$P$5:$P$41)</f>
+        <f aca="false">SUMIF(Parois!$B$5:$B$43,A10,Parois!$O$5:$O$43)+SUMIF(Parois!$C$5:$C$43,A10,Parois!$P$5:$P$43)</f>
         <v>2133.02375</v>
       </c>
       <c r="H10" s="24" t="n">
@@ -8573,7 +8755,7 @@
         <v>410.592</v>
       </c>
       <c r="G11" s="24" t="n">
-        <f aca="false">SUMIF(Parois!$B$5:$B$41,A11,Parois!$O$5:$O$41)+SUMIF(Parois!$C$5:$C$41,A11,Parois!$P$5:$P$41)</f>
+        <f aca="false">SUMIF(Parois!$B$5:$B$43,A11,Parois!$O$5:$O$43)+SUMIF(Parois!$C$5:$C$43,A11,Parois!$P$5:$P$43)</f>
         <v>123.2</v>
       </c>
       <c r="H11" s="24" t="n">
@@ -8677,7 +8859,7 @@
         <v>1741.7604</v>
       </c>
       <c r="G12" s="24" t="n">
-        <f aca="false">SUMIF(Parois!$B$5:$B$41,A12,Parois!$O$5:$O$41)+SUMIF(Parois!$C$5:$C$41,A12,Parois!$P$5:$P$41)</f>
+        <f aca="false">SUMIF(Parois!$B$5:$B$43,A12,Parois!$O$5:$O$43)+SUMIF(Parois!$C$5:$C$43,A12,Parois!$P$5:$P$43)</f>
         <v>2582.9056</v>
       </c>
       <c r="H12" s="24" t="n">
@@ -8781,7 +8963,7 @@
         <v>450.3</v>
       </c>
       <c r="G13" s="24" t="n">
-        <f aca="false">SUMIF(Parois!$B$5:$B$41,A13,Parois!$O$5:$O$41)+SUMIF(Parois!$C$5:$C$41,A13,Parois!$P$5:$P$41)</f>
+        <f aca="false">SUMIF(Parois!$B$5:$B$43,A13,Parois!$O$5:$O$43)+SUMIF(Parois!$C$5:$C$43,A13,Parois!$P$5:$P$43)</f>
         <v>1071.3912</v>
       </c>
       <c r="H13" s="24" t="n">
@@ -8878,15 +9060,15 @@
       </c>
       <c r="E14" s="35" t="n">
         <f aca="false">Zones!E14</f>
-        <v>314.48</v>
+        <v>286.11</v>
       </c>
       <c r="F14" s="34" t="n">
         <f aca="false">Zones!H14</f>
-        <v>1886.88</v>
+        <v>1716.66</v>
       </c>
       <c r="G14" s="24" t="n">
-        <f aca="false">SUMIF(Parois!$B$5:$B$41,A14,Parois!$O$5:$O$41)+SUMIF(Parois!$C$5:$C$41,A14,Parois!$P$5:$P$41)</f>
-        <v>137.5</v>
+        <f aca="false">SUMIF(Parois!$B$5:$B$43,A14,Parois!$O$5:$O$43)+SUMIF(Parois!$C$5:$C$43,A14,Parois!$P$5:$P$43)</f>
+        <v>163.02</v>
       </c>
       <c r="H14" s="24" t="n">
         <f aca="false">IF(Zones!L14&gt;0,Hypothèses!$B$4/(Zones!L14/1000),0)*Zones!N14*MAX(0,Hypothèses!$B$14-D14)</f>
@@ -8953,7 +9135,7 @@
       </c>
       <c r="AA14" s="24" t="n">
         <f aca="false">G14+H14+I14+L14+P14+S14+T14+Z14</f>
-        <v>137.5</v>
+        <v>163.02</v>
       </c>
       <c r="AB14" s="10" t="n">
         <v>18</v>
@@ -8965,7 +9147,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="28" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="AC15" s="38" t="n">
         <f aca="false">SUM(AC5:AC14)</f>
@@ -8974,32 +9156,32 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="5" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="39" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="39" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="39" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="39" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="39" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
P1 RDC v6: can line with SOMME PE-6 MIX seamer in sertissage
Dosomat moved 4 m south; north part of sertissage now holds the can
line: can filler reserve (2.0 x 2.0), SOMME PE-6 MIX seamer
(2.355 x 1.20 m), outfeed conveyor and basket loader reserve at the
retort aisle opening. Workbook gains an Équipements sheet (footprints,
weights, power, air, water, noise from the vendor documents).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011Ghrdsx3moo1sM21DD7JVm
</commit_message>
<xml_diff>
--- a/DWG_Plan_Modificatif/DWG Plan Modificatif/Unite Humide - dimensions panneaux froid.xlsx
+++ b/DWG_Plan_Modificatif/DWG Plan Modificatif/Unite Humide - dimensions panneaux froid.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Parois" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Panneaux" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="Bilan frigorifique" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Équipements" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -1700,7 +1701,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="345">
   <si>
     <t xml:space="preserve">Unité Humide – RDC Modifié (P1 RDC v2) : dimensions, panneaux sandwich et puissance frigorifique</t>
   </si>
@@ -1723,6 +1724,9 @@
     <t xml:space="preserve">• Bilan frigorifique : pré-dimensionnement de la puissance par zone réfrigérée.</t>
   </si>
   <si>
+    <t xml:space="preserve">• Équipements : encombrements, poids, puissances et utilités des machines (documents fournisseurs).</t>
+  </si>
+  <si>
     <t xml:space="preserve">• Hypothèses : tous les paramètres modifiables (températures, λ, règles d'épaisseur, prix, hauteurs de portes).</t>
   </si>
   <si>
@@ -1987,7 +1991,7 @@
     <t xml:space="preserve">Zone de sertissage</t>
   </si>
   <si>
-    <t xml:space="preserve">Waldner Dosomat 12.6 (2,88 × 5,35 m, ~20 kW). Ouverte sur l'allée des autoclaves.</t>
+    <t xml:space="preserve">Waldner Dosomat 12.6 + ligne boîtes (réserve remplisseuse, sertisseuse SOMME PE-6 MIX, réserve chargeur paniers). Ouverte sur l'allée des autoclaves.</t>
   </si>
   <si>
     <t xml:space="preserve">Z5</t>
@@ -2573,6 +2577,165 @@
   </si>
   <si>
     <t xml:space="preserve">• Résultat = puissance frigorifique utile à l'évaporateur ; la puissance électrique absorbée dépend du COP de l'installation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Équipements process – encombrements et utilités (d'après les documents fournisseurs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valeurs saisies telles qu'indiquées par les fournisseurs (mm, kg, kW). Vide = non communiqué. « est. » = estimé sur plan.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Équipement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qté</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Longueur (mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Largeur (mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hauteur (mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poids unit. (kg)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puissance unit. (kW)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puissance totale (kW)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Air comprimé</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eau / vapeur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bruit (dB)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remarques</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Karl Schnell – mélangeur 1500 + trémie 2000 + émulsionneur FD225 DK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Groupe complet avec plateforme et élévateur (hauteur maxi 4 903 au basculement)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Karl Schnell 24_001-G (18.03.2025)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Karl Schnell – hachoir automatique AG-K280 T470 + élévateur + chariot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zone de maintenance devant la machine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Karl Schnell 24_001-G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Karl Schnell – armoire électrique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JBT FTNON – trémie émulsion 1000 L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ø 1 800</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JBT 05X0292.000 rev. A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Z6/Z5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JBT FTNON – extrudeuse 800 + tunnel vapeur 800×8000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vapeur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Largeur capot ouvert 3 056 ; 2 extractions Ø356</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JBT FTNON – convoyeur de refroidissement 800×4000 + découpe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Longueur est. (convoyeur 4 000 + découpe ~2 000)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JBT 05X0292.000 (est. à l'échelle)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Waldner Dosomat 12.6 – 13308 (barquettes alu)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">600 l/min à 6 bar, 1/2"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eau 60 l/h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Encombrement porte armoire comprise ; dimensions d'introduction 3 600 × 2 950 × 2 500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Waldner 100594254 (23.07.2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOMME PE-6 MIX – sertisseuse boîtes Ø73–99</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3–4 bar ; 80 l/h à 6 bar (à vérifier)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrée/sortie boîtes à 1 000 mm ; 50–200 b/min recommandé, 250 maxi (demande 220)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Somme offre 42400084/00 (13.05.2024)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remplisseuse boîtes (réserve)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">À définir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">—</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chargeur de paniers (réserve)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">À définir, à l'entrée de l'allée autoclaves</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Steriflow – stérilisateur 1300 (LU 5 530)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AAC 1"1/2, SAC 1"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vapeur DN50, eau froide DN50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Largeur est. ~1 650 (1 510 démonté) ; poids plein d'eau 10 350 daN, vide 2 600 daN ; 7 750 L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Steriflow SC-NG2-1361 rév. B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL puissance connue (kW)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Charge totale connue (kg, autoclaves pleins d'eau)</t>
   </si>
 </sst>
 </file>
@@ -2766,7 +2929,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="46">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2924,6 +3087,30 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3179,7 +3366,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="120"/>
@@ -3229,28 +3416,28 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2"/>
+      <c r="A10" s="2" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
-        <v>8</v>
-      </c>
+      <c r="A11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2"/>
+      <c r="A13" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
+      <c r="A14" s="2"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3259,7 +3446,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
         <v>13</v>
       </c>
@@ -3282,6 +3469,11 @@
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="2" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -3311,176 +3503,176 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B4" s="7" t="n">
         <v>0.022</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B5" s="7" t="n">
         <v>1.2</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B6" s="7" t="n">
         <v>0.25</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B7" s="7" t="n">
         <v>0.6</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B8" s="9" t="n">
         <v>0.2</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B9" s="9" t="n">
         <v>0.05</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B10" s="9" t="n">
         <v>0.15</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B13" s="10" t="n">
         <v>40</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B14" s="10" t="n">
         <v>40</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B15" s="10" t="n">
         <v>20</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B16" s="10" t="n">
         <v>30</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B17" s="10" t="n">
         <v>25</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B18" s="10" t="n">
         <v>30</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3529,28 +3721,28 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B30" s="15" t="n">
         <v>2.1</v>
@@ -3561,7 +3753,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="14" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B31" s="15" t="n">
         <v>2.1</v>
@@ -3572,7 +3764,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="14" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B32" s="15" t="n">
         <v>3</v>
@@ -3583,7 +3775,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B33" s="15" t="n">
         <v>2.8</v>
@@ -3594,26 +3786,26 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B37" s="11" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C37" s="11" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3798,7 +3990,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B48" s="18" t="n">
         <f aca="false">Hypothèses!$B$13</f>
@@ -3808,12 +4000,12 @@
         <v>0</v>
       </c>
       <c r="D48" s="14" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="14" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B49" s="18" t="n">
         <f aca="false">Hypothèses!$B$14</f>
@@ -3823,12 +4015,12 @@
         <v>0</v>
       </c>
       <c r="D49" s="14" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="14" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B50" s="18" t="n">
         <f aca="false">Hypothèses!$B$15</f>
@@ -3838,12 +4030,12 @@
         <v>0</v>
       </c>
       <c r="D50" s="14" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="14" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B51" s="18" t="n">
         <f aca="false">Hypothèses!$B$16</f>
@@ -3853,12 +4045,12 @@
         <v>0</v>
       </c>
       <c r="D51" s="14" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B52" s="18" t="n">
         <f aca="false">Hypothèses!$B$17</f>
@@ -3868,12 +4060,12 @@
         <v>0</v>
       </c>
       <c r="D52" s="14" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="14" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B53" s="18" t="n">
         <f aca="false">Hypothèses!$B$18</f>
@@ -3883,7 +4075,7 @@
         <v>0</v>
       </c>
       <c r="D53" s="14" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -3915,67 +4107,67 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="I4" s="19" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="J4" s="19" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="K4" s="19" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="L4" s="19" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="M4" s="19" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="N4" s="19" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O4" s="19" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="20" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C5" s="21" t="n">
         <v>11.83</v>
@@ -3999,10 +4191,10 @@
         <v>1734.7512</v>
       </c>
       <c r="I5" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J5" s="25" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K5" s="10" t="n">
         <v>30</v>
@@ -4023,10 +4215,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C6" s="21" t="n">
         <v>12.5</v>
@@ -4050,10 +4242,10 @@
         <v>1281</v>
       </c>
       <c r="I6" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J6" s="25" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K6" s="10" t="n">
         <v>30</v>
@@ -4074,10 +4266,10 @@
     </row>
     <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C7" s="21" t="n">
         <v>8.5</v>
@@ -4101,10 +4293,10 @@
         <v>1037.34</v>
       </c>
       <c r="I7" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J7" s="25" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K7" s="10" t="n">
         <v>35</v>
@@ -4122,15 +4314,15 @@
         <v>172.89</v>
       </c>
       <c r="O7" s="26" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C8" s="21" t="n">
         <v>19.8</v>
@@ -4154,10 +4346,10 @@
         <v>831.006</v>
       </c>
       <c r="I8" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J8" s="25" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K8" s="10" t="n">
         <v>30</v>
@@ -4175,15 +4367,15 @@
         <v>138.501</v>
       </c>
       <c r="O8" s="26" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C9" s="21" t="n">
         <v>19.8</v>
@@ -4207,10 +4399,10 @@
         <v>1186.218</v>
       </c>
       <c r="I9" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J9" s="25" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K9" s="10" t="n">
         <v>35</v>
@@ -4228,21 +4420,21 @@
         <v>197.703</v>
       </c>
       <c r="O9" s="26" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E10" s="27" t="n">
         <v>160.51</v>
@@ -4258,10 +4450,10 @@
         <v>963.06</v>
       </c>
       <c r="I10" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J10" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="K10" s="10" t="n">
         <v>10</v>
@@ -4279,15 +4471,15 @@
         <v>160.51</v>
       </c>
       <c r="O10" s="26" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C11" s="21" t="n">
         <v>2.8</v>
@@ -4311,10 +4503,10 @@
         <v>410.592</v>
       </c>
       <c r="I11" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J11" s="25" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K11" s="10" t="n">
         <v>30</v>
@@ -4332,15 +4524,15 @@
         <v>68.432</v>
       </c>
       <c r="O11" s="26" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C12" s="21" t="n">
         <v>15.01</v>
@@ -4364,10 +4556,10 @@
         <v>1741.7604</v>
       </c>
       <c r="I12" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J12" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="K12" s="10" t="n">
         <v>-20</v>
@@ -4385,15 +4577,15 @@
         <v>290.2934</v>
       </c>
       <c r="O12" s="26" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C13" s="21" t="n">
         <v>15.01</v>
@@ -4417,10 +4609,10 @@
         <v>450.3</v>
       </c>
       <c r="I13" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J13" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="K13" s="10" t="n">
         <v>2</v>
@@ -4441,16 +4633,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E14" s="27" t="n">
         <v>286.11</v>
@@ -4466,10 +4658,10 @@
         <v>1716.66</v>
       </c>
       <c r="I14" s="25" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J14" s="25" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K14" s="10" t="n">
         <v>30</v>
@@ -4487,12 +4679,12 @@
         <v>0</v>
       </c>
       <c r="O14" s="26" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="28" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E15" s="29" t="n">
         <f aca="false">SUM(E5:E14)</f>
@@ -4546,58 +4738,58 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I4" s="19" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="20" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F5" s="21" t="n">
         <v>1.5</v>
@@ -4611,24 +4803,24 @@
         <v>3.15</v>
       </c>
       <c r="I5" s="26" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F6" s="21" t="n">
         <v>1.4</v>
@@ -4645,19 +4837,19 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F7" s="21" t="n">
         <v>1.4</v>
@@ -4674,19 +4866,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F8" s="21" t="n">
         <v>1.4</v>
@@ -4703,19 +4895,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F9" s="21" t="n">
         <v>1.4</v>
@@ -4732,19 +4924,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F10" s="21" t="n">
         <v>1.4</v>
@@ -4761,19 +4953,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F11" s="21" t="n">
         <v>1.4</v>
@@ -4790,19 +4982,19 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F12" s="21" t="n">
         <v>1.4</v>
@@ -4816,24 +5008,24 @@
         <v>2.94</v>
       </c>
       <c r="I12" s="26" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F13" s="21" t="n">
         <v>1.4</v>
@@ -4847,24 +5039,24 @@
         <v>2.94</v>
       </c>
       <c r="I13" s="26" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F14" s="21" t="n">
         <v>1.4</v>
@@ -4878,24 +5070,24 @@
         <v>2.94</v>
       </c>
       <c r="I14" s="26" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F15" s="21" t="n">
         <v>1.4</v>
@@ -4912,19 +5104,19 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="20" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F16" s="21" t="n">
         <v>1.4</v>
@@ -4938,24 +5130,24 @@
         <v>2.94</v>
       </c>
       <c r="I16" s="26" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E17" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F17" s="21" t="n">
         <v>1.4</v>
@@ -4969,24 +5161,24 @@
         <v>2.94</v>
       </c>
       <c r="I17" s="26" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="20" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F18" s="21" t="n">
         <v>1.4</v>
@@ -5000,24 +5192,24 @@
         <v>2.94</v>
       </c>
       <c r="I18" s="26" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="20" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F19" s="21" t="n">
         <v>1.4</v>
@@ -5031,24 +5223,24 @@
         <v>2.94</v>
       </c>
       <c r="I19" s="26" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E20" s="14" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F20" s="21" t="n">
         <v>2.8</v>
@@ -5062,24 +5254,24 @@
         <v>8.4</v>
       </c>
       <c r="I20" s="26" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F21" s="21" t="n">
         <v>1.4</v>
@@ -5093,24 +5285,24 @@
         <v>2.94</v>
       </c>
       <c r="I21" s="26" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="20" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E22" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F22" s="21" t="n">
         <v>1.4</v>
@@ -5124,24 +5316,24 @@
         <v>2.94</v>
       </c>
       <c r="I22" s="26" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E23" s="14" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F23" s="21" t="n">
         <v>2</v>
@@ -5155,7 +5347,7 @@
         <v>5.6</v>
       </c>
       <c r="I23" s="26" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
   </sheetData>
@@ -5191,76 +5383,76 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
+        <v>121</v>
+      </c>
+      <c r="B4" s="19" t="s">
+        <v>119</v>
+      </c>
+      <c r="C4" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="B4" s="19" t="s">
-        <v>118</v>
-      </c>
-      <c r="C4" s="19" t="s">
-        <v>119</v>
-      </c>
       <c r="D4" s="19" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="I4" s="19" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J4" s="19" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K4" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="L4" s="19" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="M4" s="19" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="N4" s="19" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="O4" s="19" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="P4" s="19" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="20" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E5" s="21" t="n">
         <v>24.44</v>
@@ -5312,16 +5504,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E6" s="21" t="n">
         <v>11.83</v>
@@ -5373,16 +5565,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="E7" s="21" t="n">
         <v>11.83</v>
@@ -5434,16 +5626,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="E8" s="21" t="n">
         <v>7.26</v>
@@ -5495,16 +5687,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E9" s="21" t="n">
         <v>17.08</v>
@@ -5556,16 +5748,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E10" s="21" t="n">
         <v>12.5</v>
@@ -5617,16 +5809,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E11" s="21" t="n">
         <v>17.08</v>
@@ -5678,16 +5870,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E12" s="21" t="n">
         <v>12.5</v>
@@ -5739,16 +5931,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E13" s="21" t="n">
         <v>8.5</v>
@@ -5800,16 +5992,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E14" s="21" t="n">
         <v>8.5</v>
@@ -5861,16 +6053,16 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E15" s="21" t="n">
         <v>3.16</v>
@@ -5922,16 +6114,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="20" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E16" s="21" t="n">
         <v>3.16</v>
@@ -5983,16 +6175,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E17" s="21" t="n">
         <v>9.985</v>
@@ -6044,16 +6236,16 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="20" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E18" s="21" t="n">
         <v>19.8</v>
@@ -6105,16 +6297,16 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="20" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E19" s="21" t="n">
         <v>19.8</v>
@@ -6166,16 +6358,16 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E20" s="21" t="n">
         <v>19.8</v>
@@ -6227,16 +6419,16 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E21" s="21" t="n">
         <v>6.995</v>
@@ -6288,16 +6480,16 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E22" s="21" t="n">
         <v>5.165</v>
@@ -6349,16 +6541,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E23" s="21" t="n">
         <v>9.985</v>
@@ -6410,16 +6602,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E24" s="21" t="n">
         <v>6.2</v>
@@ -6471,16 +6663,16 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="20" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E25" s="21" t="n">
         <v>8.33</v>
@@ -6532,16 +6724,16 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E26" s="21" t="n">
         <v>3.93</v>
@@ -6593,16 +6785,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E27" s="21" t="n">
         <v>2.2</v>
@@ -6654,16 +6846,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="20" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E28" s="21" t="n">
         <v>8.4</v>
@@ -6715,16 +6907,16 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="20" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E29" s="21" t="n">
         <v>9.985</v>
@@ -6776,16 +6968,16 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="20" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E30" s="21" t="n">
         <v>10.43</v>
@@ -6837,16 +7029,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="20" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E31" s="21" t="n">
         <v>3.93</v>
@@ -6898,16 +7090,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="20" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E32" s="21" t="n">
         <v>2.8</v>
@@ -6959,16 +7151,16 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="20" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E33" s="21" t="n">
         <v>2.8</v>
@@ -7020,16 +7212,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="20" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B34" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E34" s="21" t="n">
         <v>2.8</v>
@@ -7081,16 +7273,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="20" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B35" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E35" s="21" t="n">
         <v>19.34</v>
@@ -7142,16 +7334,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="20" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B36" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E36" s="21" t="n">
         <v>5</v>
@@ -7203,16 +7395,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="20" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B37" s="14" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E37" s="21" t="n">
         <v>15.01</v>
@@ -7264,16 +7456,16 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="20" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E38" s="21" t="n">
         <v>15.01</v>
@@ -7325,16 +7517,16 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="20" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D39" s="14" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E39" s="21" t="n">
         <v>19.34</v>
@@ -7386,16 +7578,16 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="20" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B40" s="14" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D40" s="14" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E40" s="21" t="n">
         <v>5</v>
@@ -7447,16 +7639,16 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="20" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B41" s="14" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D41" s="14" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E41" s="21" t="n">
         <v>15.01</v>
@@ -7508,16 +7700,16 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="20" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B42" s="14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D42" s="14" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E42" s="21" t="n">
         <v>49.5</v>
@@ -7569,16 +7761,16 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="20" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B43" s="14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D43" s="14" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E43" s="21" t="n">
         <v>17.6</v>
@@ -7630,7 +7822,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D44" s="28" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E44" s="29" t="n">
         <f aca="false">SUM(E5:E43)</f>
@@ -7651,7 +7843,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D46" s="33" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
   </sheetData>
@@ -7684,35 +7876,35 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7837,7 +8029,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="28" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B9" s="29" t="n">
         <f aca="false">SUM(B5:B8)</f>
@@ -7862,7 +8054,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="G10" s="24" t="n">
         <f aca="false">G9*Hypothèses!$B$10</f>
@@ -7871,16 +8063,16 @@
     </row>
     <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="19" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7957,7 +8149,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="28" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D17" s="30" t="n">
         <f aca="false">SUM(D13:D16)</f>
@@ -7966,7 +8158,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="28" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B19" s="28"/>
       <c r="C19" s="28"/>
@@ -8008,101 +8200,101 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="I4" s="19" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="J4" s="19" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="K4" s="19" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="L4" s="19" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="M4" s="19" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="N4" s="19" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="O4" s="19" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="P4" s="19" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="Q4" s="19" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="R4" s="19" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="S4" s="19" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="T4" s="19" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="U4" s="19" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="V4" s="19" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="W4" s="19" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="X4" s="19" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="Y4" s="19" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="Z4" s="19" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="AA4" s="19" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="AB4" s="19" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="AC4" s="19" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9147,7 +9339,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="28" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="AC15" s="38" t="n">
         <f aca="false">SUM(AC5:AC14)</f>
@@ -9156,32 +9348,535 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="5" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="39" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="39" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="39" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="39" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="39" t="s">
-        <v>290</v>
+        <v>291</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:N17"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="4" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="34"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="8" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="B4" s="19" t="s">
+        <v>294</v>
+      </c>
+      <c r="C4" s="19" t="s">
+        <v>295</v>
+      </c>
+      <c r="D4" s="19" t="s">
+        <v>296</v>
+      </c>
+      <c r="E4" s="19" t="s">
+        <v>297</v>
+      </c>
+      <c r="F4" s="19" t="s">
+        <v>298</v>
+      </c>
+      <c r="G4" s="19" t="s">
+        <v>299</v>
+      </c>
+      <c r="H4" s="19" t="s">
+        <v>300</v>
+      </c>
+      <c r="I4" s="19" t="s">
+        <v>301</v>
+      </c>
+      <c r="J4" s="19" t="s">
+        <v>302</v>
+      </c>
+      <c r="K4" s="19" t="s">
+        <v>303</v>
+      </c>
+      <c r="L4" s="19" t="s">
+        <v>304</v>
+      </c>
+      <c r="M4" s="19" t="s">
+        <v>305</v>
+      </c>
+      <c r="N4" s="19" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>307</v>
+      </c>
+      <c r="C5" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="41" t="n">
+        <v>4834</v>
+      </c>
+      <c r="E5" s="41" t="n">
+        <v>5247</v>
+      </c>
+      <c r="F5" s="41" t="n">
+        <v>3857</v>
+      </c>
+      <c r="G5" s="41"/>
+      <c r="H5" s="42"/>
+      <c r="I5" s="43" t="str">
+        <f aca="false">IF(H5="","",C5*H5)</f>
+        <v/>
+      </c>
+      <c r="J5" s="44"/>
+      <c r="K5" s="44"/>
+      <c r="L5" s="42"/>
+      <c r="M5" s="26" t="s">
+        <v>308</v>
+      </c>
+      <c r="N5" s="14" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>310</v>
+      </c>
+      <c r="C6" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="41" t="n">
+        <v>1858</v>
+      </c>
+      <c r="E6" s="41" t="n">
+        <v>5953</v>
+      </c>
+      <c r="F6" s="41" t="n">
+        <v>3422</v>
+      </c>
+      <c r="G6" s="41"/>
+      <c r="H6" s="42"/>
+      <c r="I6" s="43" t="str">
+        <f aca="false">IF(H6="","",C6*H6)</f>
+        <v/>
+      </c>
+      <c r="J6" s="44"/>
+      <c r="K6" s="44"/>
+      <c r="L6" s="42"/>
+      <c r="M6" s="26" t="s">
+        <v>311</v>
+      </c>
+      <c r="N6" s="14" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>313</v>
+      </c>
+      <c r="C7" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="41" t="n">
+        <v>2400</v>
+      </c>
+      <c r="E7" s="41" t="n">
+        <v>500</v>
+      </c>
+      <c r="F7" s="41" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G7" s="41"/>
+      <c r="H7" s="42"/>
+      <c r="I7" s="43" t="str">
+        <f aca="false">IF(H7="","",C7*H7)</f>
+        <v/>
+      </c>
+      <c r="J7" s="44"/>
+      <c r="K7" s="44"/>
+      <c r="L7" s="42"/>
+      <c r="M7" s="26"/>
+      <c r="N7" s="14" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>314</v>
+      </c>
+      <c r="C8" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="41" t="n">
+        <v>1800</v>
+      </c>
+      <c r="E8" s="41" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F8" s="41" t="n">
+        <v>1850</v>
+      </c>
+      <c r="G8" s="41"/>
+      <c r="H8" s="42"/>
+      <c r="I8" s="43" t="str">
+        <f aca="false">IF(H8="","",C8*H8)</f>
+        <v/>
+      </c>
+      <c r="J8" s="44"/>
+      <c r="K8" s="44"/>
+      <c r="L8" s="42"/>
+      <c r="M8" s="26" t="s">
+        <v>315</v>
+      </c>
+      <c r="N8" s="14" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="14" t="s">
+        <v>317</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>318</v>
+      </c>
+      <c r="C9" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="41" t="n">
+        <v>12547</v>
+      </c>
+      <c r="E9" s="41" t="n">
+        <v>3056</v>
+      </c>
+      <c r="F9" s="41" t="n">
+        <v>2719</v>
+      </c>
+      <c r="G9" s="41"/>
+      <c r="H9" s="42"/>
+      <c r="I9" s="43" t="str">
+        <f aca="false">IF(H9="","",C9*H9)</f>
+        <v/>
+      </c>
+      <c r="J9" s="44"/>
+      <c r="K9" s="44" t="s">
+        <v>319</v>
+      </c>
+      <c r="L9" s="42"/>
+      <c r="M9" s="26" t="s">
+        <v>320</v>
+      </c>
+      <c r="N9" s="14" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>321</v>
+      </c>
+      <c r="C10" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="41" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E10" s="41" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F10" s="41" t="n">
+        <v>1340</v>
+      </c>
+      <c r="G10" s="41"/>
+      <c r="H10" s="42"/>
+      <c r="I10" s="43" t="str">
+        <f aca="false">IF(H10="","",C10*H10)</f>
+        <v/>
+      </c>
+      <c r="J10" s="44"/>
+      <c r="K10" s="44"/>
+      <c r="L10" s="42"/>
+      <c r="M10" s="26" t="s">
+        <v>322</v>
+      </c>
+      <c r="N10" s="14" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>324</v>
+      </c>
+      <c r="C11" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="41" t="n">
+        <v>5350</v>
+      </c>
+      <c r="E11" s="41" t="n">
+        <v>2880</v>
+      </c>
+      <c r="F11" s="41" t="n">
+        <v>2466</v>
+      </c>
+      <c r="G11" s="41"/>
+      <c r="H11" s="42" t="n">
+        <v>20</v>
+      </c>
+      <c r="I11" s="43" t="n">
+        <f aca="false">IF(H11="","",C11*H11)</f>
+        <v>20</v>
+      </c>
+      <c r="J11" s="44" t="s">
+        <v>325</v>
+      </c>
+      <c r="K11" s="44" t="s">
+        <v>326</v>
+      </c>
+      <c r="L11" s="42"/>
+      <c r="M11" s="26" t="s">
+        <v>327</v>
+      </c>
+      <c r="N11" s="14" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>329</v>
+      </c>
+      <c r="C12" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="41" t="n">
+        <v>2355</v>
+      </c>
+      <c r="E12" s="41" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F12" s="41" t="n">
+        <v>2015</v>
+      </c>
+      <c r="G12" s="41" t="n">
+        <v>1700</v>
+      </c>
+      <c r="H12" s="42" t="n">
+        <v>5</v>
+      </c>
+      <c r="I12" s="43" t="n">
+        <f aca="false">IF(H12="","",C12*H12)</f>
+        <v>5</v>
+      </c>
+      <c r="J12" s="44" t="s">
+        <v>330</v>
+      </c>
+      <c r="K12" s="44"/>
+      <c r="L12" s="42" t="n">
+        <v>82.9</v>
+      </c>
+      <c r="M12" s="26" t="s">
+        <v>331</v>
+      </c>
+      <c r="N12" s="14" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>333</v>
+      </c>
+      <c r="C13" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="41" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E13" s="41" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F13" s="41"/>
+      <c r="G13" s="41"/>
+      <c r="H13" s="42"/>
+      <c r="I13" s="43" t="str">
+        <f aca="false">IF(H13="","",C13*H13)</f>
+        <v/>
+      </c>
+      <c r="J13" s="44"/>
+      <c r="K13" s="44"/>
+      <c r="L13" s="42"/>
+      <c r="M13" s="26" t="s">
+        <v>334</v>
+      </c>
+      <c r="N13" s="14" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>336</v>
+      </c>
+      <c r="C14" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="41" t="n">
+        <v>1800</v>
+      </c>
+      <c r="E14" s="41" t="n">
+        <v>1700</v>
+      </c>
+      <c r="F14" s="41"/>
+      <c r="G14" s="41"/>
+      <c r="H14" s="42"/>
+      <c r="I14" s="43" t="str">
+        <f aca="false">IF(H14="","",C14*H14)</f>
+        <v/>
+      </c>
+      <c r="J14" s="44"/>
+      <c r="K14" s="44"/>
+      <c r="L14" s="42"/>
+      <c r="M14" s="26" t="s">
+        <v>337</v>
+      </c>
+      <c r="N14" s="14" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="B15" s="14" t="s">
+        <v>338</v>
+      </c>
+      <c r="C15" s="40" t="n">
+        <v>6</v>
+      </c>
+      <c r="D15" s="41" t="n">
+        <v>7225</v>
+      </c>
+      <c r="E15" s="41" t="n">
+        <v>1650</v>
+      </c>
+      <c r="F15" s="41" t="n">
+        <v>2052</v>
+      </c>
+      <c r="G15" s="41" t="n">
+        <v>10350</v>
+      </c>
+      <c r="H15" s="42"/>
+      <c r="I15" s="43" t="str">
+        <f aca="false">IF(H15="","",C15*H15)</f>
+        <v/>
+      </c>
+      <c r="J15" s="44" t="s">
+        <v>339</v>
+      </c>
+      <c r="K15" s="44" t="s">
+        <v>340</v>
+      </c>
+      <c r="L15" s="42"/>
+      <c r="M15" s="26" t="s">
+        <v>341</v>
+      </c>
+      <c r="N15" s="14" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="28" t="s">
+        <v>343</v>
+      </c>
+      <c r="I16" s="45" t="n">
+        <f aca="false">SUM(I5:I15)</f>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="28" t="s">
+        <v>344</v>
+      </c>
+      <c r="G17" s="30" t="n">
+        <f aca="false">SUMPRODUCT(C5:C15,G5:G15)</f>
+        <v>63800</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
P1 RDC v7: Zilli & Bellini pocket filler on the can line
Filler reserve replaced by the TB pocket filler footprint (LAY00537):
guard 2630 x 2500, 5300 with conveyor stubs, 4930 x 4350 door-open
envelope, separate control panel on the west wall, 1100 -> 1000 mm
transfer to the SOMME seamer. Workbook Équipements sheet updated
(8 kW, 400 Nl/min, speeds and open points).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011Ghrdsx3moo1sM21DD7JVm
</commit_message>
<xml_diff>
--- a/DWG_Plan_Modificatif/DWG Plan Modificatif/Unite Humide - dimensions panneaux froid.xlsx
+++ b/DWG_Plan_Modificatif/DWG Plan Modificatif/Unite Humide - dimensions panneaux froid.xlsx
@@ -1701,7 +1701,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="348">
   <si>
     <t xml:space="preserve">Unité Humide – RDC Modifié (P1 RDC v2) : dimensions, panneaux sandwich et puissance frigorifique</t>
   </si>
@@ -1991,7 +1991,7 @@
     <t xml:space="preserve">Zone de sertissage</t>
   </si>
   <si>
-    <t xml:space="preserve">Waldner Dosomat 12.6 + ligne boîtes (réserve remplisseuse, sertisseuse SOMME PE-6 MIX, réserve chargeur paniers). Ouverte sur l'allée des autoclaves.</t>
+    <t xml:space="preserve">Waldner Dosomat 12.6 + ligne boîtes (remplisseuse Zilli &amp; Bellini TB, sertisseuse SOMME PE-6 MIX, réserve chargeur paniers). Ouverte sur l'allée des autoclaves.</t>
   </si>
   <si>
     <t xml:space="preserve">Z5</t>
@@ -2702,19 +2702,28 @@
     <t xml:space="preserve">Somme offre 42400084/00 (13.05.2024)</t>
   </si>
   <si>
-    <t xml:space="preserve">Remplisseuse boîtes (réserve)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">À définir</t>
+    <t xml:space="preserve">Zilli &amp; Bellini – remplisseuse à poches TB (12 ou 16 télescopes, à confirmer)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">400 Nl/min à 6 bar, 1/2" G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exclus (vapeur, eau, CIP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carter 2 630 × 2 500 ; portes ouvertes 4 930 × 4 350 ; convoyeur boîtes à 1 100 ± 50 (sertisseuse à 1 000) ; 80 b/min (400 g), 30 b/min (1 250 g) ; armoire séparée à 2–3 m ; tension 50 Hz à confirmer (offre : 60 Hz)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zilli &amp; Bellini O24/450 + LAY00537 (01/08/2024)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chargeur de paniers (réserve)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">À définir, à l'entrée de l'allée autoclaves</t>
   </si>
   <si>
     <t xml:space="preserve">—</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chargeur de paniers (réserve)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">À définir, à l'entrée de l'allée autoclaves</t>
   </si>
   <si>
     <t xml:space="preserve">Steriflow – stérilisateur 1300 (LU 5 530)</t>
@@ -9754,7 +9763,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
         <v>94</v>
       </c>
@@ -9765,26 +9774,32 @@
         <v>1</v>
       </c>
       <c r="D13" s="41" t="n">
-        <v>2000</v>
+        <v>5300</v>
       </c>
       <c r="E13" s="41" t="n">
-        <v>2000</v>
+        <v>2500</v>
       </c>
       <c r="F13" s="41"/>
       <c r="G13" s="41"/>
-      <c r="H13" s="42"/>
-      <c r="I13" s="43" t="str">
+      <c r="H13" s="42" t="n">
+        <v>8</v>
+      </c>
+      <c r="I13" s="43" t="n">
         <f aca="false">IF(H13="","",C13*H13)</f>
-        <v/>
-      </c>
-      <c r="J13" s="44"/>
-      <c r="K13" s="44"/>
+        <v>8</v>
+      </c>
+      <c r="J13" s="44" t="s">
+        <v>334</v>
+      </c>
+      <c r="K13" s="44" t="s">
+        <v>335</v>
+      </c>
       <c r="L13" s="42"/>
       <c r="M13" s="26" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="N13" s="14" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9792,7 +9807,7 @@
         <v>94</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="C14" s="40" t="n">
         <v>1</v>
@@ -9814,10 +9829,10 @@
       <c r="K14" s="44"/>
       <c r="L14" s="42"/>
       <c r="M14" s="26" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="N14" s="14" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9825,7 +9840,7 @@
         <v>91</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="C15" s="40" t="n">
         <v>6</v>
@@ -9848,31 +9863,31 @@
         <v/>
       </c>
       <c r="J15" s="44" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="K15" s="44" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="L15" s="42"/>
       <c r="M15" s="26" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="N15" s="14" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="28" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="I16" s="45" t="n">
         <f aca="false">SUM(I5:I15)</f>
-        <v>25</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="28" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="G17" s="30" t="n">
         <f aca="false">SUMPRODUCT(C5:C15,G5:G15)</f>

</xml_diff>